<commit_message>
Reportar solo afectaciones documentadas a servicios MTDH y corregir carga concurrente
</commit_message>
<xml_diff>
--- a/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
+++ b/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
@@ -14,18 +14,18 @@
     <sheet name="Ficha técnica" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Alertas!$B$8:$I$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Alertas!$B$8:$K$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Kits!$B$8:$E$15</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Resumen!$A$1:$N$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Resumen!$A$1:$N$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="145">
-  <si>
-    <t>Seguimiento ENOS</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="131">
+  <si>
+    <t>Seguimiento y respuesta MTDH</t>
   </si>
   <si>
     <t>29/09 al 26/10/2026 · Nacional · Alertas, kits y bono de contingencia</t>
@@ -40,7 +40,7 @@
     <t>29/09 al 26/10/2026</t>
   </si>
   <si>
-    <t>Alertas registradas</t>
+    <t>Alertas de servicios MTDH</t>
   </si>
   <si>
     <t>Desde el 29/09/2026</t>
@@ -52,7 +52,7 @@
     <t>Pendientes o en seguimiento</t>
   </si>
   <si>
-    <t>UA identificadas en alertas</t>
+    <t>UA con afectación documentada</t>
   </si>
   <si>
     <t>Códigos de unidad distintos</t>
@@ -82,237 +82,189 @@
     <t>Manabí</t>
   </si>
   <si>
-    <t>Pichincha</t>
-  </si>
-  <si>
-    <t>Cotopaxi</t>
+    <t>Total de la selección</t>
+  </si>
+  <si>
+    <t>Aspectos destacados</t>
+  </si>
+  <si>
+    <t>8 alertas con afectación a servicios MTDH desde el 29/09 en 3 provincias.</t>
+  </si>
+  <si>
+    <t>802 kits documentados en el fin de semana del 24–25/10.</t>
+  </si>
+  <si>
+    <t>Afectaciones a servicios MTDH</t>
+  </si>
+  <si>
+    <t>Detalle desde el 29/09</t>
+  </si>
+  <si>
+    <t>Alerta</t>
+  </si>
+  <si>
+    <t>Fecha de registro</t>
+  </si>
+  <si>
+    <t>Cantón</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Código UA</t>
+  </si>
+  <si>
+    <t>Unidad de atención</t>
+  </si>
+  <si>
+    <t>Servicio</t>
+  </si>
+  <si>
+    <t>Afectación al servicio</t>
+  </si>
+  <si>
+    <t>Afectados (campo fuente)</t>
+  </si>
+  <si>
+    <t>ALT-2026-000325</t>
+  </si>
+  <si>
+    <t>2026-10-20</t>
+  </si>
+  <si>
+    <t>Milagro</t>
+  </si>
+  <si>
+    <t>Pendiente</t>
+  </si>
+  <si>
+    <t>62210</t>
+  </si>
+  <si>
+    <t>GOTITA DEL AMOR</t>
+  </si>
+  <si>
+    <t>Desarrollo Infantil</t>
+  </si>
+  <si>
+    <t>Ingreso de agua en la unidad; sin energía ni agua</t>
+  </si>
+  <si>
+    <t>ALT-2026-000323</t>
+  </si>
+  <si>
+    <t>14294</t>
+  </si>
+  <si>
+    <t>MIS PEQUEÑOS ANGELITOS</t>
+  </si>
+  <si>
+    <t>Ingreso de agua y goteras en la unidad</t>
+  </si>
+  <si>
+    <t>ALT-2026-000322</t>
+  </si>
+  <si>
+    <t>13916</t>
+  </si>
+  <si>
+    <t>NIÑOS JUGUETONES</t>
+  </si>
+  <si>
+    <t>Agua dentro y fuera de la unidad</t>
+  </si>
+  <si>
+    <t>ALT-2026-000321</t>
+  </si>
+  <si>
+    <t>62208</t>
+  </si>
+  <si>
+    <t>PEQUEÑOS JILGUERITOS</t>
+  </si>
+  <si>
+    <t>Acumulación de agua en la entrada de la unidad</t>
+  </si>
+  <si>
+    <t>ALT-2026-000319</t>
+  </si>
+  <si>
+    <t>El Guabo</t>
+  </si>
+  <si>
+    <t>En seguimiento</t>
+  </si>
+  <si>
+    <t>60221</t>
+  </si>
+  <si>
+    <t>CENTRO DE DESARROLLO INFANTIL ESTRELLITA DE MAR</t>
+  </si>
+  <si>
+    <t>Ingreso de agua; cambio temporal a modalidad virtual</t>
+  </si>
+  <si>
+    <t>ALT-2026-000318</t>
+  </si>
+  <si>
+    <t>60220</t>
+  </si>
+  <si>
+    <t>CENTRO DE DESARROLLO INFANTIL SUPER NIÑO</t>
+  </si>
+  <si>
+    <t>ALT-2026-000310</t>
+  </si>
+  <si>
+    <t>2026-10-16</t>
+  </si>
+  <si>
+    <t>Flavio Alfaro</t>
+  </si>
+  <si>
+    <t>56744</t>
+  </si>
+  <si>
+    <t>CNH ESTRELLITAS DEL AMANECER</t>
+  </si>
+  <si>
+    <t>Creciendo con Nuestros Hijos (CNH)</t>
+  </si>
+  <si>
+    <t>Acceso impedido para atención presencial; contacto telefónico temporal</t>
+  </si>
+  <si>
+    <t>ALT-2026-000309</t>
+  </si>
+  <si>
+    <t>56204</t>
+  </si>
+  <si>
+    <t>CORREO INFANTIL</t>
+  </si>
+  <si>
+    <t>Solo se incluyen alertas con afectación documentada a instalaciones, acceso, continuidad o modalidad de atención de los servicios MTDH, registradas desde el 29 de septiembre de 2026. Se excluyen daños externos o a viviendas de familias usuarias sin impacto documentado en el servicio. Un código UA por sí solo no acredita afectación. La fecha corresponde al registro de la alerta; una alerta no equivale necesariamente a un evento único. El campo Afectados mezcla personas, familias y usuarios, por lo que no se presenta un total de personas únicas. La base no certifica atribución causal a ENOS.</t>
+  </si>
+  <si>
+    <t>Entregas de fin de semana</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Kits</t>
+  </si>
+  <si>
+    <t>2026-10-24</t>
+  </si>
+  <si>
+    <t>Portoviejo</t>
   </si>
   <si>
     <t>Esmeraldas</t>
   </si>
   <si>
-    <t>Santa Elena</t>
-  </si>
-  <si>
-    <t>Total de la selección</t>
-  </si>
-  <si>
-    <t>Aspectos destacados</t>
-  </si>
-  <si>
-    <t>17 alertas registradas desde el 29/09 en 7 provincias.</t>
-  </si>
-  <si>
-    <t>802 kits documentados en el fin de semana del 24–25/10.</t>
-  </si>
-  <si>
-    <t>Alertas territoriales</t>
-  </si>
-  <si>
-    <t>Detalle desde el 29/09</t>
-  </si>
-  <si>
-    <t>Alerta</t>
-  </si>
-  <si>
-    <t>Fecha de registro</t>
-  </si>
-  <si>
-    <t>Cantón</t>
-  </si>
-  <si>
-    <t>Estado</t>
-  </si>
-  <si>
-    <t>Código UA</t>
-  </si>
-  <si>
-    <t>Unidad de atención</t>
-  </si>
-  <si>
-    <t>Afectados (campo fuente)</t>
-  </si>
-  <si>
-    <t>ALT-2026-000346</t>
-  </si>
-  <si>
-    <t>2026-10-23</t>
-  </si>
-  <si>
-    <t>Distrito Metropolitano de Quito</t>
-  </si>
-  <si>
-    <t>Pendiente</t>
-  </si>
-  <si>
-    <t>Sin unidad registrada</t>
-  </si>
-  <si>
-    <t>ALT-2026-000325</t>
-  </si>
-  <si>
-    <t>2026-10-20</t>
-  </si>
-  <si>
-    <t>Milagro</t>
-  </si>
-  <si>
-    <t>62210</t>
-  </si>
-  <si>
-    <t>GOTITA DEL AMOR</t>
-  </si>
-  <si>
-    <t>ALT-2026-000324</t>
-  </si>
-  <si>
-    <t>Pangua</t>
-  </si>
-  <si>
-    <t>Resuelto</t>
-  </si>
-  <si>
-    <t>ALT-2026-000323</t>
-  </si>
-  <si>
-    <t>14294</t>
-  </si>
-  <si>
-    <t>MIS PEQUEÑOS ANGELITOS</t>
-  </si>
-  <si>
-    <t>ALT-2026-000322</t>
-  </si>
-  <si>
-    <t>13916</t>
-  </si>
-  <si>
-    <t>NIÑOS JUGUETONES</t>
-  </si>
-  <si>
-    <t>ALT-2026-000321</t>
-  </si>
-  <si>
-    <t>62208</t>
-  </si>
-  <si>
-    <t>PEQUEÑOS JILGUERITOS</t>
-  </si>
-  <si>
-    <t>ALT-2026-000320</t>
-  </si>
-  <si>
-    <t>En seguimiento</t>
-  </si>
-  <si>
-    <t>ALT-2026-000319</t>
-  </si>
-  <si>
-    <t>El Guabo</t>
-  </si>
-  <si>
-    <t>60221</t>
-  </si>
-  <si>
-    <t>CENTRO DE DESARROLLO INFANTIL ESTRELLITA DE MAR</t>
-  </si>
-  <si>
-    <t>ALT-2026-000318</t>
-  </si>
-  <si>
-    <t>60220</t>
-  </si>
-  <si>
-    <t>CENTRO DE DESARROLLO INFANTIL SUPER NIÑO</t>
-  </si>
-  <si>
-    <t>ALT-2026-000317</t>
-  </si>
-  <si>
-    <t>Pasaje</t>
-  </si>
-  <si>
-    <t>ALT-2026-000316</t>
-  </si>
-  <si>
-    <t>2026-10-19</t>
-  </si>
-  <si>
-    <t>Guayaquil</t>
-  </si>
-  <si>
-    <t>58337</t>
-  </si>
-  <si>
-    <t>CDI NIÑOS DE SAN RAFAEL</t>
-  </si>
-  <si>
-    <t>ALT-2026-000315</t>
-  </si>
-  <si>
-    <t>58336</t>
-  </si>
-  <si>
-    <t>CDI LOS NIÑOS DEL CISNE</t>
-  </si>
-  <si>
-    <t>ALT-2026-000312</t>
-  </si>
-  <si>
-    <t>Eloy Alfaro</t>
-  </si>
-  <si>
-    <t>ALT-2026-000310</t>
-  </si>
-  <si>
-    <t>2026-10-16</t>
-  </si>
-  <si>
-    <t>Flavio Alfaro</t>
-  </si>
-  <si>
-    <t>56744</t>
-  </si>
-  <si>
-    <t>CNH ESTRELLITAS DEL AMANECER</t>
-  </si>
-  <si>
-    <t>ALT-2026-000309</t>
-  </si>
-  <si>
-    <t>56204</t>
-  </si>
-  <si>
-    <t>CORREO INFANTIL</t>
-  </si>
-  <si>
-    <t>ALT-2026-000303</t>
-  </si>
-  <si>
-    <t>ALT-2026-000301</t>
-  </si>
-  <si>
-    <t>Nobol</t>
-  </si>
-  <si>
-    <t>Alertas de desastre natural registradas desde el 29 de septiembre de 2026. La fecha corresponde al registro de la alerta; una alerta no equivale necesariamente a un evento único. El campo Afectados mezcla personas, familias y usuarios, por lo que no se presenta un total de personas únicas. La base no certifica atribución causal a ENOS.</t>
-  </si>
-  <si>
-    <t>Entregas de fin de semana</t>
-  </si>
-  <si>
-    <t>Fecha</t>
-  </si>
-  <si>
-    <t>Kits</t>
-  </si>
-  <si>
-    <t>2026-10-24</t>
-  </si>
-  <si>
-    <t>Portoviejo</t>
-  </si>
-  <si>
     <t>Palestina</t>
   </si>
   <si>
@@ -421,7 +373,7 @@
     <t>Control de calidad</t>
   </si>
   <si>
-    <t>Se usó la hoja Detalle: los resúmenes del Excel abarcan otras fechas y categorías. El registro ALT-2026-000301 consigna Nobol, pero su descripción menciona Balao; se conserva el territorio de la fuente, pendiente de validación.</t>
+    <t>Se revisaron Detalle y Acciones realizadas de cada alerta. Los casos sin evidencia de afectación al servicio no se incorporan a indicadores ni exportables.</t>
   </si>
   <si>
     <t>Fuentes oficiales</t>
@@ -443,6 +395,12 @@
   </si>
   <si>
     <t>enos_kits_2026-10-25.csv</t>
+  </si>
+  <si>
+    <t>Fuente 4</t>
+  </si>
+  <si>
+    <t>enos_revision_servicios_2026-10-26.csv</t>
   </si>
   <si>
     <t>Contenido del libro</t>
@@ -970,9 +928,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Resumen!$B$16:$B$22</c:f>
+              <c:f>Resumen!$B$16:$B$18</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>Guayas</c:v>
                 </c:pt>
@@ -982,47 +940,23 @@
                 <c:pt idx="2">
                   <c:v>Manabí</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>Pichincha</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Cotopaxi</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Esmeraldas</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Santa Elena</c:v>
-                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Resumen!$J$16:$J$22</c:f>
+              <c:f>Resumen!$J$16:$J$18</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>7</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1182,13 +1116,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>43</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>43</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>342900</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1206,7 +1140,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="495300" y="10477500"/>
+          <a:off x="495300" y="9334500"/>
           <a:ext cx="247650" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1220,13 +1154,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>45</xdr:row>
+      <xdr:row>41</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>45</xdr:row>
+      <xdr:row>41</xdr:row>
       <xdr:rowOff>342900</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1244,7 +1178,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="495300" y="10982325"/>
+          <a:off x="495300" y="9839325"/>
           <a:ext cx="247650" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1258,13 +1192,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>34</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1291,13 +1225,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>2571750</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>3705225</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>1512404</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>400050</xdr:rowOff>
@@ -1317,7 +1251,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11934825" y="171450"/>
+          <a:off x="18364200" y="171450"/>
           <a:ext cx="2188679" cy="381000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1748,7 +1682,7 @@
     <tabColor rgb="FF512F8D"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.140625" customWidth="1"/>
@@ -1884,17 +1818,17 @@
     </row>
     <row r="10" spans="1:14" ht="21" customHeight="1">
       <c r="B10" s="13">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
       <c r="E10" s="13">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F10" s="14"/>
       <c r="G10" s="14"/>
       <c r="H10" s="13">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I10" s="14"/>
       <c r="J10" s="14"/>
@@ -1986,7 +1920,7 @@
       <c r="H16" s="18"/>
       <c r="I16" s="18"/>
       <c r="J16" s="19">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K16" s="19"/>
       <c r="L16" s="19"/>
@@ -2004,7 +1938,7 @@
       <c r="H17" s="20"/>
       <c r="I17" s="20"/>
       <c r="J17" s="21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K17" s="21"/>
       <c r="L17" s="21"/>
@@ -2028,149 +1962,77 @@
       <c r="L18" s="19"/>
       <c r="M18" s="19"/>
     </row>
-    <row r="19" spans="2:13" ht="23" customHeight="1">
-      <c r="B19" s="20" t="s">
+    <row r="19" spans="2:13" ht="22" customHeight="1">
+      <c r="B19" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
-      <c r="J19" s="21">
-        <v>2</v>
-      </c>
-      <c r="K19" s="21"/>
-      <c r="L19" s="21"/>
-      <c r="M19" s="21"/>
-    </row>
-    <row r="20" spans="2:13" ht="23" customHeight="1">
-      <c r="B20" s="18" t="s">
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="23">
+        <f>SUM(J16:J18)</f>
+        <v>8</v>
+      </c>
+      <c r="K19" s="23"/>
+      <c r="L19" s="23"/>
+      <c r="M19" s="23"/>
+    </row>
+    <row r="39" spans="2:13" ht="27" customHeight="1">
+      <c r="B39" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="19">
-        <v>1</v>
-      </c>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-    </row>
-    <row r="21" spans="2:13" ht="23" customHeight="1">
-      <c r="B21" s="20" t="s">
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="7"/>
+      <c r="J39" s="7"/>
+      <c r="K39" s="7"/>
+      <c r="L39" s="7"/>
+      <c r="M39" s="7"/>
+    </row>
+    <row r="40" spans="2:13" ht="34" customHeight="1">
+      <c r="B40" s="24"/>
+      <c r="C40" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="20"/>
-      <c r="J21" s="21">
-        <v>1</v>
-      </c>
-      <c r="K21" s="21"/>
-      <c r="L21" s="21"/>
-      <c r="M21" s="21"/>
-    </row>
-    <row r="22" spans="2:13" ht="23" customHeight="1">
-      <c r="B22" s="18" t="s">
+      <c r="D40" s="25"/>
+      <c r="E40" s="25"/>
+      <c r="F40" s="25"/>
+      <c r="G40" s="25"/>
+      <c r="H40" s="25"/>
+      <c r="I40" s="25"/>
+      <c r="J40" s="25"/>
+      <c r="K40" s="25"/>
+      <c r="L40" s="25"/>
+      <c r="M40" s="25"/>
+    </row>
+    <row r="41" spans="2:13" ht="6" customHeight="1"/>
+    <row r="42" spans="2:13" ht="34" customHeight="1">
+      <c r="B42" s="24"/>
+      <c r="C42" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="19">
-        <v>1</v>
-      </c>
-      <c r="K22" s="19"/>
-      <c r="L22" s="19"/>
-      <c r="M22" s="19"/>
-    </row>
-    <row r="23" spans="2:13" ht="22" customHeight="1">
-      <c r="B23" s="22" t="s">
-        <v>23</v>
-      </c>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="22"/>
-      <c r="J23" s="23">
-        <f>SUM(J16:J22)</f>
-        <v>17</v>
-      </c>
-      <c r="K23" s="23"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="23"/>
-    </row>
-    <row r="43" spans="2:13" ht="27" customHeight="1">
-      <c r="B43" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C43" s="7"/>
-      <c r="D43" s="7"/>
-      <c r="E43" s="7"/>
-      <c r="F43" s="7"/>
-      <c r="G43" s="7"/>
-      <c r="H43" s="7"/>
-      <c r="I43" s="7"/>
-      <c r="J43" s="7"/>
-      <c r="K43" s="7"/>
-      <c r="L43" s="7"/>
-      <c r="M43" s="7"/>
-    </row>
-    <row r="44" spans="2:13" ht="34" customHeight="1">
-      <c r="B44" s="24"/>
-      <c r="C44" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="D44" s="25"/>
-      <c r="E44" s="25"/>
-      <c r="F44" s="25"/>
-      <c r="G44" s="25"/>
-      <c r="H44" s="25"/>
-      <c r="I44" s="25"/>
-      <c r="J44" s="25"/>
-      <c r="K44" s="25"/>
-      <c r="L44" s="25"/>
-      <c r="M44" s="25"/>
-    </row>
-    <row r="45" spans="2:13" ht="6" customHeight="1"/>
-    <row r="46" spans="2:13" ht="34" customHeight="1">
-      <c r="B46" s="24"/>
-      <c r="C46" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="D46" s="25"/>
-      <c r="E46" s="25"/>
-      <c r="F46" s="25"/>
-      <c r="G46" s="25"/>
-      <c r="H46" s="25"/>
-      <c r="I46" s="25"/>
-      <c r="J46" s="25"/>
-      <c r="K46" s="25"/>
-      <c r="L46" s="25"/>
-      <c r="M46" s="25"/>
-    </row>
-    <row r="47" spans="2:13" ht="6" customHeight="1"/>
+      <c r="D42" s="25"/>
+      <c r="E42" s="25"/>
+      <c r="F42" s="25"/>
+      <c r="G42" s="25"/>
+      <c r="H42" s="25"/>
+      <c r="I42" s="25"/>
+      <c r="J42" s="25"/>
+      <c r="K42" s="25"/>
+      <c r="L42" s="25"/>
+      <c r="M42" s="25"/>
+    </row>
+    <row r="43" spans="2:13" ht="6" customHeight="1"/>
   </sheetData>
-  <mergeCells count="32">
+  <mergeCells count="24">
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="B10:D11"/>
     <mergeCell ref="B12:D12"/>
@@ -2193,16 +2055,8 @@
     <mergeCell ref="J18:M18"/>
     <mergeCell ref="B19:I19"/>
     <mergeCell ref="J19:M19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="J20:M20"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="J21:M21"/>
-    <mergeCell ref="B22:I22"/>
-    <mergeCell ref="J22:M22"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="J23:M23"/>
-    <mergeCell ref="C44:M44"/>
-    <mergeCell ref="C46:M46"/>
+    <mergeCell ref="C40:M40"/>
+    <mergeCell ref="C42:M42"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.55" header="0.3" footer="0.3"/>
@@ -2221,7 +2075,7 @@
     <tabColor rgb="FF512F8D"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.140625" customWidth="1"/>
@@ -2232,11 +2086,13 @@
     <col min="6" max="6" width="21.7109375" customWidth="1"/>
     <col min="7" max="7" width="18.7109375" customWidth="1"/>
     <col min="8" max="8" width="48.7109375" customWidth="1"/>
-    <col min="9" max="9" width="24.7109375" customWidth="1"/>
-    <col min="10" max="10" width="3.140625" customWidth="1"/>
+    <col min="9" max="9" width="30.7109375" customWidth="1"/>
+    <col min="10" max="10" width="65.7109375" customWidth="1"/>
+    <col min="11" max="11" width="24.7109375" customWidth="1"/>
+    <col min="12" max="12" width="3.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="12" customHeight="1">
+    <row r="1" spans="1:12" ht="12" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2247,11 +2103,13 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10" ht="40" customHeight="1">
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+    </row>
+    <row r="2" spans="1:12" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -2261,8 +2119,10 @@
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-    </row>
-    <row r="3" spans="1:10" ht="22" customHeight="1">
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="3" spans="1:12" ht="22" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="3" t="s">
         <v>1</v>
@@ -2275,8 +2135,10 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-    </row>
-    <row r="4" spans="1:10" ht="20" customHeight="1">
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+    </row>
+    <row r="4" spans="1:12" ht="20" customHeight="1">
       <c r="A4" s="1"/>
       <c r="B4" s="4" t="s">
         <v>2</v>
@@ -2289,8 +2151,10 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-    </row>
-    <row r="5" spans="1:10" ht="5" customHeight="1">
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+    </row>
+    <row r="5" spans="1:12" ht="5" customHeight="1">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -2301,10 +2165,12 @@
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
-    </row>
-    <row r="7" spans="1:10" ht="27" customHeight="1">
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+    </row>
+    <row r="7" spans="1:12" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -2313,477 +2179,315 @@
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
-    </row>
-    <row r="8" spans="1:10" ht="36" customHeight="1">
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+    </row>
+    <row r="8" spans="1:12" ht="36" customHeight="1">
       <c r="B8" s="16" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D8" s="26" t="s">
         <v>14</v>
       </c>
       <c r="E8" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="I8" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="J8" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="G8" s="26" t="s">
+      <c r="K8" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H8" s="26" t="s">
+    </row>
+    <row r="9" spans="1:12" ht="45" customHeight="1">
+      <c r="B9" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="I8" s="17" t="s">
+      <c r="C9" s="27" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" ht="32" customHeight="1">
-      <c r="B9" s="18" t="s">
+      <c r="D9" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="F9" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="27" t="s">
+      <c r="G9" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="F9" s="27" t="s">
+      <c r="H9" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G9" s="28"/>
-      <c r="H9" s="27" t="s">
+      <c r="I9" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="I9" s="19">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="32" customHeight="1">
+      <c r="J9" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="K9" s="19">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="45" customHeight="1">
       <c r="B10" s="20" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="D10" s="29" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="F10" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="G10" s="30" t="s">
+      <c r="H10" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="H10" s="29" t="s">
+      <c r="I10" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="J10" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="I10" s="21">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="32" customHeight="1">
+      <c r="K10" s="21">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="45" customHeight="1">
       <c r="B11" s="18" t="s">
         <v>46</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E11" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="G11" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="27" t="s">
+      <c r="H11" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="G11" s="28"/>
-      <c r="H11" s="27" t="s">
+      <c r="I11" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="I11" s="19">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="32" customHeight="1">
+      <c r="J11" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="K11" s="19">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="45" customHeight="1">
       <c r="B12" s="20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="D12" s="29" t="s">
         <v>16</v>
       </c>
       <c r="E12" s="29" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="F12" s="29" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G12" s="30" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H12" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="I12" s="21">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="32" customHeight="1">
+        <v>52</v>
+      </c>
+      <c r="I12" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="J12" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="K12" s="21">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="45" customHeight="1">
       <c r="B13" s="18" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E13" s="27" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="F13" s="27" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="G13" s="28" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H13" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="I13" s="19">
+        <v>58</v>
+      </c>
+      <c r="I13" s="27" t="s">
+        <v>40</v>
+      </c>
+      <c r="J13" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="K13" s="19">
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="32" customHeight="1">
+    <row r="14" spans="1:12" ht="45" customHeight="1">
       <c r="B14" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>16</v>
-      </c>
-      <c r="E14" s="29" t="s">
-        <v>43</v>
-      </c>
       <c r="F14" s="29" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="G14" s="30" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="H14" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="I14" s="21">
+        <v>62</v>
+      </c>
+      <c r="I14" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="J14" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="K14" s="21">
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="32" customHeight="1">
+    <row r="15" spans="1:12" ht="45" customHeight="1">
       <c r="B15" s="18" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>22</v>
+        <v>65</v>
       </c>
       <c r="F15" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="G15" s="28"/>
+        <v>37</v>
+      </c>
+      <c r="G15" s="28" t="s">
+        <v>66</v>
+      </c>
       <c r="H15" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="I15" s="19">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="32" customHeight="1">
+        <v>67</v>
+      </c>
+      <c r="I15" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="J15" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="K15" s="19">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="45" customHeight="1">
       <c r="B16" s="20" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E16" s="29" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F16" s="29" t="s">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="G16" s="30" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="H16" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="I16" s="21">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" ht="32" customHeight="1">
-      <c r="B17" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17" s="27" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="27" t="s">
-        <v>17</v>
-      </c>
-      <c r="E17" s="27" t="s">
-        <v>61</v>
-      </c>
-      <c r="F17" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="G17" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="H17" s="27" t="s">
-        <v>66</v>
-      </c>
-      <c r="I17" s="19">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18" spans="2:9" ht="32" customHeight="1">
-      <c r="B18" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="C18" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="D18" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="I16" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="F18" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="G18" s="30"/>
-      <c r="H18" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="I18" s="21">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" ht="32" customHeight="1">
-      <c r="B19" s="18" t="s">
+      <c r="J16" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="27" t="s">
-        <v>70</v>
-      </c>
-      <c r="D19" s="27" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19" s="27" t="s">
-        <v>71</v>
-      </c>
-      <c r="F19" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="G19" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="H19" s="27" t="s">
+      <c r="K16" s="21">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" ht="70" customHeight="1">
+      <c r="B18" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="I19" s="19">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="20" spans="2:9" ht="32" customHeight="1">
-      <c r="B20" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="C20" s="29" t="s">
-        <v>70</v>
-      </c>
-      <c r="D20" s="29" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" s="29" t="s">
-        <v>71</v>
-      </c>
-      <c r="F20" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="G20" s="30" t="s">
-        <v>75</v>
-      </c>
-      <c r="H20" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="I20" s="21">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="21" spans="2:9" ht="32" customHeight="1">
-      <c r="B21" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="C21" s="27" t="s">
-        <v>70</v>
-      </c>
-      <c r="D21" s="27" t="s">
-        <v>21</v>
-      </c>
-      <c r="E21" s="27" t="s">
-        <v>78</v>
-      </c>
-      <c r="F21" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="G21" s="28"/>
-      <c r="H21" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="I21" s="19">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="22" spans="2:9" ht="32" customHeight="1">
-      <c r="B22" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="C22" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="D22" s="29" t="s">
-        <v>18</v>
-      </c>
-      <c r="E22" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="F22" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="G22" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="H22" s="29" t="s">
-        <v>83</v>
-      </c>
-      <c r="I22" s="21">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" ht="32" customHeight="1">
-      <c r="B23" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="C23" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="D23" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="E23" s="27" t="s">
-        <v>81</v>
-      </c>
-      <c r="F23" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="G23" s="28" t="s">
-        <v>85</v>
-      </c>
-      <c r="H23" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I23" s="19">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="24" spans="2:9" ht="32" customHeight="1">
-      <c r="B24" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="C24" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="D24" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="E24" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="F24" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="G24" s="30"/>
-      <c r="H24" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="I24" s="21">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="2:9" ht="32" customHeight="1">
-      <c r="B25" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="C25" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="D25" s="27" t="s">
-        <v>16</v>
-      </c>
-      <c r="E25" s="27" t="s">
-        <v>89</v>
-      </c>
-      <c r="F25" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="G25" s="28"/>
-      <c r="H25" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="I25" s="19">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="27" spans="2:9" ht="55" customHeight="1">
-      <c r="B27" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="31"/>
-      <c r="G27" s="31"/>
-      <c r="H27" s="31"/>
-      <c r="I27" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
     </row>
   </sheetData>
-  <autoFilter ref="B8:I25"/>
+  <autoFilter ref="B8:K16"/>
   <mergeCells count="1">
-    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B18:K18"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.55" header="0.3" footer="0.3"/>
@@ -2861,7 +2565,7 @@
     </row>
     <row r="7" spans="1:6" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -2869,27 +2573,27 @@
     </row>
     <row r="8" spans="1:6" ht="36" customHeight="1">
       <c r="B8" s="16" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="C8" s="26" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>93</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="23" customHeight="1">
       <c r="B9" s="18" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>18</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="E9" s="19">
         <v>30</v>
@@ -2897,13 +2601,13 @@
     </row>
     <row r="10" spans="1:6" ht="23" customHeight="1">
       <c r="B10" s="20" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="C10" s="29" t="s">
         <v>18</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="E10" s="21">
         <v>25</v>
@@ -2911,13 +2615,13 @@
     </row>
     <row r="11" spans="1:6" ht="23" customHeight="1">
       <c r="B11" s="18" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>21</v>
+        <v>79</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>21</v>
+        <v>79</v>
       </c>
       <c r="E11" s="19">
         <v>150</v>
@@ -2925,13 +2629,13 @@
     </row>
     <row r="12" spans="1:6" ht="23" customHeight="1">
       <c r="B12" s="20" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="C12" s="29" t="s">
         <v>16</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="E12" s="21">
         <v>100</v>
@@ -2939,13 +2643,13 @@
     </row>
     <row r="13" spans="1:6" ht="23" customHeight="1">
       <c r="B13" s="18" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="E13" s="19">
         <v>97</v>
@@ -2953,13 +2657,13 @@
     </row>
     <row r="14" spans="1:6" ht="23" customHeight="1">
       <c r="B14" s="20" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="E14" s="21">
         <v>100</v>
@@ -2967,13 +2671,13 @@
     </row>
     <row r="15" spans="1:6" ht="23" customHeight="1">
       <c r="B15" s="18" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="C15" s="27" t="s">
         <v>16</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E15" s="19">
         <v>300</v>
@@ -2981,7 +2685,7 @@
     </row>
     <row r="16" spans="1:6" ht="22" customHeight="1">
       <c r="B16" s="22" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C16" s="32"/>
       <c r="D16" s="32"/>
@@ -2992,7 +2696,7 @@
     </row>
     <row r="18" spans="2:5" ht="45" customHeight="1">
       <c r="B18" s="31" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="C18" s="31"/>
       <c r="D18" s="31"/>
@@ -3042,7 +2746,7 @@
     <row r="2" spans="1:6" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3079,7 +2783,7 @@
     </row>
     <row r="7" spans="1:6" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -3087,47 +2791,47 @@
     </row>
     <row r="8" spans="1:6" ht="34" customHeight="1">
       <c r="B8" s="16" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C8" s="16"/>
       <c r="D8" s="17" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="25" customHeight="1">
       <c r="B9" s="18" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="C9" s="18"/>
       <c r="D9" s="19">
         <v>145523</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="25" customHeight="1">
       <c r="B10" s="20" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="C10" s="20"/>
       <c r="D10" s="21">
         <v>44098</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="25" customHeight="1">
       <c r="B11" s="18" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="C11" s="18"/>
       <c r="D11" s="33" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="E11" s="35">
         <v>13405351.02</v>
@@ -3135,7 +2839,7 @@
     </row>
     <row r="13" spans="1:6" ht="40" customHeight="1">
       <c r="B13" s="31" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="C13" s="31"/>
       <c r="D13" s="31"/>
@@ -3143,7 +2847,7 @@
     </row>
     <row r="15" spans="1:6" ht="27" customHeight="1">
       <c r="B15" s="6" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -3154,21 +2858,21 @@
         <v>14</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="24" customHeight="1">
       <c r="B17" s="18" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="D17" s="19">
         <v>1</v>
@@ -3182,7 +2886,7 @@
         <v>16</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="D18" s="21">
         <v>67</v>
@@ -3196,7 +2900,7 @@
         <v>18</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="D19" s="19">
         <v>45</v>
@@ -3207,7 +2911,7 @@
     </row>
     <row r="20" spans="2:5" ht="22" customHeight="1">
       <c r="B20" s="22" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C20" s="32"/>
       <c r="D20" s="23">
@@ -3221,7 +2925,7 @@
     </row>
     <row r="22" spans="2:5" ht="27" customHeight="1">
       <c r="B22" s="6" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="7"/>
@@ -3232,13 +2936,13 @@
         <v>14</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="24" customHeight="1">
@@ -3246,7 +2950,7 @@
         <v>17</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="D24" s="19">
         <v>181</v>
@@ -3257,10 +2961,10 @@
     </row>
     <row r="25" spans="2:5" ht="24" customHeight="1">
       <c r="B25" s="20" t="s">
-        <v>21</v>
+        <v>79</v>
       </c>
       <c r="C25" s="29" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="D25" s="21">
         <v>530</v>
@@ -3274,7 +2978,7 @@
         <v>16</v>
       </c>
       <c r="C26" s="27" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="D26" s="19">
         <v>344</v>
@@ -3285,10 +2989,10 @@
     </row>
     <row r="27" spans="2:5" ht="24" customHeight="1">
       <c r="B27" s="20" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="C27" s="29" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="D27" s="21">
         <v>5</v>
@@ -3299,10 +3003,10 @@
     </row>
     <row r="28" spans="2:5" ht="24" customHeight="1">
       <c r="B28" s="18" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="C28" s="27" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="D28" s="19">
         <v>109</v>
@@ -3313,7 +3017,7 @@
     </row>
     <row r="29" spans="2:5" ht="22" customHeight="1">
       <c r="B29" s="22" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C29" s="32"/>
       <c r="D29" s="23">
@@ -3327,7 +3031,7 @@
     </row>
     <row r="31" spans="2:5" ht="100" customHeight="1">
       <c r="B31" s="31" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="C31" s="31"/>
       <c r="D31" s="31"/>
@@ -3359,7 +3063,7 @@
     <tabColor rgb="FF5A5765"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.140625" customWidth="1"/>
@@ -3377,7 +3081,7 @@
     <row r="2" spans="1:4" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3406,21 +3110,21 @@
     </row>
     <row r="7" spans="1:4" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="C7" s="7"/>
     </row>
     <row r="8" spans="1:4" ht="34" customHeight="1">
       <c r="B8" s="16" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="22" customHeight="1">
       <c r="B9" s="18" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>4</v>
@@ -3428,148 +3132,156 @@
     </row>
     <row r="10" spans="1:4" ht="22" customHeight="1">
       <c r="B10" s="20" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="22" customHeight="1">
       <c r="B11" s="18" t="s">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="22" customHeight="1">
       <c r="B12" s="20" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="27" customHeight="1">
       <c r="B14" s="6" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="C14" s="7"/>
     </row>
     <row r="15" spans="1:4" ht="34" customHeight="1">
       <c r="B15" s="16" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="60" customHeight="1">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="120" customHeight="1">
       <c r="B16" s="18" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="27" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="40" customHeight="1">
       <c r="B17" s="20" t="s">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="75" customHeight="1">
       <c r="B18" s="18" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" ht="45" customHeight="1">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" ht="40" customHeight="1">
       <c r="B19" s="20" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="C19" s="29" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="27" customHeight="1">
       <c r="B21" s="6" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="C21" s="7"/>
     </row>
     <row r="22" spans="2:3" ht="34" customHeight="1">
       <c r="B22" s="38" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="C22" s="39" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23" spans="2:3" ht="34" customHeight="1">
       <c r="B23" s="38" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="C23" s="39" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="34" customHeight="1">
       <c r="B24" s="38" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
       <c r="C24" s="39" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="26" spans="2:3" ht="27" customHeight="1">
-      <c r="B26" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="C26" s="7"/>
-    </row>
-    <row r="27" spans="2:3" ht="22" customHeight="1">
-      <c r="B27" s="40" t="s">
-        <v>141</v>
-      </c>
-      <c r="C27" s="41" t="s">
-        <v>3</v>
-      </c>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" ht="34" customHeight="1">
+      <c r="B25" s="38" t="s">
+        <v>124</v>
+      </c>
+      <c r="C25" s="39" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" ht="27" customHeight="1">
+      <c r="B27" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C27" s="7"/>
     </row>
     <row r="28" spans="2:3" ht="22" customHeight="1">
       <c r="B28" s="40" t="s">
-        <v>15</v>
+        <v>127</v>
       </c>
       <c r="C28" s="41" t="s">
-        <v>142</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29" spans="2:3" ht="22" customHeight="1">
       <c r="B29" s="40" t="s">
-        <v>93</v>
+        <v>15</v>
       </c>
       <c r="C29" s="41" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="22" customHeight="1">
       <c r="B30" s="40" t="s">
-        <v>127</v>
+        <v>76</v>
       </c>
       <c r="C30" s="41" t="s">
-        <v>144</v>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" ht="22" customHeight="1">
+      <c r="B31" s="40" t="s">
+        <v>111</v>
+      </c>
+      <c r="C31" s="41" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B27" location="'Resumen'!A1" tooltip="Ir a la hoja Resumen" display="Resumen"/>
-    <hyperlink ref="B28" location="'Alertas'!A1" tooltip="Ir a la hoja Alertas" display="Alertas"/>
-    <hyperlink ref="B29" location="'Kits'!A1" tooltip="Ir a la hoja Kits" display="Kits"/>
-    <hyperlink ref="B30" location="'Bonos'!A1" tooltip="Ir a la hoja Bonos" display="Bonos"/>
+    <hyperlink ref="B28" location="'Resumen'!A1" tooltip="Ir a la hoja Resumen" display="Resumen"/>
+    <hyperlink ref="B29" location="'Alertas'!A1" tooltip="Ir a la hoja Alertas" display="Alertas"/>
+    <hyperlink ref="B30" location="'Kits'!A1" tooltip="Ir a la hoja Kits" display="Kits"/>
+    <hyperlink ref="B31" location="'Bonos'!A1" tooltip="Ir a la hoja Bonos" display="Bonos"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.55" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Completar alertas desde el 14 de septiembre y validar tablero y exportables
</commit_message>
<xml_diff>
--- a/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
+++ b/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Ficha técnica" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Alertas!$B$8:$K$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Alertas!$B$8:$K$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Kits!$B$8:$E$15</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Resumen!$A$1:$N$44</definedName>
   </definedNames>
@@ -23,9 +23,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="131">
-  <si>
-    <t>Riesgos y respuesta</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="151">
+  <si>
+    <t>Seguimiento y respuesta MTDH</t>
   </si>
   <si>
     <t>14/09 al 26/10/2026 · Nacional · Alertas, kits y bono de contingencia</t>
@@ -52,10 +52,10 @@
     <t>Pendientes o en seguimiento</t>
   </si>
   <si>
-    <t>UA con afectación documentada</t>
-  </si>
-  <si>
-    <t>Códigos de unidad distintos</t>
+    <t>UA afectadas con código</t>
+  </si>
+  <si>
+    <t>Solo códigos registrados en la fuente</t>
   </si>
   <si>
     <t>Kits entregados</t>
@@ -73,22 +73,22 @@
     <t>Alertas</t>
   </si>
   <si>
+    <t>Manabí</t>
+  </si>
+  <si>
     <t>Guayas</t>
   </si>
   <si>
     <t>El Oro</t>
   </si>
   <si>
-    <t>Manabí</t>
-  </si>
-  <si>
     <t>Total de la selección</t>
   </si>
   <si>
     <t>Aspectos destacados</t>
   </si>
   <si>
-    <t>8 alertas con afectación a servicios MTDH desde el 14/09 en 3 provincias.</t>
+    <t>13 alertas con afectación a servicios MTDH desde el 14/09 en 3 provincias.</t>
   </si>
   <si>
     <t>802 kits documentados en el fin de semana del 24–25/10.</t>
@@ -244,6 +244,66 @@
     <t>CORREO INFANTIL</t>
   </si>
   <si>
+    <t>ALT-2026-000291</t>
+  </si>
+  <si>
+    <t>2026-09-27</t>
+  </si>
+  <si>
+    <t>Balao</t>
+  </si>
+  <si>
+    <t>CNH Cien Familias</t>
+  </si>
+  <si>
+    <t>Inundación que afecta la prestación del servicio</t>
+  </si>
+  <si>
+    <t>ALT-2026-000288</t>
+  </si>
+  <si>
+    <t>2026-09-24</t>
+  </si>
+  <si>
+    <t>Junín</t>
+  </si>
+  <si>
+    <t>CDI Divino Niño</t>
+  </si>
+  <si>
+    <t>Filtración de agua en instalaciones; limpieza para continuar la atención</t>
+  </si>
+  <si>
+    <t>ALT-2026-000289</t>
+  </si>
+  <si>
+    <t>Chone</t>
+  </si>
+  <si>
+    <t>CDI Mis Pequeños Traviesos</t>
+  </si>
+  <si>
+    <t>Filtraciones e inundación; actividades suspendidas; nombre de UA por validar</t>
+  </si>
+  <si>
+    <t>ALT-2026-000283</t>
+  </si>
+  <si>
+    <t>CDI Gotitas de Miel</t>
+  </si>
+  <si>
+    <t>Ingreso de agua; suspensión del servicio el 24/09 y limpieza; actividades retomadas</t>
+  </si>
+  <si>
+    <t>ALT-2026-000287</t>
+  </si>
+  <si>
+    <t>CDI Lucerito</t>
+  </si>
+  <si>
+    <t>Filtraciones e ingreso de agua; limpieza sin suspensión del servicio</t>
+  </si>
+  <si>
     <t>Solo se incluyen alertas con afectación documentada a instalaciones, acceso, continuidad o modalidad de atención de los servicios MTDH, registradas desde el 14 de septiembre de 2026. Se excluyen daños externos o a viviendas de familias usuarias sin impacto documentado en el servicio. Un código UA por sí solo no acredita afectación. La fecha corresponde al registro de la alerta; una alerta no equivale necesariamente a un evento único. El campo Afectados mezcla personas, familias y usuarios, por lo que no se presenta un total de personas únicas. La base no certifica atribución causal a ENOS.</t>
   </si>
   <si>
@@ -373,7 +433,7 @@
     <t>Control de calidad</t>
   </si>
   <si>
-    <t>Se revisaron Detalle y Acciones realizadas de cada alerta. Los casos sin evidencia de afectación al servicio no se incorporan a indicadores ni exportables.</t>
+    <t>Solo afectaciones documentadas al servicio. En el corte nacional, cinco alertas carecen de código UA. En ALT-2026-000289 el nombre difiere entre Detalle y Acciones realizadas; requiere validación.</t>
   </si>
   <si>
     <t>Fuentes oficiales</t>
@@ -382,7 +442,7 @@
     <t>Fuente 1</t>
   </si>
   <si>
-    <t>05-analisis-alertas-2026-10-26-2-.xlsx</t>
+    <t>01-analisis-alertas-2026-10-26-2-.xlsx</t>
   </si>
   <si>
     <t>Fuente 2</t>
@@ -932,13 +992,13 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
+                  <c:v>Manabí</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>Guayas</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>El Oro</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Manabí</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -950,10 +1010,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>4</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
@@ -1818,12 +1878,12 @@
     </row>
     <row r="10" spans="1:14" ht="21" customHeight="1">
       <c r="B10" s="13">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
       <c r="E10" s="13">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F10" s="14"/>
       <c r="G10" s="14"/>
@@ -1920,7 +1980,7 @@
       <c r="H16" s="18"/>
       <c r="I16" s="18"/>
       <c r="J16" s="19">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K16" s="19"/>
       <c r="L16" s="19"/>
@@ -1938,7 +1998,7 @@
       <c r="H17" s="20"/>
       <c r="I17" s="20"/>
       <c r="J17" s="21">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K17" s="21"/>
       <c r="L17" s="21"/>
@@ -1975,7 +2035,7 @@
       <c r="I19" s="22"/>
       <c r="J19" s="23">
         <f>SUM(J16:J18)</f>
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="K19" s="23"/>
       <c r="L19" s="23"/>
@@ -2075,7 +2135,7 @@
     <tabColor rgb="FF512F8D"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.140625" customWidth="1"/>
@@ -2222,7 +2282,7 @@
         <v>35</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E9" s="27" t="s">
         <v>36</v>
@@ -2254,7 +2314,7 @@
         <v>35</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E10" s="29" t="s">
         <v>36</v>
@@ -2286,7 +2346,7 @@
         <v>35</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E11" s="27" t="s">
         <v>36</v>
@@ -2318,7 +2378,7 @@
         <v>35</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E12" s="29" t="s">
         <v>36</v>
@@ -2350,7 +2410,7 @@
         <v>35</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E13" s="27" t="s">
         <v>55</v>
@@ -2382,7 +2442,7 @@
         <v>35</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E14" s="29" t="s">
         <v>55</v>
@@ -2414,7 +2474,7 @@
         <v>64</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E15" s="27" t="s">
         <v>65</v>
@@ -2446,7 +2506,7 @@
         <v>64</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E16" s="29" t="s">
         <v>65</v>
@@ -2470,24 +2530,174 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="2:11" ht="70" customHeight="1">
-      <c r="B18" s="31" t="s">
+    <row r="17" spans="2:11" ht="45" customHeight="1">
+      <c r="B17" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="31"/>
-      <c r="H18" s="31"/>
-      <c r="I18" s="31"/>
-      <c r="J18" s="31"/>
-      <c r="K18" s="31"/>
+      <c r="C17" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" s="27" t="s">
+        <v>75</v>
+      </c>
+      <c r="F17" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="G17" s="28"/>
+      <c r="H17" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="I17" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="J17" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="K17" s="19">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" ht="45" customHeight="1">
+      <c r="B18" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="C18" s="29" t="s">
+        <v>79</v>
+      </c>
+      <c r="D18" s="29" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="F18" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="G18" s="30"/>
+      <c r="H18" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="I18" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="J18" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="K18" s="21">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" ht="45" customHeight="1">
+      <c r="B19" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="D19" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="F19" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="G19" s="28"/>
+      <c r="H19" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="I19" s="27" t="s">
+        <v>40</v>
+      </c>
+      <c r="J19" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="K19" s="19">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" ht="45" customHeight="1">
+      <c r="B20" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>79</v>
+      </c>
+      <c r="D20" s="29" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="F20" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="G20" s="30"/>
+      <c r="H20" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="I20" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="J20" s="29" t="s">
+        <v>89</v>
+      </c>
+      <c r="K20" s="21">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" ht="45" customHeight="1">
+      <c r="B21" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="C21" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="D21" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="F21" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="G21" s="28"/>
+      <c r="H21" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="I21" s="27" t="s">
+        <v>40</v>
+      </c>
+      <c r="J21" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="K21" s="19">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" ht="70" customHeight="1">
+      <c r="B23" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="31"/>
+      <c r="G23" s="31"/>
+      <c r="H23" s="31"/>
+      <c r="I23" s="31"/>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31"/>
     </row>
   </sheetData>
-  <autoFilter ref="B8:K16"/>
+  <autoFilter ref="B8:K21"/>
   <mergeCells count="1">
-    <mergeCell ref="B18:K18"/>
+    <mergeCell ref="B23:K23"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.55" header="0.3" footer="0.3"/>
@@ -2565,7 +2775,7 @@
     </row>
     <row r="7" spans="1:6" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -2573,7 +2783,7 @@
     </row>
     <row r="8" spans="1:6" ht="36" customHeight="1">
       <c r="B8" s="16" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="C8" s="26" t="s">
         <v>14</v>
@@ -2582,18 +2792,18 @@
         <v>27</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="23" customHeight="1">
       <c r="B9" s="18" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="E9" s="19">
         <v>30</v>
@@ -2601,13 +2811,13 @@
     </row>
     <row r="10" spans="1:6" ht="23" customHeight="1">
       <c r="B10" s="20" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="E10" s="21">
         <v>25</v>
@@ -2615,13 +2825,13 @@
     </row>
     <row r="11" spans="1:6" ht="23" customHeight="1">
       <c r="B11" s="18" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="E11" s="19">
         <v>150</v>
@@ -2629,13 +2839,13 @@
     </row>
     <row r="12" spans="1:6" ht="23" customHeight="1">
       <c r="B12" s="20" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="E12" s="21">
         <v>100</v>
@@ -2643,13 +2853,13 @@
     </row>
     <row r="13" spans="1:6" ht="23" customHeight="1">
       <c r="B13" s="18" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="E13" s="19">
         <v>97</v>
@@ -2657,13 +2867,13 @@
     </row>
     <row r="14" spans="1:6" ht="23" customHeight="1">
       <c r="B14" s="20" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="E14" s="21">
         <v>100</v>
@@ -2671,10 +2881,10 @@
     </row>
     <row r="15" spans="1:6" ht="23" customHeight="1">
       <c r="B15" s="18" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D15" s="27" t="s">
         <v>36</v>
@@ -2696,7 +2906,7 @@
     </row>
     <row r="18" spans="2:5" ht="45" customHeight="1">
       <c r="B18" s="31" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="C18" s="31"/>
       <c r="D18" s="31"/>
@@ -2746,7 +2956,7 @@
     <row r="2" spans="1:6" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -2783,7 +2993,7 @@
     </row>
     <row r="7" spans="1:6" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -2791,47 +3001,47 @@
     </row>
     <row r="8" spans="1:6" ht="34" customHeight="1">
       <c r="B8" s="16" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="C8" s="16"/>
       <c r="D8" s="17" t="s">
-        <v>88</v>
+        <v>108</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>89</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="25" customHeight="1">
       <c r="B9" s="18" t="s">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="C9" s="18"/>
       <c r="D9" s="19">
         <v>145523</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>91</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="25" customHeight="1">
       <c r="B10" s="20" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
       <c r="C10" s="20"/>
       <c r="D10" s="21">
         <v>44098</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>91</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="25" customHeight="1">
       <c r="B11" s="18" t="s">
-        <v>93</v>
+        <v>113</v>
       </c>
       <c r="C11" s="18"/>
       <c r="D11" s="33" t="s">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="E11" s="35">
         <v>13405351.02</v>
@@ -2839,7 +3049,7 @@
     </row>
     <row r="13" spans="1:6" ht="40" customHeight="1">
       <c r="B13" s="31" t="s">
-        <v>94</v>
+        <v>114</v>
       </c>
       <c r="C13" s="31"/>
       <c r="D13" s="31"/>
@@ -2847,7 +3057,7 @@
     </row>
     <row r="15" spans="1:6" ht="27" customHeight="1">
       <c r="B15" s="6" t="s">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -2858,21 +3068,21 @@
         <v>14</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>97</v>
+        <v>117</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>89</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="24" customHeight="1">
       <c r="B17" s="18" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="D17" s="19">
         <v>1</v>
@@ -2883,10 +3093,10 @@
     </row>
     <row r="18" spans="2:5" ht="24" customHeight="1">
       <c r="B18" s="20" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="D18" s="21">
         <v>67</v>
@@ -2897,10 +3107,10 @@
     </row>
     <row r="19" spans="2:5" ht="24" customHeight="1">
       <c r="B19" s="18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="D19" s="19">
         <v>45</v>
@@ -2925,7 +3135,7 @@
     </row>
     <row r="22" spans="2:5" ht="27" customHeight="1">
       <c r="B22" s="6" t="s">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="7"/>
@@ -2936,21 +3146,21 @@
         <v>14</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>97</v>
+        <v>117</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>89</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="24" customHeight="1">
       <c r="B24" s="18" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="D24" s="19">
         <v>181</v>
@@ -2961,10 +3171,10 @@
     </row>
     <row r="25" spans="2:5" ht="24" customHeight="1">
       <c r="B25" s="20" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="C25" s="29" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="D25" s="21">
         <v>530</v>
@@ -2975,10 +3185,10 @@
     </row>
     <row r="26" spans="2:5" ht="24" customHeight="1">
       <c r="B26" s="18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C26" s="27" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="D26" s="19">
         <v>344</v>
@@ -2989,10 +3199,10 @@
     </row>
     <row r="27" spans="2:5" ht="24" customHeight="1">
       <c r="B27" s="20" t="s">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="C27" s="29" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="D27" s="21">
         <v>5</v>
@@ -3003,10 +3213,10 @@
     </row>
     <row r="28" spans="2:5" ht="24" customHeight="1">
       <c r="B28" s="18" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="C28" s="27" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="D28" s="19">
         <v>109</v>
@@ -3031,7 +3241,7 @@
     </row>
     <row r="31" spans="2:5" ht="100" customHeight="1">
       <c r="B31" s="31" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="C31" s="31"/>
       <c r="D31" s="31"/>
@@ -3081,7 +3291,7 @@
     <row r="2" spans="1:4" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3110,21 +3320,21 @@
     </row>
     <row r="7" spans="1:4" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>104</v>
+        <v>124</v>
       </c>
       <c r="C7" s="7"/>
     </row>
     <row r="8" spans="1:4" ht="34" customHeight="1">
       <c r="B8" s="16" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>106</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="22" customHeight="1">
       <c r="B9" s="18" t="s">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>4</v>
@@ -3132,40 +3342,40 @@
     </row>
     <row r="10" spans="1:4" ht="22" customHeight="1">
       <c r="B10" s="20" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>109</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="22" customHeight="1">
       <c r="B11" s="18" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="22" customHeight="1">
       <c r="B12" s="20" t="s">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>112</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="27" customHeight="1">
       <c r="B14" s="6" t="s">
-        <v>113</v>
+        <v>133</v>
       </c>
       <c r="C14" s="7"/>
     </row>
     <row r="15" spans="1:4" ht="34" customHeight="1">
       <c r="B15" s="16" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>114</v>
+        <v>134</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="120" customHeight="1">
@@ -3173,80 +3383,80 @@
         <v>15</v>
       </c>
       <c r="C16" s="27" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="40" customHeight="1">
       <c r="B17" s="20" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="75" customHeight="1">
       <c r="B18" s="18" t="s">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" ht="40" customHeight="1">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" ht="45" customHeight="1">
       <c r="B19" s="20" t="s">
-        <v>115</v>
+        <v>135</v>
       </c>
       <c r="C19" s="29" t="s">
-        <v>116</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="27" customHeight="1">
       <c r="B21" s="6" t="s">
-        <v>117</v>
+        <v>137</v>
       </c>
       <c r="C21" s="7"/>
     </row>
     <row r="22" spans="2:3" ht="34" customHeight="1">
       <c r="B22" s="38" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="C22" s="39" t="s">
-        <v>119</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" spans="2:3" ht="34" customHeight="1">
       <c r="B23" s="38" t="s">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="C23" s="39" t="s">
-        <v>121</v>
+        <v>141</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="34" customHeight="1">
       <c r="B24" s="38" t="s">
-        <v>122</v>
+        <v>142</v>
       </c>
       <c r="C24" s="39" t="s">
-        <v>123</v>
+        <v>143</v>
       </c>
     </row>
     <row r="25" spans="2:3" ht="34" customHeight="1">
       <c r="B25" s="38" t="s">
-        <v>124</v>
+        <v>144</v>
       </c>
       <c r="C25" s="39" t="s">
-        <v>125</v>
+        <v>145</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="27" customHeight="1">
       <c r="B27" s="6" t="s">
-        <v>126</v>
+        <v>146</v>
       </c>
       <c r="C27" s="7"/>
     </row>
     <row r="28" spans="2:3" ht="22" customHeight="1">
       <c r="B28" s="40" t="s">
-        <v>127</v>
+        <v>147</v>
       </c>
       <c r="C28" s="41" t="s">
         <v>3</v>
@@ -3257,23 +3467,23 @@
         <v>15</v>
       </c>
       <c r="C29" s="41" t="s">
-        <v>128</v>
+        <v>148</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="22" customHeight="1">
       <c r="B30" s="40" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="C30" s="41" t="s">
-        <v>129</v>
+        <v>149</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="22" customHeight="1">
       <c r="B31" s="40" t="s">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="C31" s="41" t="s">
-        <v>130</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aclarar entregas de kits en provincias priorizadas en tablero y exportables
</commit_message>
<xml_diff>
--- a/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
+++ b/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="152">
   <si>
     <t>Seguimiento y respuesta MTDH</t>
   </si>
@@ -61,7 +61,7 @@
     <t>Kits entregados</t>
   </si>
   <si>
-    <t>Fin de semana 24–25/10</t>
+    <t>Provincias priorizadas · 24–25/10</t>
   </si>
   <si>
     <t>Alertas por provincia</t>
@@ -91,7 +91,7 @@
     <t>13 alertas con afectación a servicios MTDH desde el 14/09 en 3 provincias.</t>
   </si>
   <si>
-    <t>802 kits documentados en el fin de semana del 24–25/10.</t>
+    <t>802 kits entregados en provincias priorizadas el 24–25/10.</t>
   </si>
   <si>
     <t>Afectaciones a servicios MTDH</t>
@@ -307,6 +307,9 @@
     <t>Solo se incluyen alertas con afectación documentada a instalaciones, acceso, continuidad o modalidad de atención de los servicios MTDH, registradas desde el 14 de septiembre de 2026. Se excluyen daños externos o a viviendas de familias usuarias sin impacto documentado en el servicio. Un código UA por sí solo no acredita afectación. La fecha corresponde al registro de la alerta; una alerta no equivale necesariamente a un evento único. El campo Afectados mezcla personas, familias y usuarios, por lo que no se presenta un total de personas únicas. La base no certifica atribución causal a ENOS.</t>
   </si>
   <si>
+    <t>Kits entregados en provincias priorizadas</t>
+  </si>
+  <si>
     <t>Entregas de fin de semana</t>
   </si>
   <si>
@@ -337,7 +340,7 @@
     <t>2026-10-25</t>
   </si>
   <si>
-    <t>Entregas documentadas del 24 y 25 de octubre de 2026, corte 25/10 a las 19:00. No representan el acumulado desde el 14/09.</t>
+    <t>Kits entregados en provincias priorizadas el 24–25/10/2026; corte 25/10, 19:00. No es el acumulado desde el 14/09.</t>
   </si>
   <si>
     <t>Bono de contingencia</t>
@@ -2738,7 +2741,7 @@
     <row r="2" spans="1:6" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>11</v>
+        <v>94</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -2775,7 +2778,7 @@
     </row>
     <row r="7" spans="1:6" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -2783,7 +2786,7 @@
     </row>
     <row r="8" spans="1:6" ht="36" customHeight="1">
       <c r="B8" s="16" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C8" s="26" t="s">
         <v>14</v>
@@ -2792,18 +2795,18 @@
         <v>27</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="23" customHeight="1">
       <c r="B9" s="18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E9" s="19">
         <v>30</v>
@@ -2811,13 +2814,13 @@
     </row>
     <row r="10" spans="1:6" ht="23" customHeight="1">
       <c r="B10" s="20" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C10" s="29" t="s">
         <v>16</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E10" s="21">
         <v>25</v>
@@ -2825,13 +2828,13 @@
     </row>
     <row r="11" spans="1:6" ht="23" customHeight="1">
       <c r="B11" s="18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E11" s="19">
         <v>150</v>
@@ -2839,13 +2842,13 @@
     </row>
     <row r="12" spans="1:6" ht="23" customHeight="1">
       <c r="B12" s="20" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C12" s="29" t="s">
         <v>17</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E12" s="21">
         <v>100</v>
@@ -2853,13 +2856,13 @@
     </row>
     <row r="13" spans="1:6" ht="23" customHeight="1">
       <c r="B13" s="18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E13" s="19">
         <v>97</v>
@@ -2867,13 +2870,13 @@
     </row>
     <row r="14" spans="1:6" ht="23" customHeight="1">
       <c r="B14" s="20" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E14" s="21">
         <v>100</v>
@@ -2881,7 +2884,7 @@
     </row>
     <row r="15" spans="1:6" ht="23" customHeight="1">
       <c r="B15" s="18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C15" s="27" t="s">
         <v>17</v>
@@ -2906,7 +2909,7 @@
     </row>
     <row r="18" spans="2:5" ht="45" customHeight="1">
       <c r="B18" s="31" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C18" s="31"/>
       <c r="D18" s="31"/>
@@ -2956,7 +2959,7 @@
     <row r="2" spans="1:6" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -2993,7 +2996,7 @@
     </row>
     <row r="7" spans="1:6" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -3001,47 +3004,47 @@
     </row>
     <row r="8" spans="1:6" ht="34" customHeight="1">
       <c r="B8" s="16" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C8" s="16"/>
       <c r="D8" s="17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="25" customHeight="1">
       <c r="B9" s="18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C9" s="18"/>
       <c r="D9" s="19">
         <v>145523</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="25" customHeight="1">
       <c r="B10" s="20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C10" s="20"/>
       <c r="D10" s="21">
         <v>44098</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="25" customHeight="1">
       <c r="B11" s="18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C11" s="18"/>
       <c r="D11" s="33" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E11" s="35">
         <v>13405351.02</v>
@@ -3049,7 +3052,7 @@
     </row>
     <row r="13" spans="1:6" ht="40" customHeight="1">
       <c r="B13" s="31" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C13" s="31"/>
       <c r="D13" s="31"/>
@@ -3057,7 +3060,7 @@
     </row>
     <row r="15" spans="1:6" ht="27" customHeight="1">
       <c r="B15" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -3068,21 +3071,21 @@
         <v>14</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="24" customHeight="1">
       <c r="B17" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D17" s="19">
         <v>1</v>
@@ -3096,7 +3099,7 @@
         <v>17</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D18" s="21">
         <v>67</v>
@@ -3110,7 +3113,7 @@
         <v>16</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D19" s="19">
         <v>45</v>
@@ -3135,7 +3138,7 @@
     </row>
     <row r="22" spans="2:5" ht="27" customHeight="1">
       <c r="B22" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="7"/>
@@ -3146,13 +3149,13 @@
         <v>14</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="24" customHeight="1">
@@ -3160,7 +3163,7 @@
         <v>18</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D24" s="19">
         <v>181</v>
@@ -3171,10 +3174,10 @@
     </row>
     <row r="25" spans="2:5" ht="24" customHeight="1">
       <c r="B25" s="20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C25" s="29" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D25" s="21">
         <v>530</v>
@@ -3188,7 +3191,7 @@
         <v>17</v>
       </c>
       <c r="C26" s="27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D26" s="19">
         <v>344</v>
@@ -3199,10 +3202,10 @@
     </row>
     <row r="27" spans="2:5" ht="24" customHeight="1">
       <c r="B27" s="20" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C27" s="29" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D27" s="21">
         <v>5</v>
@@ -3213,10 +3216,10 @@
     </row>
     <row r="28" spans="2:5" ht="24" customHeight="1">
       <c r="B28" s="18" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C28" s="27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D28" s="19">
         <v>109</v>
@@ -3241,7 +3244,7 @@
     </row>
     <row r="31" spans="2:5" ht="100" customHeight="1">
       <c r="B31" s="31" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C31" s="31"/>
       <c r="D31" s="31"/>
@@ -3291,7 +3294,7 @@
     <row r="2" spans="1:4" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3320,21 +3323,21 @@
     </row>
     <row r="7" spans="1:4" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C7" s="7"/>
     </row>
     <row r="8" spans="1:4" ht="34" customHeight="1">
       <c r="B8" s="16" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="22" customHeight="1">
       <c r="B9" s="18" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>4</v>
@@ -3342,40 +3345,40 @@
     </row>
     <row r="10" spans="1:4" ht="22" customHeight="1">
       <c r="B10" s="20" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="22" customHeight="1">
       <c r="B11" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="22" customHeight="1">
       <c r="B12" s="20" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="27" customHeight="1">
       <c r="B14" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C14" s="7"/>
     </row>
     <row r="15" spans="1:4" ht="34" customHeight="1">
       <c r="B15" s="16" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="120" customHeight="1">
@@ -3388,75 +3391,75 @@
     </row>
     <row r="17" spans="2:3" ht="40" customHeight="1">
       <c r="B17" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="75" customHeight="1">
       <c r="B18" s="18" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19" spans="2:3" ht="45" customHeight="1">
       <c r="B19" s="20" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C19" s="29" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="27" customHeight="1">
       <c r="B21" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C21" s="7"/>
     </row>
     <row r="22" spans="2:3" ht="34" customHeight="1">
       <c r="B22" s="38" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C22" s="39" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="23" spans="2:3" ht="34" customHeight="1">
       <c r="B23" s="38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C23" s="39" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="34" customHeight="1">
       <c r="B24" s="38" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C24" s="39" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25" spans="2:3" ht="34" customHeight="1">
       <c r="B25" s="38" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C25" s="39" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="27" customHeight="1">
       <c r="B27" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C27" s="7"/>
     </row>
     <row r="28" spans="2:3" ht="22" customHeight="1">
       <c r="B28" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C28" s="41" t="s">
         <v>3</v>
@@ -3467,23 +3470,23 @@
         <v>15</v>
       </c>
       <c r="C29" s="41" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="22" customHeight="1">
       <c r="B30" s="40" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C30" s="41" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="22" customHeight="1">
       <c r="B31" s="40" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C31" s="41" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rediseñar el resumen ejecutivo de Riesgos en tres páginas y ajustar nota del bono
</commit_message>
<xml_diff>
--- a/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
+++ b/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
@@ -63,7 +63,7 @@
     <t>Monto de bonos gestionados</t>
   </si>
   <si>
-    <t>Gestionado no acredita cobro</t>
+    <t>Corte del bono: 23/10/2026</t>
   </si>
   <si>
     <t>Alertas por provincia</t>
@@ -540,7 +540,7 @@
     <t>Bono de contingencia</t>
   </si>
   <si>
-    <t>La ayuda memoria no identifica pagos exclusivamente atribuibles a ENOS ni fechas individuales para recortar desde el 14/09. Se muestran únicamente las filas de inundación como referencia: pagos gestionados desde el 29/08 y casos en articulación al 23/10. Gestionado no acredita cobro; articulación no equivale a pago. Las proyecciones corresponden a planificación nacional 2026–2027.</t>
+    <t>La ayuda memoria no identifica pagos exclusivamente atribuibles a ENOS ni fechas individuales para recortar desde el 14/09. Se muestran únicamente las filas de inundación como referencia: pagos gestionados desde el 29/08 y casos en articulación al 23/10. Articulación no equivale a pago. Las proyecciones corresponden a planificación nacional 2026–2027.</t>
   </si>
   <si>
     <t>Filtros</t>
@@ -4965,7 +4965,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="87" customHeight="1">
+    <row r="15" spans="1:4" ht="72" customHeight="1">
       <c r="B15" s="36" t="s">
         <v>170</v>
       </c>

</xml_diff>

<commit_message>
Incorporar KPI de unidades cerradas y gráficos de continuidad en Riesgos
</commit_message>
<xml_diff>
--- a/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
+++ b/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
@@ -17,15 +17,15 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Alertas!$B$7:$K$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Evolución!$B$7:$D$50</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'Ficha técnica'!$A$1:$D$17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Resumen!$A$1:$N$98</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Ficha técnica'!$A$1:$D$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Resumen!$A$1:$N$142</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="186">
   <si>
     <t>Riesgos · Respuesta del Ministerio</t>
   </si>
@@ -66,21 +66,51 @@
     <t>Corte del bono: 23/10/2026</t>
   </si>
   <si>
+    <t>Unidades de atención cerradas</t>
+  </si>
+  <si>
+    <t>Atención suspendida · corte 26/10/2026, 16:00</t>
+  </si>
+  <si>
+    <t>Unidades cerradas por provincia</t>
+  </si>
+  <si>
+    <t>Categoría</t>
+  </si>
+  <si>
+    <t>Unidades</t>
+  </si>
+  <si>
+    <t>El Oro</t>
+  </si>
+  <si>
+    <t>Santa Elena</t>
+  </si>
+  <si>
+    <t>Estado de atención reportado</t>
+  </si>
+  <si>
+    <t>CNH: suspensión presencial</t>
+  </si>
+  <si>
+    <t>Cerradas / suspendidas</t>
+  </si>
+  <si>
+    <t>Modalidad por confirmar</t>
+  </si>
+  <si>
+    <t>CDI: atención virtual</t>
+  </si>
+  <si>
     <t>Alertas por provincia</t>
   </si>
   <si>
-    <t>Categoría</t>
-  </si>
-  <si>
     <t>Alertas</t>
   </si>
   <si>
     <t>Guayas</t>
   </si>
   <si>
-    <t>El Oro</t>
-  </si>
-  <si>
     <t>Manabí</t>
   </si>
   <si>
@@ -99,7 +129,7 @@
     <t>Aspectos destacados</t>
   </si>
   <si>
-    <t>10 alertas con 10 códigos UA distintos: 8 Desarrollo Infantil; 2 Creciendo con Nuestros Hijos (CNH). 8 con afectación documentada y 2 por confirmar. Se excluyen los registros sin código UA; el código por sí solo no confirma una afectación.</t>
+    <t>10 alertas con 10 códigos UA distintos: 8 Desarrollo Infantil; 2 Creciendo con Nuestros Hijos (CNH). 8 con afectación documentada y 2 por confirmar. Se excluyen los registros sin código UA.</t>
   </si>
   <si>
     <t>802 kits en 4 provincias priorizadas; corte 25/10/2026.</t>
@@ -516,7 +546,7 @@
     <t>Fuentes</t>
   </si>
   <si>
-    <t>Subsecretaría Territorial (análisis de alertas); reporte ministerial de kits; ayuda memoria del bono de contingencia.</t>
+    <t>Subsecretaría Territorial (análisis de alertas); reporte ministerial de kits; ayuda memoria del bono de contingencia; base territorial de afectaciones por lluvias.</t>
   </si>
   <si>
     <t>Conteo</t>
@@ -528,7 +558,13 @@
     <t>https://geoportal.trabajo.gob.ec/ua_amenazas</t>
   </si>
   <si>
-    <t>Se muestran únicamente alertas revisadas con código UA registrado, desde el 14 de septiembre de 2026. El conteo corresponde a códigos de alerta distintos vinculados a unidades identificadas; tener código UA no confirma afectación al servicio. Los registros sin código quedan fuera de este alcance. La fecha corresponde al registro y una alerta no equivale necesariamente a un evento único. El campo Afectados mezcla personas, familias y usuarios; no se suma como personas únicas. La base no certifica atribución causal a ENOS.</t>
+    <t>Continuidad de atención</t>
+  </si>
+  <si>
+    <t>Fuente: base territorial de afectaciones por lluvias, corte 26/10/2026, 16:00. Cerradas corresponde al estado Suspendida (18 CDI y 1 CNH). Los 63 CNH con suspensión presencial y los 11 CDI en atención virtual se muestran por separado. Son cifras reportadas, sin códigos UA en esta base; no se suman a las 10 alertas ni constituyen un censo nacional de cierres.</t>
+  </si>
+  <si>
+    <t>Se muestran únicamente alertas revisadas con código UA registrado, desde el 14 de septiembre de 2026. El conteo corresponde a códigos de alerta distintos vinculados a unidades identificadas. Los registros sin código quedan fuera de este alcance. La fecha corresponde al registro y una alerta no equivale necesariamente a un evento único. El campo Afectados mezcla personas, familias y usuarios; no se suma como personas únicas. La base no certifica atribución causal a ENOS.</t>
   </si>
   <si>
     <t>Revisión de alertas</t>
@@ -546,7 +582,7 @@
     <t>Filtros</t>
   </si>
   <si>
-    <t>El territorio se aplica a todas las acciones; el servicio, solo a las alertas según la UA registrada. Kits y bono no se asocian a un servicio. La planificación del bono es nacional.</t>
+    <t>El territorio se aplica a todas las acciones; el servicio, a las alertas y al seguimiento de continuidad de atención. Kits y bono no se asocian a un servicio. La planificación del bono es nacional.</t>
   </si>
 </sst>
 </file>
@@ -963,7 +999,7 @@
                 </a:solidFill>
                 <a:latin typeface="Century Gothic"/>
               </a:rPr>
-              <a:t>Alertas por provincia</a:t>
+              <a:t>Unidades cerradas por provincia</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -979,7 +1015,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Alertas por provincia</c:v>
+            <c:v>Unidades cerradas por provincia</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill>
@@ -1010,35 +1046,29 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Resumen!$B$17:$B$19</c:f>
+              <c:f>Resumen!$B$21:$B$22</c:f>
               <c:strCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>Guayas</c:v>
+                  <c:v>El Oro</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>El Oro</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Manabí</c:v>
+                  <c:v>Santa Elena</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Resumen!$C$17:$C$19</c:f>
+              <c:f>Resumen!$C$21:$C$22</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>6</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1179,7 +1209,7 @@
                 </a:solidFill>
                 <a:latin typeface="Century Gothic"/>
               </a:rPr>
-              <a:t>Alertas por servicio</a:t>
+              <a:t>Estado de atención reportado</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1195,7 +1225,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Alertas por servicio</c:v>
+            <c:v>Estado de atención reportado</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill>
@@ -1226,29 +1256,41 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Resumen!$B$37:$B$38</c:f>
+              <c:f>Resumen!$B$40:$B$43</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>Desarrollo Infantil</c:v>
+                  <c:v>CNH: suspensión presencial</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Creciendo con Nuestros Hijos (CNH)</c:v>
+                  <c:v>Cerradas / suspendidas</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Modalidad por confirmar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>CDI: atención virtual</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Resumen!$C$37:$C$38</c:f>
+              <c:f>Resumen!$C$40:$C$43</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>8</c:v>
+                  <c:v>63</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2</c:v>
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>11</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1375,6 +1417,432 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
+              <a:defRPr sz="1100" b="1" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="2B164F"/>
+                </a:solidFill>
+                <a:latin typeface="Century Gothic"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="2B164F"/>
+                </a:solidFill>
+                <a:latin typeface="Century Gothic"/>
+              </a:rPr>
+              <a:t>Alertas por provincia</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Alertas por provincia</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="512F8D"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="20202B"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showVal val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Resumen!$B$61:$B$63</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Guayas</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>El Oro</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Manabí</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Resumen!$C$61:$C$63</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="55"/>
+        <c:axId val="50030001"/>
+        <c:axId val="50030002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50030001"/>
+        <c:scaling>
+          <c:orientation val="maxMin"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="D8D0F4"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="20202B"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50030002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50030002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:axPos val="t"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525">
+              <a:solidFill>
+                <a:srgbClr val="EEEAF4"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:tickLblPos val="none"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="6E6880"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50030001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:solidFill>
+        <a:srgbClr val="E7E2EF"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1100" b="1" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="2B164F"/>
+                </a:solidFill>
+                <a:latin typeface="Century Gothic"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="2B164F"/>
+                </a:solidFill>
+                <a:latin typeface="Century Gothic"/>
+              </a:rPr>
+              <a:t>Alertas por servicio</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Alertas por servicio</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="512F8D"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="20202B"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showVal val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Resumen!$B$81:$B$82</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Desarrollo Infantil</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Creciendo con Nuestros Hijos (CNH)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Resumen!$C$81:$C$82</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="55"/>
+        <c:axId val="50040001"/>
+        <c:axId val="50040002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50040001"/>
+        <c:scaling>
+          <c:orientation val="maxMin"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="D8D0F4"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="20202B"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50040002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50040002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:axPos val="t"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525">
+              <a:solidFill>
+                <a:srgbClr val="EEEAF4"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:tickLblPos val="none"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="6E6880"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50040001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:solidFill>
+        <a:srgbClr val="E7E2EF"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
               <a:defRPr/>
             </a:pPr>
             <a:r>
@@ -1975,24 +2443,24 @@
           </c:val>
         </c:ser>
         <c:marker val="1"/>
-        <c:axId val="50030001"/>
-        <c:axId val="50030002"/>
+        <c:axId val="50050001"/>
+        <c:axId val="50050002"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="50030001"/>
+        <c:axId val="50050001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50030002"/>
+        <c:crossAx val="50050002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50030002"/>
+        <c:axId val="50050002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2000,7 +2468,7 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50030001"/>
+        <c:crossAx val="50050001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2063,13 +2531,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>53</xdr:row>
+      <xdr:row>97</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>67</xdr:row>
+      <xdr:row>111</xdr:row>
       <xdr:rowOff>83344</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2087,7 +2555,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="209550" y="12220575"/>
+          <a:off x="209550" y="22183725"/>
           <a:ext cx="4000500" cy="2750344"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2101,13 +2569,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>72</xdr:row>
+      <xdr:row>116</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>86</xdr:row>
+      <xdr:row>130</xdr:row>
       <xdr:rowOff>83344</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2125,7 +2593,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="209550" y="15992475"/>
+          <a:off x="209550" y="25955625"/>
           <a:ext cx="4000500" cy="2750344"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2139,13 +2607,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>91</xdr:row>
+      <xdr:row>135</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>91</xdr:row>
+      <xdr:row>135</xdr:row>
       <xdr:rowOff>342900</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2163,7 +2631,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="495300" y="19859625"/>
+          <a:off x="495300" y="29822775"/>
           <a:ext cx="247650" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2177,13 +2645,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>93</xdr:row>
+      <xdr:row>137</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>93</xdr:row>
+      <xdr:row>137</xdr:row>
       <xdr:rowOff>342900</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2201,7 +2669,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="495300" y="20364450"/>
+          <a:off x="495300" y="30327600"/>
           <a:ext cx="247650" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2215,13 +2683,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>95</xdr:row>
+      <xdr:row>139</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>95</xdr:row>
+      <xdr:row>139</xdr:row>
       <xdr:rowOff>342900</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2239,7 +2707,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="495300" y="20869275"/>
+          <a:off x="495300" y="30832425"/>
           <a:ext cx="247650" cy="247650"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2253,13 +2721,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>657225</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2283,13 +2751,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>657225</xdr:colOff>
-      <xdr:row>49</xdr:row>
+      <xdr:row>54</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2304,6 +2772,66 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>657225</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="10" name="Chart 9"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>657225</xdr:colOff>
+      <xdr:row>93</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="11" name="Chart 10"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2846,7 +3374,7 @@
     <tabColor rgb="FF512F8D"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N97"/>
+  <dimension ref="A1:N141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.140625" customWidth="1"/>
@@ -3038,195 +3566,353 @@
       <c r="L12" s="16"/>
       <c r="M12" s="16"/>
     </row>
-    <row r="15" spans="1:14" ht="27" customHeight="1">
-      <c r="B15" s="6" t="s">
+    <row r="14" spans="1:14" ht="24" customHeight="1">
+      <c r="B14" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="7"/>
-    </row>
-    <row r="16" spans="1:14" ht="36" customHeight="1">
-      <c r="B16" s="17" t="s">
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+    </row>
+    <row r="15" spans="1:14" ht="21" customHeight="1">
+      <c r="B15" s="13">
+        <v>19</v>
+      </c>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="14"/>
+      <c r="L15" s="14"/>
+      <c r="M15" s="14"/>
+    </row>
+    <row r="16" spans="1:14" ht="21" customHeight="1">
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
+      <c r="M16" s="14"/>
+    </row>
+    <row r="17" spans="2:13" ht="30" customHeight="1">
+      <c r="B17" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="16"/>
+    </row>
+    <row r="19" spans="2:13" ht="27" customHeight="1">
+      <c r="B19" s="6" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="2:3" ht="19" customHeight="1">
-      <c r="B17" s="19" t="s">
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
+    </row>
+    <row r="20" spans="2:13" ht="36" customHeight="1">
+      <c r="B20" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="20">
+      <c r="C20" s="18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" ht="19" customHeight="1">
+      <c r="B21" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="20">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" ht="19" customHeight="1">
+      <c r="B22" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="22">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" spans="2:13" ht="27" customHeight="1">
+      <c r="B38" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="7"/>
+      <c r="J38" s="7"/>
+      <c r="K38" s="7"/>
+      <c r="L38" s="7"/>
+      <c r="M38" s="7"/>
+    </row>
+    <row r="39" spans="2:13" ht="36" customHeight="1">
+      <c r="B39" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C39" s="18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="2:13" ht="19" customHeight="1">
+      <c r="B40" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C40" s="20">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="41" spans="2:13" ht="19" customHeight="1">
+      <c r="B41" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="C41" s="22">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="42" spans="2:13" ht="19" customHeight="1">
+      <c r="B42" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="C42" s="20">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="43" spans="2:13" ht="19" customHeight="1">
+      <c r="B43" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C43" s="22">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="59" spans="2:13" ht="27" customHeight="1">
+      <c r="B59" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C59" s="7"/>
+      <c r="D59" s="7"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="7"/>
+      <c r="G59" s="7"/>
+      <c r="H59" s="7"/>
+      <c r="I59" s="7"/>
+      <c r="J59" s="7"/>
+      <c r="K59" s="7"/>
+      <c r="L59" s="7"/>
+      <c r="M59" s="7"/>
+    </row>
+    <row r="60" spans="2:13" ht="36" customHeight="1">
+      <c r="B60" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C60" s="18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="61" spans="2:13" ht="19" customHeight="1">
+      <c r="B61" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C61" s="20">
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="19" customHeight="1">
-      <c r="B18" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18" s="22">
+    <row r="62" spans="2:13" ht="19" customHeight="1">
+      <c r="B62" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="C62" s="22">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="19" customHeight="1">
-      <c r="B19" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="C19" s="20">
+    <row r="63" spans="2:13" ht="19" customHeight="1">
+      <c r="B63" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C63" s="20">
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="2:13" ht="27" customHeight="1">
-      <c r="B35" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="7"/>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
-      <c r="H35" s="7"/>
-      <c r="I35" s="7"/>
-      <c r="J35" s="7"/>
-      <c r="K35" s="7"/>
-      <c r="L35" s="7"/>
-      <c r="M35" s="7"/>
-    </row>
-    <row r="36" spans="2:13" ht="36" customHeight="1">
-      <c r="B36" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="C36" s="18" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="37" spans="2:13" ht="19" customHeight="1">
-      <c r="B37" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="C37" s="20">
+    <row r="79" spans="2:13" ht="27" customHeight="1">
+      <c r="B79" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C79" s="7"/>
+      <c r="D79" s="7"/>
+      <c r="E79" s="7"/>
+      <c r="F79" s="7"/>
+      <c r="G79" s="7"/>
+      <c r="H79" s="7"/>
+      <c r="I79" s="7"/>
+      <c r="J79" s="7"/>
+      <c r="K79" s="7"/>
+      <c r="L79" s="7"/>
+      <c r="M79" s="7"/>
+    </row>
+    <row r="80" spans="2:13" ht="36" customHeight="1">
+      <c r="B80" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C80" s="18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="81" spans="2:3" ht="19" customHeight="1">
+      <c r="B81" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="C81" s="20">
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="2:13" ht="19" customHeight="1">
-      <c r="B38" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="C38" s="22">
+    <row r="82" spans="2:3" ht="19" customHeight="1">
+      <c r="B82" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="C82" s="22">
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="2:13" ht="27" customHeight="1">
-      <c r="B53" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C53" s="7"/>
-      <c r="D53" s="7"/>
-      <c r="E53" s="7"/>
-      <c r="F53" s="7"/>
-      <c r="G53" s="7"/>
-      <c r="H53" s="7"/>
-      <c r="I53" s="7"/>
-      <c r="J53" s="7"/>
-      <c r="K53" s="7"/>
-      <c r="L53" s="7"/>
-      <c r="M53" s="7"/>
-    </row>
-    <row r="72" spans="2:13" ht="27" customHeight="1">
-      <c r="B72" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C72" s="7"/>
-      <c r="D72" s="7"/>
-      <c r="E72" s="7"/>
-      <c r="F72" s="7"/>
-      <c r="G72" s="7"/>
-      <c r="H72" s="7"/>
-      <c r="I72" s="7"/>
-      <c r="J72" s="7"/>
-      <c r="K72" s="7"/>
-      <c r="L72" s="7"/>
-      <c r="M72" s="7"/>
-    </row>
-    <row r="91" spans="2:13" ht="27" customHeight="1">
-      <c r="B91" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C91" s="7"/>
-      <c r="D91" s="7"/>
-      <c r="E91" s="7"/>
-      <c r="F91" s="7"/>
-      <c r="G91" s="7"/>
-      <c r="H91" s="7"/>
-      <c r="I91" s="7"/>
-      <c r="J91" s="7"/>
-      <c r="K91" s="7"/>
-      <c r="L91" s="7"/>
-      <c r="M91" s="7"/>
-    </row>
-    <row r="92" spans="2:13" ht="34" customHeight="1">
-      <c r="B92" s="23"/>
-      <c r="C92" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="D92" s="24"/>
-      <c r="E92" s="24"/>
-      <c r="F92" s="24"/>
-      <c r="G92" s="24"/>
-      <c r="H92" s="24"/>
-      <c r="I92" s="24"/>
-      <c r="J92" s="24"/>
-      <c r="K92" s="24"/>
-      <c r="L92" s="24"/>
-      <c r="M92" s="24"/>
-    </row>
-    <row r="93" spans="2:13" ht="6" customHeight="1"/>
-    <row r="94" spans="2:13" ht="34" customHeight="1">
-      <c r="B94" s="23"/>
-      <c r="C94" s="24" t="s">
+    <row r="97" spans="2:13" ht="27" customHeight="1">
+      <c r="B97" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D94" s="24"/>
-      <c r="E94" s="24"/>
-      <c r="F94" s="24"/>
-      <c r="G94" s="24"/>
-      <c r="H94" s="24"/>
-      <c r="I94" s="24"/>
-      <c r="J94" s="24"/>
-      <c r="K94" s="24"/>
-      <c r="L94" s="24"/>
-      <c r="M94" s="24"/>
-    </row>
-    <row r="95" spans="2:13" ht="6" customHeight="1"/>
-    <row r="96" spans="2:13" ht="34" customHeight="1">
-      <c r="B96" s="23"/>
-      <c r="C96" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="D96" s="24"/>
-      <c r="E96" s="24"/>
-      <c r="F96" s="24"/>
-      <c r="G96" s="24"/>
-      <c r="H96" s="24"/>
-      <c r="I96" s="24"/>
-      <c r="J96" s="24"/>
-      <c r="K96" s="24"/>
-      <c r="L96" s="24"/>
-      <c r="M96" s="24"/>
-    </row>
-    <row r="97" ht="6" customHeight="1"/>
+      <c r="C97" s="7"/>
+      <c r="D97" s="7"/>
+      <c r="E97" s="7"/>
+      <c r="F97" s="7"/>
+      <c r="G97" s="7"/>
+      <c r="H97" s="7"/>
+      <c r="I97" s="7"/>
+      <c r="J97" s="7"/>
+      <c r="K97" s="7"/>
+      <c r="L97" s="7"/>
+      <c r="M97" s="7"/>
+    </row>
+    <row r="116" spans="2:13" ht="27" customHeight="1">
+      <c r="B116" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C116" s="7"/>
+      <c r="D116" s="7"/>
+      <c r="E116" s="7"/>
+      <c r="F116" s="7"/>
+      <c r="G116" s="7"/>
+      <c r="H116" s="7"/>
+      <c r="I116" s="7"/>
+      <c r="J116" s="7"/>
+      <c r="K116" s="7"/>
+      <c r="L116" s="7"/>
+      <c r="M116" s="7"/>
+    </row>
+    <row r="135" spans="2:13" ht="27" customHeight="1">
+      <c r="B135" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C135" s="7"/>
+      <c r="D135" s="7"/>
+      <c r="E135" s="7"/>
+      <c r="F135" s="7"/>
+      <c r="G135" s="7"/>
+      <c r="H135" s="7"/>
+      <c r="I135" s="7"/>
+      <c r="J135" s="7"/>
+      <c r="K135" s="7"/>
+      <c r="L135" s="7"/>
+      <c r="M135" s="7"/>
+    </row>
+    <row r="136" spans="2:13" ht="34" customHeight="1">
+      <c r="B136" s="23"/>
+      <c r="C136" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D136" s="24"/>
+      <c r="E136" s="24"/>
+      <c r="F136" s="24"/>
+      <c r="G136" s="24"/>
+      <c r="H136" s="24"/>
+      <c r="I136" s="24"/>
+      <c r="J136" s="24"/>
+      <c r="K136" s="24"/>
+      <c r="L136" s="24"/>
+      <c r="M136" s="24"/>
+    </row>
+    <row r="137" spans="2:13" ht="6" customHeight="1"/>
+    <row r="138" spans="2:13" ht="34" customHeight="1">
+      <c r="B138" s="23"/>
+      <c r="C138" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="D138" s="24"/>
+      <c r="E138" s="24"/>
+      <c r="F138" s="24"/>
+      <c r="G138" s="24"/>
+      <c r="H138" s="24"/>
+      <c r="I138" s="24"/>
+      <c r="J138" s="24"/>
+      <c r="K138" s="24"/>
+      <c r="L138" s="24"/>
+      <c r="M138" s="24"/>
+    </row>
+    <row r="139" spans="2:13" ht="6" customHeight="1"/>
+    <row r="140" spans="2:13" ht="34" customHeight="1">
+      <c r="B140" s="23"/>
+      <c r="C140" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="D140" s="24"/>
+      <c r="E140" s="24"/>
+      <c r="F140" s="24"/>
+      <c r="G140" s="24"/>
+      <c r="H140" s="24"/>
+      <c r="I140" s="24"/>
+      <c r="J140" s="24"/>
+      <c r="K140" s="24"/>
+      <c r="L140" s="24"/>
+      <c r="M140" s="24"/>
+    </row>
+    <row r="141" spans="2:13" ht="6" customHeight="1"/>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="18">
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="B10:D11"/>
     <mergeCell ref="B12:D12"/>
@@ -3239,9 +3925,12 @@
     <mergeCell ref="K9:M9"/>
     <mergeCell ref="K10:M11"/>
     <mergeCell ref="K12:M12"/>
-    <mergeCell ref="C92:M92"/>
-    <mergeCell ref="C94:M94"/>
-    <mergeCell ref="C96:M96"/>
+    <mergeCell ref="B14:M14"/>
+    <mergeCell ref="B15:M16"/>
+    <mergeCell ref="B17:M17"/>
+    <mergeCell ref="C136:M136"/>
+    <mergeCell ref="C138:M138"/>
+    <mergeCell ref="C140:M140"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.55" header="0.3" footer="0.3"/>
@@ -3279,7 +3968,7 @@
     <row r="2" spans="1:5" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -3312,25 +4001,25 @@
     </row>
     <row r="6" spans="1:5" ht="27" customHeight="1">
       <c r="B6" s="6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
     </row>
     <row r="7" spans="1:5" ht="36" customHeight="1">
       <c r="B7" s="17" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="19" customHeight="1">
       <c r="B8" s="19" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="C8" s="20">
         <v>0</v>
@@ -3341,7 +4030,7 @@
     </row>
     <row r="9" spans="1:5" ht="19" customHeight="1">
       <c r="B9" s="21" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="C9" s="22">
         <v>0</v>
@@ -3352,7 +4041,7 @@
     </row>
     <row r="10" spans="1:5" ht="19" customHeight="1">
       <c r="B10" s="19" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="C10" s="20">
         <v>0</v>
@@ -3363,7 +4052,7 @@
     </row>
     <row r="11" spans="1:5" ht="19" customHeight="1">
       <c r="B11" s="21" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C11" s="22">
         <v>0</v>
@@ -3374,7 +4063,7 @@
     </row>
     <row r="12" spans="1:5" ht="19" customHeight="1">
       <c r="B12" s="19" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="C12" s="20">
         <v>0</v>
@@ -3385,7 +4074,7 @@
     </row>
     <row r="13" spans="1:5" ht="19" customHeight="1">
       <c r="B13" s="21" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C13" s="22">
         <v>0</v>
@@ -3396,7 +4085,7 @@
     </row>
     <row r="14" spans="1:5" ht="19" customHeight="1">
       <c r="B14" s="19" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="C14" s="20">
         <v>0</v>
@@ -3407,7 +4096,7 @@
     </row>
     <row r="15" spans="1:5" ht="19" customHeight="1">
       <c r="B15" s="21" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="C15" s="22">
         <v>0</v>
@@ -3418,7 +4107,7 @@
     </row>
     <row r="16" spans="1:5" ht="19" customHeight="1">
       <c r="B16" s="19" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C16" s="20">
         <v>0</v>
@@ -3429,7 +4118,7 @@
     </row>
     <row r="17" spans="2:4" ht="19" customHeight="1">
       <c r="B17" s="21" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C17" s="22">
         <v>0</v>
@@ -3440,7 +4129,7 @@
     </row>
     <row r="18" spans="2:4" ht="19" customHeight="1">
       <c r="B18" s="19" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C18" s="20">
         <v>0</v>
@@ -3451,7 +4140,7 @@
     </row>
     <row r="19" spans="2:4" ht="19" customHeight="1">
       <c r="B19" s="21" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C19" s="22">
         <v>0</v>
@@ -3462,7 +4151,7 @@
     </row>
     <row r="20" spans="2:4" ht="19" customHeight="1">
       <c r="B20" s="19" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="C20" s="20">
         <v>0</v>
@@ -3473,7 +4162,7 @@
     </row>
     <row r="21" spans="2:4" ht="19" customHeight="1">
       <c r="B21" s="21" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C21" s="22">
         <v>0</v>
@@ -3484,7 +4173,7 @@
     </row>
     <row r="22" spans="2:4" ht="19" customHeight="1">
       <c r="B22" s="19" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C22" s="20">
         <v>0</v>
@@ -3495,7 +4184,7 @@
     </row>
     <row r="23" spans="2:4" ht="19" customHeight="1">
       <c r="B23" s="21" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C23" s="22">
         <v>0</v>
@@ -3506,7 +4195,7 @@
     </row>
     <row r="24" spans="2:4" ht="19" customHeight="1">
       <c r="B24" s="19" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="C24" s="20">
         <v>0</v>
@@ -3517,7 +4206,7 @@
     </row>
     <row r="25" spans="2:4" ht="19" customHeight="1">
       <c r="B25" s="21" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="C25" s="22">
         <v>0</v>
@@ -3528,7 +4217,7 @@
     </row>
     <row r="26" spans="2:4" ht="19" customHeight="1">
       <c r="B26" s="19" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C26" s="20">
         <v>0</v>
@@ -3539,7 +4228,7 @@
     </row>
     <row r="27" spans="2:4" ht="19" customHeight="1">
       <c r="B27" s="21" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="C27" s="22">
         <v>0</v>
@@ -3550,7 +4239,7 @@
     </row>
     <row r="28" spans="2:4" ht="19" customHeight="1">
       <c r="B28" s="19" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C28" s="20">
         <v>0</v>
@@ -3561,7 +4250,7 @@
     </row>
     <row r="29" spans="2:4" ht="19" customHeight="1">
       <c r="B29" s="21" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="C29" s="22">
         <v>0</v>
@@ -3572,7 +4261,7 @@
     </row>
     <row r="30" spans="2:4" ht="19" customHeight="1">
       <c r="B30" s="19" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="C30" s="20">
         <v>0</v>
@@ -3583,7 +4272,7 @@
     </row>
     <row r="31" spans="2:4" ht="19" customHeight="1">
       <c r="B31" s="21" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C31" s="22">
         <v>0</v>
@@ -3594,7 +4283,7 @@
     </row>
     <row r="32" spans="2:4" ht="19" customHeight="1">
       <c r="B32" s="19" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="C32" s="20">
         <v>0</v>
@@ -3605,7 +4294,7 @@
     </row>
     <row r="33" spans="2:4" ht="19" customHeight="1">
       <c r="B33" s="21" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="C33" s="22">
         <v>0</v>
@@ -3616,7 +4305,7 @@
     </row>
     <row r="34" spans="2:4" ht="19" customHeight="1">
       <c r="B34" s="19" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="C34" s="20">
         <v>0</v>
@@ -3627,7 +4316,7 @@
     </row>
     <row r="35" spans="2:4" ht="19" customHeight="1">
       <c r="B35" s="21" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="C35" s="22">
         <v>0</v>
@@ -3638,7 +4327,7 @@
     </row>
     <row r="36" spans="2:4" ht="19" customHeight="1">
       <c r="B36" s="19" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="C36" s="20">
         <v>0</v>
@@ -3649,7 +4338,7 @@
     </row>
     <row r="37" spans="2:4" ht="19" customHeight="1">
       <c r="B37" s="21" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="C37" s="22">
         <v>0</v>
@@ -3660,7 +4349,7 @@
     </row>
     <row r="38" spans="2:4" ht="19" customHeight="1">
       <c r="B38" s="19" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="C38" s="20">
         <v>0</v>
@@ -3671,7 +4360,7 @@
     </row>
     <row r="39" spans="2:4" ht="19" customHeight="1">
       <c r="B39" s="21" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="C39" s="22">
         <v>0</v>
@@ -3682,7 +4371,7 @@
     </row>
     <row r="40" spans="2:4" ht="19" customHeight="1">
       <c r="B40" s="19" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="C40" s="20">
         <v>2</v>
@@ -3693,7 +4382,7 @@
     </row>
     <row r="41" spans="2:4" ht="19" customHeight="1">
       <c r="B41" s="21" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="C41" s="22">
         <v>0</v>
@@ -3704,7 +4393,7 @@
     </row>
     <row r="42" spans="2:4" ht="19" customHeight="1">
       <c r="B42" s="19" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="C42" s="20">
         <v>0</v>
@@ -3715,7 +4404,7 @@
     </row>
     <row r="43" spans="2:4" ht="19" customHeight="1">
       <c r="B43" s="21" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="C43" s="22">
         <v>2</v>
@@ -3726,7 +4415,7 @@
     </row>
     <row r="44" spans="2:4" ht="19" customHeight="1">
       <c r="B44" s="19" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C44" s="20">
         <v>6</v>
@@ -3737,7 +4426,7 @@
     </row>
     <row r="45" spans="2:4" ht="19" customHeight="1">
       <c r="B45" s="21" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="C45" s="22">
         <v>0</v>
@@ -3748,7 +4437,7 @@
     </row>
     <row r="46" spans="2:4" ht="19" customHeight="1">
       <c r="B46" s="19" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="C46" s="20">
         <v>0</v>
@@ -3759,7 +4448,7 @@
     </row>
     <row r="47" spans="2:4" ht="19" customHeight="1">
       <c r="B47" s="21" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C47" s="22">
         <v>0</v>
@@ -3770,7 +4459,7 @@
     </row>
     <row r="48" spans="2:4" ht="19" customHeight="1">
       <c r="B48" s="19" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="C48" s="20">
         <v>0</v>
@@ -3781,7 +4470,7 @@
     </row>
     <row r="49" spans="2:4" ht="19" customHeight="1">
       <c r="B49" s="21" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="C49" s="22">
         <v>0</v>
@@ -3792,7 +4481,7 @@
     </row>
     <row r="50" spans="2:4" ht="19" customHeight="1">
       <c r="B50" s="19" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="C50" s="20">
         <v>0</v>
@@ -3914,7 +4603,7 @@
     </row>
     <row r="6" spans="1:12" ht="27" customHeight="1">
       <c r="B6" s="6" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -3925,359 +4614,359 @@
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
       <c r="K6" s="8" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="36" customHeight="1">
       <c r="B7" s="17" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G7" s="25" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H7" s="25" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="I7" s="25" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="J7" s="25" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="K7" s="25" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="48" customHeight="1">
       <c r="B8" s="19" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="G8" s="26" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="H8" s="26" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I8" s="26" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="J8" s="26" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="K8" s="26" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="48" customHeight="1">
       <c r="B9" s="21" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="F9" s="27" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="G9" s="27" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="H9" s="27" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I9" s="27" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="J9" s="27" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="K9" s="27" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="48" customHeight="1">
       <c r="B10" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="C10" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="D10" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="26" t="s">
-        <v>87</v>
-      </c>
       <c r="F10" s="26" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="G10" s="26" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="H10" s="26" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I10" s="26" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="J10" s="26" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="K10" s="26" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="48" customHeight="1">
       <c r="B11" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="D11" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="F11" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="G11" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="H11" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="I11" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="J11" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="C11" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="D11" s="27" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" s="27" t="s">
-        <v>87</v>
-      </c>
-      <c r="F11" s="27" t="s">
+      <c r="K11" s="27" t="s">
         <v>102</v>
-      </c>
-      <c r="G11" s="27" t="s">
-        <v>103</v>
-      </c>
-      <c r="H11" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="I11" s="27" t="s">
-        <v>104</v>
-      </c>
-      <c r="J11" s="27" t="s">
-        <v>91</v>
-      </c>
-      <c r="K11" s="27" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="48" customHeight="1">
       <c r="B12" s="19" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E12" s="26" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="F12" s="26" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="G12" s="26" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="H12" s="26" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I12" s="26" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="J12" s="26" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="K12" s="26" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="48" customHeight="1">
       <c r="B13" s="21" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E13" s="27" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="F13" s="27" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="G13" s="27" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="H13" s="27" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I13" s="27" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="J13" s="27" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="K13" s="27" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="48" customHeight="1">
       <c r="B14" s="19" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="D14" s="26" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="F14" s="26" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="G14" s="26" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="H14" s="26" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I14" s="26" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="J14" s="26" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="K14" s="26" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="48" customHeight="1">
       <c r="B15" s="21" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="F15" s="27" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="G15" s="27" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="H15" s="27" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I15" s="27" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="J15" s="27" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="K15" s="27" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="48" customHeight="1">
       <c r="B16" s="19" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="D16" s="26" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E16" s="26" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="G16" s="26" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="H16" s="26" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="I16" s="26" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="J16" s="26" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="K16" s="26" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="17" spans="2:11" ht="48" customHeight="1">
       <c r="B17" s="21" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="F17" s="27" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="G17" s="27" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="H17" s="27" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="I17" s="27" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="J17" s="27" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="K17" s="27" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -4327,7 +5016,7 @@
     <row r="2" spans="1:9" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4376,7 +5065,7 @@
     </row>
     <row r="6" spans="1:9" ht="27" customHeight="1">
       <c r="B6" s="6" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -4387,33 +5076,33 @@
     </row>
     <row r="7" spans="1:9" ht="36" customHeight="1">
       <c r="B7" s="17" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="19" customHeight="1">
       <c r="B8" s="19" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="D8" s="20">
         <v>197</v>
@@ -4433,10 +5122,10 @@
     </row>
     <row r="9" spans="1:9" ht="19" customHeight="1">
       <c r="B9" s="21" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="D9" s="22">
         <v>0</v>
@@ -4456,10 +5145,10 @@
     </row>
     <row r="10" spans="1:9" ht="19" customHeight="1">
       <c r="B10" s="19" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="D10" s="20">
         <v>150</v>
@@ -4479,10 +5168,10 @@
     </row>
     <row r="11" spans="1:9" ht="19" customHeight="1">
       <c r="B11" s="21" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="D11" s="22">
         <v>400</v>
@@ -4502,7 +5191,7 @@
     </row>
     <row r="12" spans="1:9" ht="19" customHeight="1">
       <c r="B12" s="19" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="C12" s="26"/>
       <c r="D12" s="20">
@@ -4523,7 +5212,7 @@
     </row>
     <row r="13" spans="1:9" ht="19" customHeight="1">
       <c r="B13" s="21" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="C13" s="27"/>
       <c r="D13" s="22">
@@ -4544,10 +5233,10 @@
     </row>
     <row r="14" spans="1:9" ht="19" customHeight="1">
       <c r="B14" s="19" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="D14" s="20">
         <v>55</v>
@@ -4567,7 +5256,7 @@
     </row>
     <row r="15" spans="1:9" ht="22" customHeight="1">
       <c r="B15" s="30" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="C15" s="31"/>
       <c r="D15" s="32">
@@ -4630,7 +5319,7 @@
     <row r="2" spans="1:6" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4667,37 +5356,37 @@
     </row>
     <row r="6" spans="1:6" ht="27" customHeight="1">
       <c r="B6" s="6" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="8" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="36" customHeight="1">
       <c r="B7" s="17" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="19" customHeight="1">
       <c r="B8" s="19" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="E8" s="20">
         <v>150</v>
@@ -4705,13 +5394,13 @@
     </row>
     <row r="9" spans="1:6" ht="19" customHeight="1">
       <c r="B9" s="21" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="E9" s="22">
         <v>100</v>
@@ -4719,13 +5408,13 @@
     </row>
     <row r="10" spans="1:6" ht="19" customHeight="1">
       <c r="B10" s="19" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="E10" s="20">
         <v>100</v>
@@ -4733,13 +5422,13 @@
     </row>
     <row r="11" spans="1:6" ht="19" customHeight="1">
       <c r="B11" s="21" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="E11" s="22">
         <v>97</v>
@@ -4747,13 +5436,13 @@
     </row>
     <row r="12" spans="1:6" ht="19" customHeight="1">
       <c r="B12" s="19" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="E12" s="20">
         <v>30</v>
@@ -4761,13 +5450,13 @@
     </row>
     <row r="13" spans="1:6" ht="19" customHeight="1">
       <c r="B13" s="21" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="E13" s="22">
         <v>25</v>
@@ -4775,13 +5464,13 @@
     </row>
     <row r="14" spans="1:6" ht="19" customHeight="1">
       <c r="B14" s="19" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="D14" s="26" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="E14" s="20">
         <v>300</v>
@@ -4789,7 +5478,7 @@
     </row>
     <row r="15" spans="1:6" ht="22" customHeight="1">
       <c r="B15" s="30" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="C15" s="31"/>
       <c r="D15" s="31"/>
@@ -4800,23 +5489,23 @@
     </row>
     <row r="18" spans="2:5" ht="27" customHeight="1">
       <c r="B18" s="6" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
       <c r="E18" s="8" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="36" customHeight="1">
       <c r="B19" s="34" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="19" customHeight="1">
@@ -4848,7 +5537,7 @@
     <tabColor rgb="FF5A5765"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.140625" customWidth="1"/>
@@ -4866,7 +5555,7 @@
     <row r="2" spans="1:4" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4895,7 +5584,7 @@
     </row>
     <row r="6" spans="1:4" ht="32" customHeight="1">
       <c r="B6" s="36" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="C6" s="37" t="s">
         <v>4</v>
@@ -4903,82 +5592,90 @@
     </row>
     <row r="7" spans="1:4" ht="32" customHeight="1">
       <c r="B7" s="36" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="32" customHeight="1">
       <c r="B8" s="36" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="42" customHeight="1">
       <c r="B9" s="36" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="57" customHeight="1">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="42" customHeight="1">
       <c r="B10" s="36" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="32" customHeight="1">
       <c r="B11" s="36" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="102" customHeight="1">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="72" customHeight="1">
       <c r="B12" s="36" t="s">
-        <v>15</v>
+        <v>177</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="57" customHeight="1">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="87" customHeight="1">
       <c r="B13" s="36" t="s">
-        <v>168</v>
+        <v>26</v>
       </c>
       <c r="C13" s="37" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="42" customHeight="1">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="57" customHeight="1">
       <c r="B14" s="36" t="s">
-        <v>133</v>
+        <v>180</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="72" customHeight="1">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="42" customHeight="1">
       <c r="B15" s="36" t="s">
-        <v>170</v>
+        <v>143</v>
       </c>
       <c r="C15" s="37" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="42" customHeight="1">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="72" customHeight="1">
       <c r="B16" s="36" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="C16" s="37" t="s">
-        <v>173</v>
+        <v>183</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" ht="57" customHeight="1">
+      <c r="B17" s="36" t="s">
+        <v>184</v>
+      </c>
+      <c r="C17" s="37" t="s">
+        <v>185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Confirmar 13.390 kits oficiales, etiquetar núcleos familiares y actualizar fecha con montos verificados
</commit_message>
<xml_diff>
--- a/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
+++ b/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
@@ -56,7 +56,7 @@
     <t>20 provincias priorizadas · corte 26/10, 22:26</t>
   </si>
   <si>
-    <t>Núcleos con bono gestionado</t>
+    <t>Núcleos familiares con bono gestionado</t>
   </si>
   <si>
     <t>Por inundaciones · gestión del bono</t>
@@ -131,7 +131,7 @@
     <t>13390 kits en 20 provincias priorizadas; corte 26/10/2026.</t>
   </si>
   <si>
-    <t>113 núcleos con bono gestionado: USD 33.200,80.</t>
+    <t>113 núcleos familiares con bono gestionado: USD 33.200,80.</t>
   </si>
   <si>
     <t>Evolución de las alertas</t>
@@ -455,7 +455,7 @@
     <t>Kits</t>
   </si>
   <si>
-    <t>Bono gestionado (núcleos)</t>
+    <t>Bono gestionado (núcleos familiares)</t>
   </si>
   <si>
     <t>Monto gestionado (USD)</t>
@@ -584,13 +584,13 @@
     <t>Kits entregados en provincias priorizadas</t>
   </si>
   <si>
-    <t>Kits en provincias priorizadas: Kobo, corte 26/10/2026, 22:26:42. Entregas del 31/08 al 26/10; incluye fechas anteriores al inicio de las alertas. Reemplaza el corte anterior. Familias reportadas es una suma por entrega, no familias únicas. Datos declarados, pendientes de validación territorial.</t>
+    <t>Kits en provincias priorizadas: Kobo, corte 26/10/2026, 22:26:42. Entregas del 31/08 al 26/10; incluye fechas anteriores al inicio de las alertas. Reemplaza el corte anterior. Núcleos familiares reportados: suma por entrega, no núcleos únicos. El total de kits de este corte fue confirmado oficialmente.</t>
   </si>
   <si>
     <t>Período</t>
   </si>
   <si>
-    <t>Familias reportadas</t>
+    <t>Núcleos familiares reportados</t>
   </si>
   <si>
     <t>ID Kobo</t>

</xml_diff>

<commit_message>
Retirar notas internas y refinar gráficos de Riesgos con cantidades y porcentajes
</commit_message>
<xml_diff>
--- a/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
+++ b/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Alertas!$B$7:$K$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Evolución!$B$7:$D$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Unidades suspendidas'!$B$7:$H$106</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">'Ficha técnica'!$A$1:$D$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'Ficha técnica'!$A$1:$D$17</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Resumen!$A$1:$N$141</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1167" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1165" uniqueCount="375">
   <si>
     <t>Riesgos · Respuesta del Ministerio</t>
   </si>
@@ -125,7 +125,7 @@
     <t>Aspectos destacados</t>
   </si>
   <si>
-    <t>10 alertas con 10 códigos UA distintos: 8 Desarrollo Infantil; 2 Creciendo con Nuestros Hijos (CNH). 8 con afectación documentada y 2 por confirmar. Se excluyen los registros sin código UA.</t>
+    <t>10 alertas con 10 códigos UA distintos: 8 Desarrollo Infantil; 2 Creciendo con Nuestros Hijos (CNH). Se excluyen los registros sin código UA.</t>
   </si>
   <si>
     <t>13390 kits en 20 provincias priorizadas; corte 26/10/2026.</t>
@@ -977,10 +977,10 @@
     <t>Detalle territorial de unidades</t>
   </si>
   <si>
-    <t>99 suspendidas · base 26/10/2026, 16:00 + confirmación operativa de Guayas</t>
-  </si>
-  <si>
-    <t>Base territorial del 26/10/2026, 16:00, actualizada con la confirmación operativa posterior de Guayas: 99 UA suspendidas (35 CDI y 64 CNH). Las 17 CDI de Guayas se incluyen como suspendidas por confirmación recibida; su estado original se conserva para trazabilidad. Los 63 CNH de El Oro no tienen nombre ni cantón en la base. No constan códigos UA ni se suma este registro a las 10 alertas.</t>
+    <t>99 suspendidas · corte 26/10/2026, 16:00</t>
+  </si>
+  <si>
+    <t>Fuente: reporte territorial de unidades con suspensión total o presencial. Corte: 26/10/2026, 16:00.</t>
   </si>
   <si>
     <t>Estado de atención</t>
@@ -1140,12 +1140,6 @@
   </si>
   <si>
     <t>Se muestran únicamente alertas revisadas con código UA registrado, desde el 14 de septiembre de 2026. El conteo corresponde a códigos de alerta distintos vinculados a unidades identificadas. Los registros sin código quedan fuera de este alcance. La fecha corresponde al registro y una alerta no equivale necesariamente a un evento único. El campo Afectados mezcla personas, familias y usuarios; no se suma como personas únicas. La base no certifica atribución causal a ENOS.</t>
-  </si>
-  <si>
-    <t>Revisión de alertas</t>
-  </si>
-  <si>
-    <t>En el corte nacional hay 10 alertas con 10 códigos UA distintos: 8 con afectación documentada y 2 por confirmar. ALT-2026-000315 y ALT-2026-000316 (Tenguel) tienen código UA, pero el relato solo describe inundación territorial; no se presentan como daños confirmados al servicio.</t>
   </si>
   <si>
     <t>Bono de contingencia</t>
@@ -10360,7 +10354,7 @@
     <tabColor rgb="FF5A5765"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.140625" customWidth="1"/>
@@ -10453,7 +10447,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="87" customHeight="1">
+    <row r="12" spans="1:4" ht="42" customHeight="1">
       <c r="B12" s="36" t="s">
         <v>369</v>
       </c>
@@ -10469,36 +10463,28 @@
         <v>370</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="57" customHeight="1">
+    <row r="14" spans="1:4" ht="72" customHeight="1">
       <c r="B14" s="36" t="s">
-        <v>371</v>
+        <v>141</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>372</v>
+        <v>185</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="72" customHeight="1">
       <c r="B15" s="36" t="s">
-        <v>141</v>
+        <v>371</v>
       </c>
       <c r="C15" s="37" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="72" customHeight="1">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="57" customHeight="1">
       <c r="B16" s="36" t="s">
         <v>373</v>
       </c>
       <c r="C16" s="37" t="s">
         <v>374</v>
-      </c>
-    </row>
-    <row r="17" spans="2:3" ht="57" customHeight="1">
-      <c r="B17" s="36" t="s">
-        <v>375</v>
-      </c>
-      <c r="C17" s="37" t="s">
-        <v>376</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Quitar subtítulos de los alcances de Riesgos y enlazar el geoportal
- PDF «Alcances y fuentes», nota de la presentación y nota metodológica del tablero: cada alcance en
  su propio párrafo, sin subtítulos, en dos columnas (una en teléfono).
- Cierre común «Más información en el geoportal de unidades de atención y amenazas», con el nombre
  del geoportal como enlace en el PDF, la diapositiva y el tablero; en el libro, la fila Geoportal de
  la ficha técnica es un vínculo. La dirección ya no se imprime suelta.
- Página 3 del PDF con más aire para los kits y los alcances; prueba nueva (126 en total).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUCWMWZ6GMzdHUXxvK5iGa
</commit_message>
<xml_diff>
--- a/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
+++ b/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
@@ -1017,7 +1017,7 @@
     <t>Geoportal</t>
   </si>
   <si>
-    <t>https://geoportal.trabajo.gob.ec/ua_amenazas</t>
+    <t>Más información en el geoportal de unidades de atención y amenazas</t>
   </si>
   <si>
     <t>Continuidad de atención</t>
@@ -1050,7 +1050,7 @@
     <numFmt numFmtId="168" formatCode="#,##0;-#,##0;&quot;—&quot;"/>
     <numFmt numFmtId="169" formatCode="#,##0.00;-#,##0.00;&quot;—&quot;"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1207,6 +1207,15 @@
     <font>
       <sz val="10"/>
       <color rgb="FF20202B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF512F8D"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1384,7 +1393,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1553,6 +1562,9 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -13831,7 +13843,7 @@
       <c r="B11" s="55" t="s">
         <v>327</v>
       </c>
-      <c r="C11" s="56" t="s">
+      <c r="C11" s="57" t="s">
         <v>328</v>
       </c>
     </row>
@@ -13876,6 +13888,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C11" r:id="rId1" tooltip="https://geoportal.trabajo.gob.ec/ua_amenazas"/>
+  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.55" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="portrait"/>
@@ -13883,6 +13898,6 @@
     <oddHeader>&amp;L&amp;"Century Gothic,Bold"&amp;9&amp;K512F8DMinisterio de Trabajo y Desarrollo Humano&amp;R&amp;"Calibri,Regular"&amp;9&amp;K5A5765Del 14/09/2026 al 26/10/2026</oddHeader>
     <oddFooter>&amp;L&amp;"Calibri,Regular"&amp;8&amp;K5A5765InfoReport · Indicadores estratégicos&amp;C&amp;"Calibri,Regular"&amp;8&amp;K5A5765Página &amp;P de &amp;N&amp;R&amp;"Calibri,Regular"&amp;8&amp;K5A5765Fuente: Ministerio de Trabajo y Desarrollo Humano</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Incorporar 11 reportes sectoriales y adaptar Riesgos al PDF aprobado
</commit_message>
<xml_diff>
--- a/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
+++ b/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Ficha técnica" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Alertas!$B$8:$K$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Alertas!$B$8:$K$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Entregas Kobo'!$B$10:$H$99</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Evolución!$B$8:$D$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Provincias!$B$8:$H$28</definedName>
@@ -31,9 +31,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="335">
-  <si>
-    <t>Riesgos · Respuesta del Ministerio</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1170" uniqueCount="366">
+  <si>
+    <t>Riesgos</t>
   </si>
   <si>
     <t>Del 14/09/2026 al 26/10/2026 · Nacional · Todos los servicios</t>
@@ -48,10 +48,10 @@
     <t>Del 14/09/2026 al 26/10/2026</t>
   </si>
   <si>
-    <t>Alertas con código UA</t>
-  </si>
-  <si>
-    <t>Registros distintos · desde 14/09/2026</t>
+    <t>Alertas reportadas</t>
+  </si>
+  <si>
+    <t>Registro y reportes sectoriales</t>
   </si>
   <si>
     <t>Kits entregados</t>
@@ -123,7 +123,7 @@
     <t>Evolución de las alertas</t>
   </si>
   <si>
-    <t>10 alertas con código UA · desde el 14/09/2026</t>
+    <t>21 alertas reportada · desde el 14/09/2026</t>
   </si>
   <si>
     <t>Aspectos destacados</t>
@@ -132,7 +132,7 @@
     <t>99 unidades de atención con atención suspendida (64 CNH · 35 CDI); El Oro concentra 75 (75,8 %).</t>
   </si>
   <si>
-    <t>10 alertas con 10 códigos UA distintos: 8 Desarrollo Infantil; 2 Creciendo con Nuestros Hijos (CNH). Se excluyen los registros sin código UA.</t>
+    <t>21 alertas reportadas: 10 con código UA y 11 reportes sectoriales.</t>
   </si>
   <si>
     <t>13.390 kits en 20 provincias priorizadas; corte 26/10/2026.</t>
@@ -288,7 +288,7 @@
     <t>Mis Primeras Enseñanzas</t>
   </si>
   <si>
-    <t>10 alertas · de la más reciente a la más antigua</t>
+    <t>21 alertas · de la más reciente a la más antigua</t>
   </si>
   <si>
     <t>Alerta</t>
@@ -309,6 +309,57 @@
     <t>Prioridad</t>
   </si>
   <si>
+    <t>DIS-2026-003</t>
+  </si>
+  <si>
+    <t>Discapacidades · AHC</t>
+  </si>
+  <si>
+    <t>Inundaciones en viviendas de usuarios; acompañamiento y monitoreo. Servicio operativo.</t>
+  </si>
+  <si>
+    <t>En seguimiento</t>
+  </si>
+  <si>
+    <t>No reportada</t>
+  </si>
+  <si>
+    <t>DIS-2026-002</t>
+  </si>
+  <si>
+    <t>Inundaciones en viviendas de usuarios; monitoreo de facilitadores. Servicio operativo.</t>
+  </si>
+  <si>
+    <t>DIS-2026-001</t>
+  </si>
+  <si>
+    <t>Machala</t>
+  </si>
+  <si>
+    <t>DIS-2026-005</t>
+  </si>
+  <si>
+    <t>Los Ríos</t>
+  </si>
+  <si>
+    <t>Babahoyo</t>
+  </si>
+  <si>
+    <t>Familia por un Buen Vivir para Personas con Discapacidad 7</t>
+  </si>
+  <si>
+    <t>Inundación de vivienda de un núcleo familiar; levantamiento de información. Servicio operativo.</t>
+  </si>
+  <si>
+    <t>DIS-2026-004</t>
+  </si>
+  <si>
+    <t>Familia por un Buen Vivir para Personas con Discapacidad 5</t>
+  </si>
+  <si>
+    <t>Colapso de vivienda de un usuario; evaluación de necesidades. Servicio operativo.</t>
+  </si>
+  <si>
     <t>ALT-2026-000325</t>
   </si>
   <si>
@@ -378,9 +429,6 @@
     <t>Ingreso de agua; cambio temporal a modalidad virtual</t>
   </si>
   <si>
-    <t>En seguimiento</t>
-  </si>
-  <si>
     <t>ALT-2026-000318</t>
   </si>
   <si>
@@ -441,6 +489,69 @@
     <t>Correo Infantil</t>
   </si>
   <si>
+    <t>GER-2026-006</t>
+  </si>
+  <si>
+    <t>Agosto 2026 (sin día)</t>
+  </si>
+  <si>
+    <t>Santo Domingo de los Tsáchilas</t>
+  </si>
+  <si>
+    <t>Santo Domingo</t>
+  </si>
+  <si>
+    <t>Centros gerontológicos</t>
+  </si>
+  <si>
+    <t>Filtraciones y humedad; mitigación inmediata. Servicio operativo.</t>
+  </si>
+  <si>
+    <t>GER-2026-005</t>
+  </si>
+  <si>
+    <t>Pedernales</t>
+  </si>
+  <si>
+    <t>Filtraciones y humedad; medidas de contingencia. Servicio operativo.</t>
+  </si>
+  <si>
+    <t>GER-2026-004</t>
+  </si>
+  <si>
+    <t>Portoviejo</t>
+  </si>
+  <si>
+    <t>Filtraciones y humedad; adecuaciones provisionales. Servicio operativo.</t>
+  </si>
+  <si>
+    <t>GER-2026-003</t>
+  </si>
+  <si>
+    <t>Filtraciones y humedad; medidas preventivas y correctivas. Servicio operativo.</t>
+  </si>
+  <si>
+    <t>GER-2026-002</t>
+  </si>
+  <si>
+    <t>Esmeraldas</t>
+  </si>
+  <si>
+    <t>San Lorenzo</t>
+  </si>
+  <si>
+    <t>Filtraciones y humedad; intervención emergente. Servicio operativo.</t>
+  </si>
+  <si>
+    <t>GER-2026-001</t>
+  </si>
+  <si>
+    <t>Huaquillas</t>
+  </si>
+  <si>
+    <t>Filtraciones en techo y daños en patio; mitigación temporal. Servicio operativo.</t>
+  </si>
+  <si>
     <t>Desde el 14/09/2026</t>
   </si>
   <si>
@@ -468,9 +579,6 @@
     <t>Registros Kobo</t>
   </si>
   <si>
-    <t>Esmeraldas</t>
-  </si>
-  <si>
     <t>Carchi</t>
   </si>
   <si>
@@ -492,9 +600,6 @@
     <t>Pichincha</t>
   </si>
   <si>
-    <t>Los Ríos</t>
-  </si>
-  <si>
     <t>Napo</t>
   </si>
   <si>
@@ -504,9 +609,6 @@
     <t>Tungurahua</t>
   </si>
   <si>
-    <t>Santo Domingo de los Tsáchilas</t>
-  </si>
-  <si>
     <t>Zamora Chinchipe</t>
   </si>
   <si>
@@ -753,9 +855,6 @@
     <t>901560279</t>
   </si>
   <si>
-    <t>Babahoyo</t>
-  </si>
-  <si>
     <t>901546105</t>
   </si>
   <si>
@@ -822,9 +921,6 @@
     <t>901584335</t>
   </si>
   <si>
-    <t>Santo Domingo</t>
-  </si>
-  <si>
     <t>901577508</t>
   </si>
   <si>
@@ -864,9 +960,6 @@
     <t>901505118</t>
   </si>
   <si>
-    <t>Portoviejo</t>
-  </si>
-  <si>
     <t>901542091</t>
   </si>
   <si>
@@ -957,10 +1050,10 @@
     <t>Bolívar, Mira, Tulcán</t>
   </si>
   <si>
-    <t>El Guabo, Pasaje</t>
-  </si>
-  <si>
-    <t>Eloy Alfaro, Esmeraldas, Muisne, Quinindé</t>
+    <t>El Guabo, Huaquillas, Machala, Pasaje</t>
+  </si>
+  <si>
+    <t>Eloy Alfaro, Esmeraldas, Muisne, Quinindé, San Lorenzo</t>
   </si>
   <si>
     <t>Guayaquil, Milagro, Palestina, Salitre</t>
@@ -969,7 +1062,7 @@
     <t>Espíndola, Loja, Pindal, Quilanga</t>
   </si>
   <si>
-    <t>Flavio Alfaro, Pichincha, Portoviejo, Santa Ana</t>
+    <t>Flavio Alfaro, Pedernales, Pichincha, Portoviejo, Santa Ana</t>
   </si>
   <si>
     <t>Archidona, Tena</t>
@@ -1026,7 +1119,7 @@
     <t>Alertas</t>
   </si>
   <si>
-    <t>Se muestran únicamente alertas revisadas con código UA registrado, desde el 14 de septiembre de 2026. El conteo corresponde a códigos de alerta distintos vinculados a unidades identificadas. Los registros sin código quedan fuera de este alcance. La fecha corresponde al registro y una alerta no equivale necesariamente a un evento único. El campo Afectados mezcla personas, familias y usuarios; no se suma como personas únicas. La base no certifica atribución causal a ENOS.</t>
+    <t>Seguimiento desde el 14/09/2026, complementado con reportes sectoriales de octubre: 10 alertas con código UA y 11 reportes sectoriales. Los 6 reportes gerontológicos describen sucesos de agosto sin día exacto; no se asignan a la evolución diaria. Los identificadores DIS/GER permiten localizar las filas incorporadas, no son códigos oficiales ni códigos UA. Las fuentes sectoriales indican que la prestación del servicio se mantiene. Alertas, unidades y personas son medidas distintas.</t>
   </si>
   <si>
     <t>La ayuda memoria no identifica pagos exclusivamente atribuibles a ENOS ni fechas individuales para recortar desde el 14/09. Se muestran únicamente las filas de inundación como referencia: pagos gestionados desde el 29/08 y casos en articulación al 23/10. Articulación no equivale a pago. Las proyecciones corresponden a planificación nacional 2026–2027.</t>
@@ -2119,10 +2212,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>0</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2418,10 +2511,10 @@
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>10</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>10</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2898,10 +2991,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>0</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3197,10 +3290,10 @@
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>10</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>10</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5171,7 +5264,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2" descr="Mapa del Ecuador: alertas con código ua"/>
+        <xdr:cNvPr id="3" name="Picture 2" descr="Mapa del Ecuador: alertas reportadas"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -6367,7 +6460,7 @@
     </row>
     <row r="10" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="14">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="C10" s="15"/>
       <c r="D10" s="15"/>
@@ -8972,7 +9065,7 @@
     <tabColor rgb="FFF8C018"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.140625" customWidth="1"/>
@@ -9112,187 +9205,177 @@
         <v>91</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="21" customHeight="1">
+    <row r="9" spans="1:12" ht="35" customHeight="1">
       <c r="B9" s="21" t="s">
         <v>92</v>
       </c>
       <c r="C9" s="37">
-        <v>46315</v>
+        <v>46321</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E9" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9" s="38"/>
+      <c r="G9" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9" s="33" t="s">
         <v>93</v>
       </c>
-      <c r="F9" s="38" t="s">
+      <c r="I9" s="33" t="s">
         <v>94</v>
       </c>
-      <c r="G9" s="33" t="s">
+      <c r="J9" s="33" t="s">
         <v>95</v>
       </c>
-      <c r="H9" s="33" t="s">
+      <c r="K9" s="33" t="s">
         <v>96</v>
       </c>
-      <c r="I9" s="33" t="s">
+    </row>
+    <row r="10" spans="1:12" ht="35" customHeight="1">
+      <c r="B10" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="J9" s="33" t="s">
+      <c r="C10" s="39">
+        <v>46321</v>
+      </c>
+      <c r="D10" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" s="40"/>
+      <c r="G10" s="34" t="s">
+        <v>58</v>
+      </c>
+      <c r="H10" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="I10" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="K9" s="33" t="s">
+      <c r="J10" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="K10" s="34" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="35" customHeight="1">
+      <c r="B11" s="21" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" ht="21" customHeight="1">
-      <c r="B10" s="24" t="s">
+      <c r="C11" s="37">
+        <v>46321</v>
+      </c>
+      <c r="D11" s="33" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="33" t="s">
         <v>100</v>
       </c>
-      <c r="C10" s="39">
-        <v>46315</v>
-      </c>
-      <c r="D10" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="34" t="s">
+      <c r="F11" s="38"/>
+      <c r="G11" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="H11" s="33" t="s">
         <v>93</v>
       </c>
-      <c r="F10" s="40" t="s">
+      <c r="I11" s="33" t="s">
+        <v>98</v>
+      </c>
+      <c r="J11" s="33" t="s">
+        <v>95</v>
+      </c>
+      <c r="K11" s="33" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="35" customHeight="1">
+      <c r="B12" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="G10" s="34" t="s">
-        <v>81</v>
-      </c>
-      <c r="H10" s="34" t="s">
+      <c r="C12" s="39">
+        <v>46320</v>
+      </c>
+      <c r="D12" s="34" t="s">
+        <v>102</v>
+      </c>
+      <c r="E12" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="F12" s="40"/>
+      <c r="G12" s="34" t="s">
+        <v>104</v>
+      </c>
+      <c r="H12" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="I12" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="J12" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="K12" s="34" t="s">
         <v>96</v>
-      </c>
-      <c r="I10" s="34" t="s">
-        <v>102</v>
-      </c>
-      <c r="J10" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="K10" s="34" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="21" customHeight="1">
-      <c r="B11" s="21" t="s">
-        <v>103</v>
-      </c>
-      <c r="C11" s="37">
-        <v>46315</v>
-      </c>
-      <c r="D11" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" s="33" t="s">
-        <v>93</v>
-      </c>
-      <c r="F11" s="38" t="s">
-        <v>104</v>
-      </c>
-      <c r="G11" s="33" t="s">
-        <v>105</v>
-      </c>
-      <c r="H11" s="33" t="s">
-        <v>96</v>
-      </c>
-      <c r="I11" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="J11" s="33" t="s">
-        <v>98</v>
-      </c>
-      <c r="K11" s="33" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="21" customHeight="1">
-      <c r="B12" s="24" t="s">
-        <v>107</v>
-      </c>
-      <c r="C12" s="39">
-        <v>46315</v>
-      </c>
-      <c r="D12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="F12" s="40" t="s">
-        <v>108</v>
-      </c>
-      <c r="G12" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="H12" s="34" t="s">
-        <v>96</v>
-      </c>
-      <c r="I12" s="34" t="s">
-        <v>110</v>
-      </c>
-      <c r="J12" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="K12" s="34" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="35" customHeight="1">
       <c r="B13" s="21" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C13" s="37">
-        <v>46315</v>
+        <v>46320</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>26</v>
+        <v>102</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>43</v>
-      </c>
-      <c r="F13" s="38" t="s">
-        <v>112</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="F13" s="38"/>
       <c r="G13" s="33" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="H13" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="I13" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="J13" s="33" t="s">
+        <v>95</v>
+      </c>
+      <c r="K13" s="33" t="s">
         <v>96</v>
       </c>
-      <c r="I13" s="33" t="s">
-        <v>114</v>
-      </c>
-      <c r="J13" s="33" t="s">
-        <v>115</v>
-      </c>
-      <c r="K13" s="33" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="35" customHeight="1">
+    </row>
+    <row r="14" spans="1:12" ht="21" customHeight="1">
       <c r="B14" s="24" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="C14" s="39">
         <v>46315</v>
       </c>
       <c r="D14" s="34" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>43</v>
+        <v>110</v>
       </c>
       <c r="F14" s="40" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="G14" s="34" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="H14" s="34" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="I14" s="34" t="s">
         <v>114</v>
@@ -9301,139 +9384,479 @@
         <v>115</v>
       </c>
       <c r="K14" s="34" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="35" customHeight="1">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="21" customHeight="1">
       <c r="B15" s="21" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C15" s="37">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="D15" s="33" t="s">
         <v>27</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="F15" s="38" t="s">
+        <v>118</v>
+      </c>
+      <c r="G15" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="H15" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="I15" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="J15" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="K15" s="33" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="21" customHeight="1">
+      <c r="B16" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="G15" s="33" t="s">
-        <v>121</v>
-      </c>
-      <c r="H15" s="33" t="s">
-        <v>96</v>
-      </c>
-      <c r="I15" s="33" t="s">
-        <v>122</v>
-      </c>
-      <c r="J15" s="33" t="s">
-        <v>98</v>
-      </c>
-      <c r="K15" s="33" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="35" customHeight="1">
-      <c r="B16" s="24" t="s">
-        <v>123</v>
-      </c>
       <c r="C16" s="39">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="D16" s="34" t="s">
         <v>27</v>
       </c>
       <c r="E16" s="34" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="F16" s="40" t="s">
+        <v>121</v>
+      </c>
+      <c r="G16" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="H16" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="I16" s="34" t="s">
+        <v>123</v>
+      </c>
+      <c r="J16" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="K16" s="34" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" ht="21" customHeight="1">
+      <c r="B17" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="G16" s="34" t="s">
+      <c r="C17" s="37">
+        <v>46315</v>
+      </c>
+      <c r="D17" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="33" t="s">
+        <v>110</v>
+      </c>
+      <c r="F17" s="38" t="s">
         <v>125</v>
       </c>
-      <c r="H16" s="34" t="s">
-        <v>96</v>
-      </c>
-      <c r="I16" s="34" t="s">
-        <v>122</v>
-      </c>
-      <c r="J16" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="K16" s="34" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="17" spans="2:11" ht="35" customHeight="1">
-      <c r="B17" s="21" t="s">
+      <c r="G17" s="33" t="s">
         <v>126</v>
       </c>
-      <c r="C17" s="37">
-        <v>46311</v>
-      </c>
-      <c r="D17" s="33" t="s">
+      <c r="H17" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="I17" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="E17" s="33" t="s">
-        <v>128</v>
-      </c>
-      <c r="F17" s="38" t="s">
-        <v>129</v>
-      </c>
-      <c r="G17" s="33" t="s">
-        <v>130</v>
-      </c>
-      <c r="H17" s="33" t="s">
-        <v>131</v>
-      </c>
-      <c r="I17" s="33" t="s">
-        <v>132</v>
-      </c>
       <c r="J17" s="33" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="K17" s="33" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" spans="2:11" ht="35" customHeight="1">
       <c r="B18" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="C18" s="39">
+        <v>46315</v>
+      </c>
+      <c r="D18" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="E18" s="34" t="s">
+        <v>43</v>
+      </c>
+      <c r="F18" s="40" t="s">
+        <v>129</v>
+      </c>
+      <c r="G18" s="34" t="s">
+        <v>130</v>
+      </c>
+      <c r="H18" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="I18" s="34" t="s">
+        <v>131</v>
+      </c>
+      <c r="J18" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="K18" s="34" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" ht="35" customHeight="1">
+      <c r="B19" s="21" t="s">
+        <v>132</v>
+      </c>
+      <c r="C19" s="37">
+        <v>46315</v>
+      </c>
+      <c r="D19" s="33" t="s">
+        <v>26</v>
+      </c>
+      <c r="E19" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="F19" s="38" t="s">
         <v>133</v>
       </c>
-      <c r="C18" s="39">
+      <c r="G19" s="33" t="s">
+        <v>134</v>
+      </c>
+      <c r="H19" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="I19" s="33" t="s">
+        <v>131</v>
+      </c>
+      <c r="J19" s="33" t="s">
+        <v>95</v>
+      </c>
+      <c r="K19" s="33" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" ht="35" customHeight="1">
+      <c r="B20" s="24" t="s">
+        <v>135</v>
+      </c>
+      <c r="C20" s="39">
+        <v>46314</v>
+      </c>
+      <c r="D20" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="F20" s="40" t="s">
+        <v>136</v>
+      </c>
+      <c r="G20" s="34" t="s">
+        <v>137</v>
+      </c>
+      <c r="H20" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="I20" s="34" t="s">
+        <v>138</v>
+      </c>
+      <c r="J20" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="K20" s="34" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" ht="35" customHeight="1">
+      <c r="B21" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="C21" s="37">
+        <v>46314</v>
+      </c>
+      <c r="D21" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="33" t="s">
+        <v>60</v>
+      </c>
+      <c r="F21" s="38" t="s">
+        <v>140</v>
+      </c>
+      <c r="G21" s="33" t="s">
+        <v>141</v>
+      </c>
+      <c r="H21" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="I21" s="33" t="s">
+        <v>138</v>
+      </c>
+      <c r="J21" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="K21" s="33" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" ht="35" customHeight="1">
+      <c r="B22" s="24" t="s">
+        <v>142</v>
+      </c>
+      <c r="C22" s="39">
         <v>46311</v>
       </c>
-      <c r="D18" s="34" t="s">
-        <v>127</v>
-      </c>
-      <c r="E18" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F18" s="40" t="s">
-        <v>134</v>
-      </c>
-      <c r="G18" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="H18" s="34" t="s">
-        <v>131</v>
-      </c>
-      <c r="I18" s="34" t="s">
-        <v>132</v>
-      </c>
-      <c r="J18" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="K18" s="34" t="s">
-        <v>99</v>
+      <c r="D22" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="E22" s="34" t="s">
+        <v>144</v>
+      </c>
+      <c r="F22" s="40" t="s">
+        <v>145</v>
+      </c>
+      <c r="G22" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="H22" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="I22" s="34" t="s">
+        <v>148</v>
+      </c>
+      <c r="J22" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="K22" s="34" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" ht="35" customHeight="1">
+      <c r="B23" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="C23" s="37">
+        <v>46311</v>
+      </c>
+      <c r="D23" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="E23" s="33" t="s">
+        <v>144</v>
+      </c>
+      <c r="F23" s="38" t="s">
+        <v>150</v>
+      </c>
+      <c r="G23" s="33" t="s">
+        <v>151</v>
+      </c>
+      <c r="H23" s="33" t="s">
+        <v>147</v>
+      </c>
+      <c r="I23" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="J23" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="K23" s="33" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" ht="49" customHeight="1">
+      <c r="B24" s="24" t="s">
+        <v>152</v>
+      </c>
+      <c r="C24" s="39" t="s">
+        <v>153</v>
+      </c>
+      <c r="D24" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="E24" s="34" t="s">
+        <v>155</v>
+      </c>
+      <c r="F24" s="40"/>
+      <c r="G24" s="34" t="s">
+        <v>58</v>
+      </c>
+      <c r="H24" s="34" t="s">
+        <v>156</v>
+      </c>
+      <c r="I24" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="J24" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="K24" s="34" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" ht="35" customHeight="1">
+      <c r="B25" s="21" t="s">
+        <v>158</v>
+      </c>
+      <c r="C25" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="D25" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="E25" s="33" t="s">
+        <v>159</v>
+      </c>
+      <c r="F25" s="38"/>
+      <c r="G25" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="H25" s="33" t="s">
+        <v>156</v>
+      </c>
+      <c r="I25" s="33" t="s">
+        <v>160</v>
+      </c>
+      <c r="J25" s="33" t="s">
+        <v>95</v>
+      </c>
+      <c r="K25" s="33" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" ht="35" customHeight="1">
+      <c r="B26" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="C26" s="39" t="s">
+        <v>153</v>
+      </c>
+      <c r="D26" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="E26" s="34" t="s">
+        <v>162</v>
+      </c>
+      <c r="F26" s="40"/>
+      <c r="G26" s="34" t="s">
+        <v>58</v>
+      </c>
+      <c r="H26" s="34" t="s">
+        <v>156</v>
+      </c>
+      <c r="I26" s="34" t="s">
+        <v>163</v>
+      </c>
+      <c r="J26" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="K26" s="34" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11" ht="35" customHeight="1">
+      <c r="B27" s="21" t="s">
+        <v>164</v>
+      </c>
+      <c r="C27" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="D27" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E27" s="33" t="s">
+        <v>110</v>
+      </c>
+      <c r="F27" s="38"/>
+      <c r="G27" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="H27" s="33" t="s">
+        <v>156</v>
+      </c>
+      <c r="I27" s="33" t="s">
+        <v>165</v>
+      </c>
+      <c r="J27" s="33" t="s">
+        <v>95</v>
+      </c>
+      <c r="K27" s="33" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" ht="35" customHeight="1">
+      <c r="B28" s="24" t="s">
+        <v>166</v>
+      </c>
+      <c r="C28" s="39" t="s">
+        <v>153</v>
+      </c>
+      <c r="D28" s="34" t="s">
+        <v>167</v>
+      </c>
+      <c r="E28" s="34" t="s">
+        <v>168</v>
+      </c>
+      <c r="F28" s="40"/>
+      <c r="G28" s="34" t="s">
+        <v>58</v>
+      </c>
+      <c r="H28" s="34" t="s">
+        <v>156</v>
+      </c>
+      <c r="I28" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="J28" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="K28" s="34" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="29" spans="2:11" ht="35" customHeight="1">
+      <c r="B29" s="21" t="s">
+        <v>170</v>
+      </c>
+      <c r="C29" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="D29" s="33" t="s">
+        <v>26</v>
+      </c>
+      <c r="E29" s="33" t="s">
+        <v>171</v>
+      </c>
+      <c r="F29" s="38"/>
+      <c r="G29" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="H29" s="33" t="s">
+        <v>156</v>
+      </c>
+      <c r="I29" s="33" t="s">
+        <v>172</v>
+      </c>
+      <c r="J29" s="33" t="s">
+        <v>95</v>
+      </c>
+      <c r="K29" s="33" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B8:K18"/>
+  <autoFilter ref="B8:K29"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.55" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
@@ -9556,20 +9979,20 @@
     </row>
     <row r="7" spans="1:15" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>136</v>
+        <v>173</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
     </row>
     <row r="8" spans="1:15" ht="36" customHeight="1">
       <c r="B8" s="19" t="s">
-        <v>137</v>
+        <v>174</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>138</v>
+        <v>175</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>139</v>
+        <v>176</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="19" customHeight="1">
@@ -10028,10 +10451,10 @@
         <v>46320</v>
       </c>
       <c r="C50" s="25">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D50" s="25">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="51" spans="2:4" ht="19" customHeight="1">
@@ -10039,10 +10462,10 @@
         <v>46321</v>
       </c>
       <c r="C51" s="22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D51" s="22">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="52" spans="2:4" ht="22" customHeight="1">
@@ -10051,7 +10474,7 @@
       </c>
       <c r="C52" s="28">
         <f>SUM(C9:C51)</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D52" s="35"/>
     </row>
@@ -10108,7 +10531,7 @@
     <row r="2" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>140</v>
+        <v>177</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -10187,7 +10610,7 @@
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="F7" s="8" t="s">
-        <v>141</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.25">
@@ -10195,16 +10618,16 @@
         <v>25</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>142</v>
+        <v>179</v>
       </c>
       <c r="D8" s="20" t="s">
         <v>20</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>143</v>
+        <v>180</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>144</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
@@ -10226,7 +10649,7 @@
     </row>
     <row r="10" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="24" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="C10" s="25">
         <v>3820</v>
@@ -10243,7 +10666,7 @@
     </row>
     <row r="11" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="21" t="s">
-        <v>146</v>
+        <v>182</v>
       </c>
       <c r="C11" s="22">
         <v>780</v>
@@ -10260,7 +10683,7 @@
     </row>
     <row r="12" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="24" t="s">
-        <v>147</v>
+        <v>183</v>
       </c>
       <c r="C12" s="25">
         <v>527</v>
@@ -10277,7 +10700,7 @@
     </row>
     <row r="13" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="21" t="s">
-        <v>148</v>
+        <v>184</v>
       </c>
       <c r="C13" s="22">
         <v>498</v>
@@ -10294,7 +10717,7 @@
     </row>
     <row r="14" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="24" t="s">
-        <v>149</v>
+        <v>185</v>
       </c>
       <c r="C14" s="25">
         <v>250</v>
@@ -10311,7 +10734,7 @@
     </row>
     <row r="15" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="21" t="s">
-        <v>150</v>
+        <v>186</v>
       </c>
       <c r="C15" s="22">
         <v>141</v>
@@ -10328,7 +10751,7 @@
     </row>
     <row r="16" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="24" t="s">
-        <v>151</v>
+        <v>187</v>
       </c>
       <c r="C16" s="25">
         <v>79</v>
@@ -10345,7 +10768,7 @@
     </row>
     <row r="17" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="21" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="C17" s="22">
         <v>75</v>
@@ -10379,7 +10802,7 @@
     </row>
     <row r="19" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="21" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="C19" s="22">
         <v>64</v>
@@ -10396,7 +10819,7 @@
     </row>
     <row r="20" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="24" t="s">
-        <v>153</v>
+        <v>102</v>
       </c>
       <c r="C20" s="25">
         <v>64</v>
@@ -10413,7 +10836,7 @@
     </row>
     <row r="21" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="21" t="s">
-        <v>154</v>
+        <v>189</v>
       </c>
       <c r="C21" s="22">
         <v>60</v>
@@ -10430,7 +10853,7 @@
     </row>
     <row r="22" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="24" t="s">
-        <v>155</v>
+        <v>190</v>
       </c>
       <c r="C22" s="25">
         <v>44</v>
@@ -10447,7 +10870,7 @@
     </row>
     <row r="23" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="21" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="C23" s="22">
         <v>17</v>
@@ -10464,7 +10887,7 @@
     </row>
     <row r="24" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="24" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C24" s="25">
         <v>17</v>
@@ -10498,7 +10921,7 @@
     </row>
     <row r="26" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="24" t="s">
-        <v>158</v>
+        <v>192</v>
       </c>
       <c r="C26" s="25">
         <v>11</v>
@@ -10515,7 +10938,7 @@
     </row>
     <row r="27" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="21" t="s">
-        <v>159</v>
+        <v>193</v>
       </c>
       <c r="C27" s="22">
         <v>7</v>
@@ -10532,7 +10955,7 @@
     </row>
     <row r="28" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="24" t="s">
-        <v>160</v>
+        <v>194</v>
       </c>
       <c r="C28" s="25">
         <v>7</v>
@@ -10569,7 +10992,7 @@
     </row>
     <row r="31" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="43" t="s">
-        <v>161</v>
+        <v>195</v>
       </c>
       <c r="C31" s="43"/>
       <c r="D31" s="43"/>
@@ -10660,7 +11083,7 @@
     <row r="2" spans="1:9" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>162</v>
+        <v>196</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -10709,7 +11132,7 @@
     </row>
     <row r="7" spans="1:9" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>163</v>
+        <v>197</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -10717,12 +11140,12 @@
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="8" t="s">
-        <v>141</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="46" customHeight="1">
       <c r="B8" s="44" t="s">
-        <v>164</v>
+        <v>198</v>
       </c>
       <c r="C8" s="44"/>
       <c r="D8" s="44"/>
@@ -10734,7 +11157,7 @@
     <row r="9" spans="1:9" ht="8" customHeight="1"/>
     <row r="10" spans="1:9" ht="36" customHeight="1">
       <c r="B10" s="19" t="s">
-        <v>137</v>
+        <v>174</v>
       </c>
       <c r="C10" s="32" t="s">
         <v>25</v>
@@ -10743,16 +11166,16 @@
         <v>39</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>142</v>
+        <v>179</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>165</v>
+        <v>199</v>
       </c>
       <c r="G10" s="20" t="s">
-        <v>143</v>
+        <v>180</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>166</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="19" customHeight="1">
@@ -10760,10 +11183,10 @@
         <v>46265</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>146</v>
+        <v>182</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>167</v>
+        <v>201</v>
       </c>
       <c r="E11" s="22">
         <v>399</v>
@@ -10775,7 +11198,7 @@
         <v>399</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>168</v>
+        <v>202</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="19" customHeight="1">
@@ -10783,10 +11206,10 @@
         <v>46265</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D12" s="34" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E12" s="25">
         <v>3</v>
@@ -10798,7 +11221,7 @@
         <v>3</v>
       </c>
       <c r="H12" s="40" t="s">
-        <v>170</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="19" customHeight="1">
@@ -10806,10 +11229,10 @@
         <v>46265</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E13" s="22">
         <v>1</v>
@@ -10821,7 +11244,7 @@
         <v>1</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>171</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="19" customHeight="1">
@@ -10829,10 +11252,10 @@
         <v>46268</v>
       </c>
       <c r="C14" s="34" t="s">
-        <v>149</v>
+        <v>185</v>
       </c>
       <c r="D14" s="34" t="s">
-        <v>172</v>
+        <v>206</v>
       </c>
       <c r="E14" s="25">
         <v>250</v>
@@ -10844,7 +11267,7 @@
         <v>249</v>
       </c>
       <c r="H14" s="40" t="s">
-        <v>173</v>
+        <v>207</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="19" customHeight="1">
@@ -10852,10 +11275,10 @@
         <v>46268</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>174</v>
+        <v>208</v>
       </c>
       <c r="E15" s="22">
         <v>10</v>
@@ -10867,7 +11290,7 @@
         <v>1</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="19" customHeight="1">
@@ -10875,10 +11298,10 @@
         <v>46268</v>
       </c>
       <c r="C16" s="34" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="D16" s="34" t="s">
-        <v>176</v>
+        <v>210</v>
       </c>
       <c r="E16" s="25">
         <v>10</v>
@@ -10890,7 +11313,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="40" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="19" customHeight="1">
@@ -10898,10 +11321,10 @@
         <v>46269</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>178</v>
+        <v>212</v>
       </c>
       <c r="E17" s="22">
         <v>7</v>
@@ -10913,7 +11336,7 @@
         <v>1</v>
       </c>
       <c r="H17" s="38" t="s">
-        <v>179</v>
+        <v>213</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="19" customHeight="1">
@@ -10921,10 +11344,10 @@
         <v>46274</v>
       </c>
       <c r="C18" s="34" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="D18" s="34" t="s">
-        <v>180</v>
+        <v>214</v>
       </c>
       <c r="E18" s="25">
         <v>20</v>
@@ -10936,7 +11359,7 @@
         <v>3</v>
       </c>
       <c r="H18" s="40" t="s">
-        <v>181</v>
+        <v>215</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="19" customHeight="1">
@@ -10944,10 +11367,10 @@
         <v>46274</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D19" s="33" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E19" s="22">
         <v>2</v>
@@ -10959,7 +11382,7 @@
         <v>1</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>182</v>
+        <v>216</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="19" customHeight="1">
@@ -10967,10 +11390,10 @@
         <v>46274</v>
       </c>
       <c r="C20" s="34" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D20" s="34" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E20" s="25">
         <v>1</v>
@@ -10982,7 +11405,7 @@
         <v>1</v>
       </c>
       <c r="H20" s="40" t="s">
-        <v>183</v>
+        <v>217</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="19" customHeight="1">
@@ -10990,10 +11413,10 @@
         <v>46274</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D21" s="33" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E21" s="22">
         <v>1</v>
@@ -11005,7 +11428,7 @@
         <v>1</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>184</v>
+        <v>218</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="19" customHeight="1">
@@ -11028,7 +11451,7 @@
         <v>1</v>
       </c>
       <c r="H22" s="40" t="s">
-        <v>185</v>
+        <v>219</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="19" customHeight="1">
@@ -11051,7 +11474,7 @@
         <v>2</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>186</v>
+        <v>220</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="19" customHeight="1">
@@ -11059,10 +11482,10 @@
         <v>46275</v>
       </c>
       <c r="C24" s="34" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D24" s="34" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E24" s="25">
         <v>1</v>
@@ -11074,7 +11497,7 @@
         <v>1</v>
       </c>
       <c r="H24" s="40" t="s">
-        <v>187</v>
+        <v>221</v>
       </c>
     </row>
     <row r="25" spans="2:8" ht="19" customHeight="1">
@@ -11082,10 +11505,10 @@
         <v>46275</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D25" s="33" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E25" s="22">
         <v>1</v>
@@ -11097,7 +11520,7 @@
         <v>1</v>
       </c>
       <c r="H25" s="38" t="s">
-        <v>188</v>
+        <v>222</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="19" customHeight="1">
@@ -11105,10 +11528,10 @@
         <v>46280</v>
       </c>
       <c r="C26" s="34" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D26" s="34" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E26" s="25">
         <v>1</v>
@@ -11120,7 +11543,7 @@
         <v>1</v>
       </c>
       <c r="H26" s="40" t="s">
-        <v>189</v>
+        <v>223</v>
       </c>
     </row>
     <row r="27" spans="2:8" ht="19" customHeight="1">
@@ -11128,10 +11551,10 @@
         <v>46283</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>146</v>
+        <v>182</v>
       </c>
       <c r="D27" s="33" t="s">
-        <v>167</v>
+        <v>201</v>
       </c>
       <c r="E27" s="22">
         <v>66</v>
@@ -11143,7 +11566,7 @@
         <v>66</v>
       </c>
       <c r="H27" s="38" t="s">
-        <v>190</v>
+        <v>224</v>
       </c>
     </row>
     <row r="28" spans="2:8" ht="19" customHeight="1">
@@ -11151,10 +11574,10 @@
         <v>46283</v>
       </c>
       <c r="C28" s="34" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D28" s="34" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E28" s="25">
         <v>1</v>
@@ -11166,7 +11589,7 @@
         <v>1</v>
       </c>
       <c r="H28" s="40" t="s">
-        <v>191</v>
+        <v>225</v>
       </c>
     </row>
     <row r="29" spans="2:8" ht="19" customHeight="1">
@@ -11177,7 +11600,7 @@
         <v>27</v>
       </c>
       <c r="D29" s="33" t="s">
-        <v>192</v>
+        <v>226</v>
       </c>
       <c r="E29" s="22">
         <v>1500</v>
@@ -11189,7 +11612,7 @@
         <v>1500</v>
       </c>
       <c r="H29" s="38" t="s">
-        <v>193</v>
+        <v>227</v>
       </c>
     </row>
     <row r="30" spans="2:8" ht="19" customHeight="1">
@@ -11197,10 +11620,10 @@
         <v>46289</v>
       </c>
       <c r="C30" s="34" t="s">
-        <v>146</v>
+        <v>182</v>
       </c>
       <c r="D30" s="34" t="s">
-        <v>194</v>
+        <v>228</v>
       </c>
       <c r="E30" s="25">
         <v>182</v>
@@ -11212,7 +11635,7 @@
         <v>182</v>
       </c>
       <c r="H30" s="40" t="s">
-        <v>195</v>
+        <v>229</v>
       </c>
     </row>
     <row r="31" spans="2:8" ht="19" customHeight="1">
@@ -11220,10 +11643,10 @@
         <v>46289</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D31" s="33" t="s">
-        <v>196</v>
+        <v>230</v>
       </c>
       <c r="E31" s="22">
         <v>130</v>
@@ -11235,7 +11658,7 @@
         <v>65</v>
       </c>
       <c r="H31" s="38" t="s">
-        <v>197</v>
+        <v>231</v>
       </c>
     </row>
     <row r="32" spans="2:8" ht="19" customHeight="1">
@@ -11246,7 +11669,7 @@
         <v>27</v>
       </c>
       <c r="D32" s="34" t="s">
-        <v>192</v>
+        <v>226</v>
       </c>
       <c r="E32" s="25">
         <v>700</v>
@@ -11258,7 +11681,7 @@
         <v>700</v>
       </c>
       <c r="H32" s="40" t="s">
-        <v>198</v>
+        <v>232</v>
       </c>
     </row>
     <row r="33" spans="2:8" ht="19" customHeight="1">
@@ -11269,7 +11692,7 @@
         <v>27</v>
       </c>
       <c r="D33" s="33" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="E33" s="22">
         <v>400</v>
@@ -11281,7 +11704,7 @@
         <v>400</v>
       </c>
       <c r="H33" s="38" t="s">
-        <v>199</v>
+        <v>233</v>
       </c>
     </row>
     <row r="34" spans="2:8" ht="19" customHeight="1">
@@ -11289,10 +11712,10 @@
         <v>46293</v>
       </c>
       <c r="C34" s="34" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D34" s="34" t="s">
-        <v>196</v>
+        <v>230</v>
       </c>
       <c r="E34" s="25">
         <v>140</v>
@@ -11304,7 +11727,7 @@
         <v>140</v>
       </c>
       <c r="H34" s="40" t="s">
-        <v>200</v>
+        <v>234</v>
       </c>
     </row>
     <row r="35" spans="2:8" ht="19" customHeight="1">
@@ -11315,7 +11738,7 @@
         <v>27</v>
       </c>
       <c r="D35" s="33" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="E35" s="22">
         <v>300</v>
@@ -11327,7 +11750,7 @@
         <v>300</v>
       </c>
       <c r="H35" s="38" t="s">
-        <v>201</v>
+        <v>235</v>
       </c>
     </row>
     <row r="36" spans="2:8" ht="19" customHeight="1">
@@ -11335,10 +11758,10 @@
         <v>46294</v>
       </c>
       <c r="C36" s="34" t="s">
-        <v>147</v>
+        <v>183</v>
       </c>
       <c r="D36" s="34" t="s">
-        <v>202</v>
+        <v>236</v>
       </c>
       <c r="E36" s="25">
         <v>60</v>
@@ -11350,7 +11773,7 @@
         <v>23</v>
       </c>
       <c r="H36" s="40" t="s">
-        <v>203</v>
+        <v>237</v>
       </c>
     </row>
     <row r="37" spans="2:8" ht="19" customHeight="1">
@@ -11358,10 +11781,10 @@
         <v>46294</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>159</v>
+        <v>193</v>
       </c>
       <c r="D37" s="33" t="s">
-        <v>204</v>
+        <v>238</v>
       </c>
       <c r="E37" s="22">
         <v>7</v>
@@ -11373,7 +11796,7 @@
         <v>1</v>
       </c>
       <c r="H37" s="38" t="s">
-        <v>205</v>
+        <v>239</v>
       </c>
     </row>
     <row r="38" spans="2:8" ht="19" customHeight="1">
@@ -11381,10 +11804,10 @@
         <v>46295</v>
       </c>
       <c r="C38" s="34" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="D38" s="34" t="s">
-        <v>206</v>
+        <v>240</v>
       </c>
       <c r="E38" s="25">
         <v>10</v>
@@ -11396,7 +11819,7 @@
         <v>3</v>
       </c>
       <c r="H38" s="40" t="s">
-        <v>207</v>
+        <v>241</v>
       </c>
     </row>
     <row r="39" spans="2:8" ht="19" customHeight="1">
@@ -11404,10 +11827,10 @@
         <v>46296</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D39" s="33" t="s">
-        <v>196</v>
+        <v>230</v>
       </c>
       <c r="E39" s="22">
         <v>540</v>
@@ -11419,7 +11842,7 @@
         <v>270</v>
       </c>
       <c r="H39" s="38" t="s">
-        <v>208</v>
+        <v>242</v>
       </c>
     </row>
     <row r="40" spans="2:8" ht="19" customHeight="1">
@@ -11427,10 +11850,10 @@
         <v>46296</v>
       </c>
       <c r="C40" s="34" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D40" s="34" t="s">
-        <v>209</v>
+        <v>243</v>
       </c>
       <c r="E40" s="25">
         <v>120</v>
@@ -11442,7 +11865,7 @@
         <v>120</v>
       </c>
       <c r="H40" s="40" t="s">
-        <v>210</v>
+        <v>244</v>
       </c>
     </row>
     <row r="41" spans="2:8" ht="19" customHeight="1">
@@ -11450,10 +11873,10 @@
         <v>46296</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D41" s="33" t="s">
-        <v>209</v>
+        <v>243</v>
       </c>
       <c r="E41" s="22">
         <v>80</v>
@@ -11465,7 +11888,7 @@
         <v>80</v>
       </c>
       <c r="H41" s="38" t="s">
-        <v>211</v>
+        <v>245</v>
       </c>
     </row>
     <row r="42" spans="2:8" ht="19" customHeight="1">
@@ -11473,10 +11896,10 @@
         <v>46296</v>
       </c>
       <c r="C42" s="34" t="s">
-        <v>146</v>
+        <v>182</v>
       </c>
       <c r="D42" s="34" t="s">
-        <v>167</v>
+        <v>201</v>
       </c>
       <c r="E42" s="25">
         <v>5</v>
@@ -11488,7 +11911,7 @@
         <v>5</v>
       </c>
       <c r="H42" s="40" t="s">
-        <v>212</v>
+        <v>246</v>
       </c>
     </row>
     <row r="43" spans="2:8" ht="19" customHeight="1">
@@ -11496,10 +11919,10 @@
         <v>46296</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D43" s="33" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E43" s="22">
         <v>1</v>
@@ -11511,7 +11934,7 @@
         <v>1</v>
       </c>
       <c r="H43" s="38" t="s">
-        <v>213</v>
+        <v>247</v>
       </c>
     </row>
     <row r="44" spans="2:8" ht="19" customHeight="1">
@@ -11519,10 +11942,10 @@
         <v>46296</v>
       </c>
       <c r="C44" s="34" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D44" s="34" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E44" s="25">
         <v>1</v>
@@ -11534,7 +11957,7 @@
         <v>1</v>
       </c>
       <c r="H44" s="40" t="s">
-        <v>214</v>
+        <v>248</v>
       </c>
     </row>
     <row r="45" spans="2:8" ht="19" customHeight="1">
@@ -11542,10 +11965,10 @@
         <v>46297</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>146</v>
+        <v>182</v>
       </c>
       <c r="D45" s="33" t="s">
-        <v>150</v>
+        <v>186</v>
       </c>
       <c r="E45" s="22">
         <v>87</v>
@@ -11557,7 +11980,7 @@
         <v>87</v>
       </c>
       <c r="H45" s="38" t="s">
-        <v>215</v>
+        <v>249</v>
       </c>
     </row>
     <row r="46" spans="2:8" ht="19" customHeight="1">
@@ -11565,10 +11988,10 @@
         <v>46297</v>
       </c>
       <c r="C46" s="34" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D46" s="34" t="s">
-        <v>209</v>
+        <v>243</v>
       </c>
       <c r="E46" s="25">
         <v>85</v>
@@ -11580,7 +12003,7 @@
         <v>85</v>
       </c>
       <c r="H46" s="40" t="s">
-        <v>216</v>
+        <v>250</v>
       </c>
     </row>
     <row r="47" spans="2:8" ht="19" customHeight="1">
@@ -11588,10 +12011,10 @@
         <v>46297</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>148</v>
+        <v>184</v>
       </c>
       <c r="D47" s="33" t="s">
-        <v>217</v>
+        <v>251</v>
       </c>
       <c r="E47" s="22">
         <v>85</v>
@@ -11603,7 +12026,7 @@
         <v>85</v>
       </c>
       <c r="H47" s="38" t="s">
-        <v>218</v>
+        <v>252</v>
       </c>
     </row>
     <row r="48" spans="2:8" ht="19" customHeight="1">
@@ -11611,10 +12034,10 @@
         <v>46298</v>
       </c>
       <c r="C48" s="34" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D48" s="34" t="s">
-        <v>219</v>
+        <v>253</v>
       </c>
       <c r="E48" s="25">
         <v>772</v>
@@ -11626,7 +12049,7 @@
         <v>772</v>
       </c>
       <c r="H48" s="40" t="s">
-        <v>220</v>
+        <v>254</v>
       </c>
     </row>
     <row r="49" spans="2:8" ht="19" customHeight="1">
@@ -11634,10 +12057,10 @@
         <v>46298</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D49" s="33" t="s">
-        <v>196</v>
+        <v>230</v>
       </c>
       <c r="E49" s="22">
         <v>18</v>
@@ -11649,7 +12072,7 @@
         <v>18</v>
       </c>
       <c r="H49" s="38" t="s">
-        <v>221</v>
+        <v>255</v>
       </c>
     </row>
     <row r="50" spans="2:8" ht="19" customHeight="1">
@@ -11672,7 +12095,7 @@
         <v>1500</v>
       </c>
       <c r="H50" s="40" t="s">
-        <v>222</v>
+        <v>256</v>
       </c>
     </row>
     <row r="51" spans="2:8" ht="19" customHeight="1">
@@ -11680,10 +12103,10 @@
         <v>46300</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="D51" s="33" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="E51" s="22">
         <v>10</v>
@@ -11695,7 +12118,7 @@
         <v>10</v>
       </c>
       <c r="H51" s="38" t="s">
-        <v>223</v>
+        <v>257</v>
       </c>
     </row>
     <row r="52" spans="2:8" ht="19" customHeight="1">
@@ -11703,10 +12126,10 @@
         <v>46301</v>
       </c>
       <c r="C52" s="34" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D52" s="34" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="E52" s="25">
         <v>1270</v>
@@ -11718,7 +12141,7 @@
         <v>1270</v>
       </c>
       <c r="H52" s="40" t="s">
-        <v>224</v>
+        <v>258</v>
       </c>
     </row>
     <row r="53" spans="2:8" ht="19" customHeight="1">
@@ -11726,10 +12149,10 @@
         <v>46301</v>
       </c>
       <c r="C53" s="33" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D53" s="33" t="s">
-        <v>196</v>
+        <v>230</v>
       </c>
       <c r="E53" s="22">
         <v>50</v>
@@ -11741,7 +12164,7 @@
         <v>50</v>
       </c>
       <c r="H53" s="38" t="s">
-        <v>225</v>
+        <v>259</v>
       </c>
     </row>
     <row r="54" spans="2:8" ht="19" customHeight="1">
@@ -11749,10 +12172,10 @@
         <v>46303</v>
       </c>
       <c r="C54" s="34" t="s">
-        <v>150</v>
+        <v>186</v>
       </c>
       <c r="D54" s="34" t="s">
-        <v>226</v>
+        <v>260</v>
       </c>
       <c r="E54" s="25">
         <v>141</v>
@@ -11764,7 +12187,7 @@
         <v>141</v>
       </c>
       <c r="H54" s="40" t="s">
-        <v>227</v>
+        <v>261</v>
       </c>
     </row>
     <row r="55" spans="2:8" ht="19" customHeight="1">
@@ -11772,10 +12195,10 @@
         <v>46303</v>
       </c>
       <c r="C55" s="33" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D55" s="33" t="s">
-        <v>196</v>
+        <v>230</v>
       </c>
       <c r="E55" s="22">
         <v>125</v>
@@ -11787,7 +12210,7 @@
         <v>125</v>
       </c>
       <c r="H55" s="38" t="s">
-        <v>228</v>
+        <v>262</v>
       </c>
     </row>
     <row r="56" spans="2:8" ht="19" customHeight="1">
@@ -11795,10 +12218,10 @@
         <v>46303</v>
       </c>
       <c r="C56" s="34" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D56" s="34" t="s">
-        <v>196</v>
+        <v>230</v>
       </c>
       <c r="E56" s="25">
         <v>75</v>
@@ -11810,7 +12233,7 @@
         <v>75</v>
       </c>
       <c r="H56" s="40" t="s">
-        <v>229</v>
+        <v>263</v>
       </c>
     </row>
     <row r="57" spans="2:8" ht="19" customHeight="1">
@@ -11818,10 +12241,10 @@
         <v>46303</v>
       </c>
       <c r="C57" s="33" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D57" s="33" t="s">
-        <v>196</v>
+        <v>230</v>
       </c>
       <c r="E57" s="22">
         <v>40</v>
@@ -11833,7 +12256,7 @@
         <v>40</v>
       </c>
       <c r="H57" s="38" t="s">
-        <v>230</v>
+        <v>264</v>
       </c>
     </row>
     <row r="58" spans="2:8" ht="19" customHeight="1">
@@ -11841,10 +12264,10 @@
         <v>46303</v>
       </c>
       <c r="C58" s="34" t="s">
-        <v>148</v>
+        <v>184</v>
       </c>
       <c r="D58" s="34" t="s">
-        <v>217</v>
+        <v>251</v>
       </c>
       <c r="E58" s="25">
         <v>40</v>
@@ -11856,7 +12279,7 @@
         <v>40</v>
       </c>
       <c r="H58" s="40" t="s">
-        <v>231</v>
+        <v>265</v>
       </c>
     </row>
     <row r="59" spans="2:8" ht="19" customHeight="1">
@@ -11864,10 +12287,10 @@
         <v>46304</v>
       </c>
       <c r="C59" s="33" t="s">
-        <v>146</v>
+        <v>182</v>
       </c>
       <c r="D59" s="33" t="s">
-        <v>167</v>
+        <v>201</v>
       </c>
       <c r="E59" s="22">
         <v>11</v>
@@ -11879,7 +12302,7 @@
         <v>11</v>
       </c>
       <c r="H59" s="38" t="s">
-        <v>232</v>
+        <v>266</v>
       </c>
     </row>
     <row r="60" spans="2:8" ht="19" customHeight="1">
@@ -11887,10 +12310,10 @@
         <v>46305</v>
       </c>
       <c r="C60" s="34" t="s">
-        <v>147</v>
+        <v>183</v>
       </c>
       <c r="D60" s="34" t="s">
-        <v>233</v>
+        <v>267</v>
       </c>
       <c r="E60" s="25">
         <v>70</v>
@@ -11902,7 +12325,7 @@
         <v>30</v>
       </c>
       <c r="H60" s="40" t="s">
-        <v>234</v>
+        <v>268</v>
       </c>
     </row>
     <row r="61" spans="2:8" ht="19" customHeight="1">
@@ -11910,10 +12333,10 @@
         <v>46305</v>
       </c>
       <c r="C61" s="33" t="s">
-        <v>151</v>
+        <v>187</v>
       </c>
       <c r="D61" s="33" t="s">
-        <v>235</v>
+        <v>269</v>
       </c>
       <c r="E61" s="22">
         <v>29</v>
@@ -11925,7 +12348,7 @@
         <v>30</v>
       </c>
       <c r="H61" s="38" t="s">
-        <v>236</v>
+        <v>270</v>
       </c>
     </row>
     <row r="62" spans="2:8" ht="19" customHeight="1">
@@ -11933,10 +12356,10 @@
         <v>46307</v>
       </c>
       <c r="C62" s="34" t="s">
-        <v>148</v>
+        <v>184</v>
       </c>
       <c r="D62" s="34" t="s">
-        <v>217</v>
+        <v>251</v>
       </c>
       <c r="E62" s="25">
         <v>22</v>
@@ -11948,7 +12371,7 @@
         <v>22</v>
       </c>
       <c r="H62" s="40" t="s">
-        <v>237</v>
+        <v>271</v>
       </c>
     </row>
     <row r="63" spans="2:8" ht="19" customHeight="1">
@@ -11956,10 +12379,10 @@
         <v>46307</v>
       </c>
       <c r="C63" s="33" t="s">
-        <v>158</v>
+        <v>192</v>
       </c>
       <c r="D63" s="33" t="s">
-        <v>238</v>
+        <v>272</v>
       </c>
       <c r="E63" s="22">
         <v>6</v>
@@ -11971,7 +12394,7 @@
         <v>1</v>
       </c>
       <c r="H63" s="38" t="s">
-        <v>239</v>
+        <v>273</v>
       </c>
     </row>
     <row r="64" spans="2:8" ht="19" customHeight="1">
@@ -11979,10 +12402,10 @@
         <v>46308</v>
       </c>
       <c r="C64" s="34" t="s">
-        <v>153</v>
+        <v>102</v>
       </c>
       <c r="D64" s="34" t="s">
-        <v>240</v>
+        <v>103</v>
       </c>
       <c r="E64" s="25">
         <v>64</v>
@@ -11994,7 +12417,7 @@
         <v>32</v>
       </c>
       <c r="H64" s="40" t="s">
-        <v>241</v>
+        <v>274</v>
       </c>
     </row>
     <row r="65" spans="2:8" ht="19" customHeight="1">
@@ -12002,10 +12425,10 @@
         <v>46308</v>
       </c>
       <c r="C65" s="33" t="s">
-        <v>154</v>
+        <v>189</v>
       </c>
       <c r="D65" s="33" t="s">
-        <v>242</v>
+        <v>275</v>
       </c>
       <c r="E65" s="22">
         <v>24</v>
@@ -12017,7 +12440,7 @@
         <v>6</v>
       </c>
       <c r="H65" s="38" t="s">
-        <v>243</v>
+        <v>276</v>
       </c>
     </row>
     <row r="66" spans="2:8" ht="19" customHeight="1">
@@ -12025,10 +12448,10 @@
         <v>46309</v>
       </c>
       <c r="C66" s="34" t="s">
-        <v>148</v>
+        <v>184</v>
       </c>
       <c r="D66" s="34" t="s">
-        <v>217</v>
+        <v>251</v>
       </c>
       <c r="E66" s="25">
         <v>135</v>
@@ -12040,7 +12463,7 @@
         <v>135</v>
       </c>
       <c r="H66" s="40" t="s">
-        <v>244</v>
+        <v>277</v>
       </c>
     </row>
     <row r="67" spans="2:8" ht="19" customHeight="1">
@@ -12051,7 +12474,7 @@
         <v>28</v>
       </c>
       <c r="D67" s="33" t="s">
-        <v>245</v>
+        <v>278</v>
       </c>
       <c r="E67" s="22">
         <v>7</v>
@@ -12063,7 +12486,7 @@
         <v>7</v>
       </c>
       <c r="H67" s="38" t="s">
-        <v>246</v>
+        <v>279</v>
       </c>
     </row>
     <row r="68" spans="2:8" ht="19" customHeight="1">
@@ -12071,10 +12494,10 @@
         <v>46311</v>
       </c>
       <c r="C68" s="34" t="s">
-        <v>147</v>
+        <v>183</v>
       </c>
       <c r="D68" s="34" t="s">
-        <v>247</v>
+        <v>280</v>
       </c>
       <c r="E68" s="25">
         <v>200</v>
@@ -12086,7 +12509,7 @@
         <v>200</v>
       </c>
       <c r="H68" s="40" t="s">
-        <v>248</v>
+        <v>281</v>
       </c>
     </row>
     <row r="69" spans="2:8" ht="19" customHeight="1">
@@ -12094,10 +12517,10 @@
         <v>46311</v>
       </c>
       <c r="C69" s="33" t="s">
-        <v>155</v>
+        <v>190</v>
       </c>
       <c r="D69" s="33" t="s">
-        <v>249</v>
+        <v>282</v>
       </c>
       <c r="E69" s="22">
         <v>44</v>
@@ -12109,7 +12532,7 @@
         <v>44</v>
       </c>
       <c r="H69" s="38" t="s">
-        <v>250</v>
+        <v>283</v>
       </c>
     </row>
     <row r="70" spans="2:8" ht="19" customHeight="1">
@@ -12117,10 +12540,10 @@
         <v>46311</v>
       </c>
       <c r="C70" s="34" t="s">
-        <v>146</v>
+        <v>182</v>
       </c>
       <c r="D70" s="34" t="s">
-        <v>167</v>
+        <v>201</v>
       </c>
       <c r="E70" s="25">
         <v>30</v>
@@ -12132,7 +12555,7 @@
         <v>30</v>
       </c>
       <c r="H70" s="40" t="s">
-        <v>251</v>
+        <v>284</v>
       </c>
     </row>
     <row r="71" spans="2:8" ht="19" customHeight="1">
@@ -12140,10 +12563,10 @@
         <v>46311</v>
       </c>
       <c r="C71" s="33" t="s">
-        <v>160</v>
+        <v>194</v>
       </c>
       <c r="D71" s="33" t="s">
-        <v>252</v>
+        <v>285</v>
       </c>
       <c r="E71" s="22">
         <v>4</v>
@@ -12155,7 +12578,7 @@
         <v>4</v>
       </c>
       <c r="H71" s="38" t="s">
-        <v>253</v>
+        <v>286</v>
       </c>
     </row>
     <row r="72" spans="2:8" ht="19" customHeight="1">
@@ -12163,10 +12586,10 @@
         <v>46311</v>
       </c>
       <c r="C72" s="34" t="s">
-        <v>160</v>
+        <v>194</v>
       </c>
       <c r="D72" s="34" t="s">
-        <v>160</v>
+        <v>194</v>
       </c>
       <c r="E72" s="25">
         <v>3</v>
@@ -12178,7 +12601,7 @@
         <v>3</v>
       </c>
       <c r="H72" s="40" t="s">
-        <v>254</v>
+        <v>287</v>
       </c>
     </row>
     <row r="73" spans="2:8" ht="19" customHeight="1">
@@ -12186,10 +12609,10 @@
         <v>46312</v>
       </c>
       <c r="C73" s="33" t="s">
-        <v>151</v>
+        <v>187</v>
       </c>
       <c r="D73" s="33" t="s">
-        <v>255</v>
+        <v>288</v>
       </c>
       <c r="E73" s="22">
         <v>20</v>
@@ -12201,7 +12624,7 @@
         <v>20</v>
       </c>
       <c r="H73" s="38" t="s">
-        <v>256</v>
+        <v>289</v>
       </c>
     </row>
     <row r="74" spans="2:8" ht="19" customHeight="1">
@@ -12209,10 +12632,10 @@
         <v>46314</v>
       </c>
       <c r="C74" s="34" t="s">
-        <v>154</v>
+        <v>189</v>
       </c>
       <c r="D74" s="34" t="s">
-        <v>257</v>
+        <v>290</v>
       </c>
       <c r="E74" s="25">
         <v>36</v>
@@ -12224,7 +12647,7 @@
         <v>9</v>
       </c>
       <c r="H74" s="40" t="s">
-        <v>258</v>
+        <v>291</v>
       </c>
     </row>
     <row r="75" spans="2:8" ht="19" customHeight="1">
@@ -12247,7 +12670,7 @@
         <v>1000</v>
       </c>
       <c r="H75" s="38" t="s">
-        <v>259</v>
+        <v>292</v>
       </c>
     </row>
     <row r="76" spans="2:8" ht="19" customHeight="1">
@@ -12258,7 +12681,7 @@
         <v>27</v>
       </c>
       <c r="D76" s="34" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="E76" s="25">
         <v>800</v>
@@ -12270,7 +12693,7 @@
         <v>800</v>
       </c>
       <c r="H76" s="40" t="s">
-        <v>260</v>
+        <v>293</v>
       </c>
     </row>
     <row r="77" spans="2:8" ht="19" customHeight="1">
@@ -12281,7 +12704,7 @@
         <v>27</v>
       </c>
       <c r="D77" s="33" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="E77" s="22">
         <v>300</v>
@@ -12293,7 +12716,7 @@
         <v>300</v>
       </c>
       <c r="H77" s="38" t="s">
-        <v>261</v>
+        <v>294</v>
       </c>
     </row>
     <row r="78" spans="2:8" ht="19" customHeight="1">
@@ -12301,10 +12724,10 @@
         <v>46315</v>
       </c>
       <c r="C78" s="34" t="s">
-        <v>148</v>
+        <v>184</v>
       </c>
       <c r="D78" s="34" t="s">
-        <v>217</v>
+        <v>251</v>
       </c>
       <c r="E78" s="25">
         <v>216</v>
@@ -12316,7 +12739,7 @@
         <v>216</v>
       </c>
       <c r="H78" s="40" t="s">
-        <v>262</v>
+        <v>295</v>
       </c>
     </row>
     <row r="79" spans="2:8" ht="19" customHeight="1">
@@ -12324,10 +12747,10 @@
         <v>46316</v>
       </c>
       <c r="C79" s="33" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D79" s="33" t="s">
-        <v>263</v>
+        <v>155</v>
       </c>
       <c r="E79" s="22">
         <v>17</v>
@@ -12339,7 +12762,7 @@
         <v>17</v>
       </c>
       <c r="H79" s="38" t="s">
-        <v>264</v>
+        <v>296</v>
       </c>
     </row>
     <row r="80" spans="2:8" ht="19" customHeight="1">
@@ -12347,10 +12770,10 @@
         <v>46316</v>
       </c>
       <c r="C80" s="34" t="s">
-        <v>158</v>
+        <v>192</v>
       </c>
       <c r="D80" s="34" t="s">
-        <v>265</v>
+        <v>297</v>
       </c>
       <c r="E80" s="25">
         <v>5</v>
@@ -12362,7 +12785,7 @@
         <v>1</v>
       </c>
       <c r="H80" s="40" t="s">
-        <v>266</v>
+        <v>298</v>
       </c>
     </row>
     <row r="81" spans="2:8" ht="19" customHeight="1">
@@ -12370,10 +12793,10 @@
         <v>46316</v>
       </c>
       <c r="C81" s="33" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D81" s="33" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E81" s="22">
         <v>3</v>
@@ -12385,7 +12808,7 @@
         <v>5</v>
       </c>
       <c r="H81" s="38" t="s">
-        <v>267</v>
+        <v>299</v>
       </c>
     </row>
     <row r="82" spans="2:8" ht="19" customHeight="1">
@@ -12393,10 +12816,10 @@
         <v>46317</v>
       </c>
       <c r="C82" s="34" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="D82" s="34" t="s">
-        <v>176</v>
+        <v>210</v>
       </c>
       <c r="E82" s="25">
         <v>11</v>
@@ -12408,7 +12831,7 @@
         <v>1</v>
       </c>
       <c r="H82" s="40" t="s">
-        <v>268</v>
+        <v>300</v>
       </c>
     </row>
     <row r="83" spans="2:8" ht="19" customHeight="1">
@@ -12431,7 +12854,7 @@
         <v>3</v>
       </c>
       <c r="H83" s="38" t="s">
-        <v>269</v>
+        <v>301</v>
       </c>
     </row>
     <row r="84" spans="2:8" ht="19" customHeight="1">
@@ -12442,7 +12865,7 @@
         <v>27</v>
       </c>
       <c r="D84" s="34" t="s">
-        <v>192</v>
+        <v>226</v>
       </c>
       <c r="E84" s="25">
         <v>250</v>
@@ -12454,7 +12877,7 @@
         <v>250</v>
       </c>
       <c r="H84" s="40" t="s">
-        <v>270</v>
+        <v>302</v>
       </c>
     </row>
     <row r="85" spans="2:8" ht="19" customHeight="1">
@@ -12462,10 +12885,10 @@
         <v>46319</v>
       </c>
       <c r="C85" s="33" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D85" s="33" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="E85" s="22">
         <v>150</v>
@@ -12477,7 +12900,7 @@
         <v>150</v>
       </c>
       <c r="H85" s="38" t="s">
-        <v>271</v>
+        <v>303</v>
       </c>
     </row>
     <row r="86" spans="2:8" ht="19" customHeight="1">
@@ -12485,10 +12908,10 @@
         <v>46319</v>
       </c>
       <c r="C86" s="34" t="s">
-        <v>147</v>
+        <v>183</v>
       </c>
       <c r="D86" s="34" t="s">
-        <v>233</v>
+        <v>267</v>
       </c>
       <c r="E86" s="25">
         <v>100</v>
@@ -12500,7 +12923,7 @@
         <v>35</v>
       </c>
       <c r="H86" s="40" t="s">
-        <v>272</v>
+        <v>304</v>
       </c>
     </row>
     <row r="87" spans="2:8" ht="19" customHeight="1">
@@ -12511,7 +12934,7 @@
         <v>27</v>
       </c>
       <c r="D87" s="33" t="s">
-        <v>273</v>
+        <v>305</v>
       </c>
       <c r="E87" s="22">
         <v>100</v>
@@ -12523,7 +12946,7 @@
         <v>100</v>
       </c>
       <c r="H87" s="38" t="s">
-        <v>274</v>
+        <v>306</v>
       </c>
     </row>
     <row r="88" spans="2:8" ht="19" customHeight="1">
@@ -12531,10 +12954,10 @@
         <v>46319</v>
       </c>
       <c r="C88" s="34" t="s">
-        <v>147</v>
+        <v>183</v>
       </c>
       <c r="D88" s="34" t="s">
-        <v>233</v>
+        <v>267</v>
       </c>
       <c r="E88" s="25">
         <v>97</v>
@@ -12546,7 +12969,7 @@
         <v>30</v>
       </c>
       <c r="H88" s="40" t="s">
-        <v>275</v>
+        <v>307</v>
       </c>
     </row>
     <row r="89" spans="2:8" ht="19" customHeight="1">
@@ -12569,7 +12992,7 @@
         <v>66</v>
       </c>
       <c r="H89" s="38" t="s">
-        <v>276</v>
+        <v>308</v>
       </c>
     </row>
     <row r="90" spans="2:8" ht="19" customHeight="1">
@@ -12577,10 +13000,10 @@
         <v>46319</v>
       </c>
       <c r="C90" s="34" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="D90" s="34" t="s">
-        <v>277</v>
+        <v>162</v>
       </c>
       <c r="E90" s="25">
         <v>30</v>
@@ -12592,7 +13015,7 @@
         <v>20</v>
       </c>
       <c r="H90" s="40" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
     </row>
     <row r="91" spans="2:8" ht="19" customHeight="1">
@@ -12600,10 +13023,10 @@
         <v>46319</v>
       </c>
       <c r="C91" s="33" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="D91" s="33" t="s">
-        <v>277</v>
+        <v>162</v>
       </c>
       <c r="E91" s="22">
         <v>25</v>
@@ -12615,7 +13038,7 @@
         <v>20</v>
       </c>
       <c r="H91" s="38" t="s">
-        <v>279</v>
+        <v>310</v>
       </c>
     </row>
     <row r="92" spans="2:8" ht="19" customHeight="1">
@@ -12623,10 +13046,10 @@
         <v>46319</v>
       </c>
       <c r="C92" s="34" t="s">
-        <v>151</v>
+        <v>187</v>
       </c>
       <c r="D92" s="34" t="s">
-        <v>280</v>
+        <v>311</v>
       </c>
       <c r="E92" s="25">
         <v>15</v>
@@ -12638,7 +13061,7 @@
         <v>15</v>
       </c>
       <c r="H92" s="40" t="s">
-        <v>281</v>
+        <v>312</v>
       </c>
     </row>
     <row r="93" spans="2:8" ht="19" customHeight="1">
@@ -12646,10 +13069,10 @@
         <v>46320</v>
       </c>
       <c r="C93" s="33" t="s">
-        <v>151</v>
+        <v>187</v>
       </c>
       <c r="D93" s="33" t="s">
-        <v>151</v>
+        <v>187</v>
       </c>
       <c r="E93" s="22">
         <v>15</v>
@@ -12661,7 +13084,7 @@
         <v>15</v>
       </c>
       <c r="H93" s="38" t="s">
-        <v>282</v>
+        <v>313</v>
       </c>
     </row>
     <row r="94" spans="2:8" ht="19" customHeight="1">
@@ -12669,10 +13092,10 @@
         <v>46320</v>
       </c>
       <c r="C94" s="34" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="D94" s="34" t="s">
-        <v>180</v>
+        <v>214</v>
       </c>
       <c r="E94" s="25">
         <v>2</v>
@@ -12684,7 +13107,7 @@
         <v>1</v>
       </c>
       <c r="H94" s="40" t="s">
-        <v>283</v>
+        <v>314</v>
       </c>
     </row>
     <row r="95" spans="2:8" ht="19" customHeight="1">
@@ -12692,10 +13115,10 @@
         <v>46320</v>
       </c>
       <c r="C95" s="33" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="D95" s="33" t="s">
-        <v>180</v>
+        <v>214</v>
       </c>
       <c r="E95" s="22">
         <v>1</v>
@@ -12707,7 +13130,7 @@
         <v>1</v>
       </c>
       <c r="H95" s="38" t="s">
-        <v>284</v>
+        <v>315</v>
       </c>
     </row>
     <row r="96" spans="2:8" ht="19" customHeight="1">
@@ -12715,10 +13138,10 @@
         <v>46320</v>
       </c>
       <c r="C96" s="34" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="D96" s="34" t="s">
-        <v>180</v>
+        <v>214</v>
       </c>
       <c r="E96" s="25">
         <v>1</v>
@@ -12730,7 +13153,7 @@
         <v>1</v>
       </c>
       <c r="H96" s="40" t="s">
-        <v>285</v>
+        <v>316</v>
       </c>
     </row>
     <row r="97" spans="2:8" ht="19" customHeight="1">
@@ -12738,10 +13161,10 @@
         <v>46320</v>
       </c>
       <c r="C97" s="33" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="D97" s="33" t="s">
-        <v>180</v>
+        <v>214</v>
       </c>
       <c r="E97" s="22">
         <v>1</v>
@@ -12753,7 +13176,7 @@
         <v>1</v>
       </c>
       <c r="H97" s="38" t="s">
-        <v>286</v>
+        <v>317</v>
       </c>
     </row>
     <row r="98" spans="2:8" ht="19" customHeight="1">
@@ -12761,10 +13184,10 @@
         <v>46320</v>
       </c>
       <c r="C98" s="34" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="D98" s="34" t="s">
-        <v>180</v>
+        <v>214</v>
       </c>
       <c r="E98" s="25">
         <v>1</v>
@@ -12776,7 +13199,7 @@
         <v>1</v>
       </c>
       <c r="H98" s="40" t="s">
-        <v>287</v>
+        <v>318</v>
       </c>
     </row>
     <row r="99" spans="2:8" ht="19" customHeight="1">
@@ -12784,10 +13207,10 @@
         <v>46321</v>
       </c>
       <c r="C99" s="33" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="D99" s="33" t="s">
-        <v>219</v>
+        <v>253</v>
       </c>
       <c r="E99" s="22">
         <v>225</v>
@@ -12799,7 +13222,7 @@
         <v>225</v>
       </c>
       <c r="H99" s="38" t="s">
-        <v>288</v>
+        <v>319</v>
       </c>
     </row>
     <row r="100" spans="2:8" ht="22" customHeight="1">
@@ -12863,7 +13286,7 @@
     <row r="2" spans="1:7" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>289</v>
+        <v>320</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -12904,13 +13327,13 @@
     </row>
     <row r="7" spans="1:7" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>290</v>
+        <v>321</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="F7" s="8" t="s">
-        <v>291</v>
+        <v>322</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="36" customHeight="1">
@@ -12918,21 +13341,21 @@
         <v>25</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>292</v>
+        <v>323</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>293</v>
+        <v>324</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>294</v>
+        <v>325</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>295</v>
+        <v>326</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="19" customHeight="1">
       <c r="B9" s="21" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="C9" s="45">
         <v>0</v>
@@ -12983,7 +13406,7 @@
     </row>
     <row r="12" spans="1:7" ht="19" customHeight="1">
       <c r="B12" s="24" t="s">
-        <v>153</v>
+        <v>102</v>
       </c>
       <c r="C12" s="47">
         <v>0</v>
@@ -13000,7 +13423,7 @@
     </row>
     <row r="13" spans="1:7" ht="19" customHeight="1">
       <c r="B13" s="21" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="C13" s="45">
         <v>45</v>
@@ -13017,7 +13440,7 @@
     </row>
     <row r="14" spans="1:7" ht="19" customHeight="1">
       <c r="B14" s="24" t="s">
-        <v>148</v>
+        <v>184</v>
       </c>
       <c r="C14" s="47">
         <v>0</v>
@@ -13034,7 +13457,7 @@
     </row>
     <row r="15" spans="1:7" ht="19" customHeight="1">
       <c r="B15" s="21" t="s">
-        <v>147</v>
+        <v>183</v>
       </c>
       <c r="C15" s="45">
         <v>1</v>
@@ -13072,18 +13495,18 @@
     </row>
     <row r="33" spans="2:6" ht="27" customHeight="1">
       <c r="B33" s="6" t="s">
-        <v>296</v>
+        <v>327</v>
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
       <c r="E33" s="7"/>
       <c r="F33" s="8" t="s">
-        <v>297</v>
+        <v>328</v>
       </c>
     </row>
     <row r="34" spans="2:6" ht="30" customHeight="1">
       <c r="B34" s="51" t="s">
-        <v>298</v>
+        <v>329</v>
       </c>
       <c r="C34" s="51"/>
       <c r="D34" s="52">
@@ -13094,7 +13517,7 @@
     </row>
     <row r="35" spans="2:6" ht="30" customHeight="1">
       <c r="B35" s="51" t="s">
-        <v>299</v>
+        <v>330</v>
       </c>
       <c r="C35" s="51"/>
       <c r="D35" s="52">
@@ -13105,7 +13528,7 @@
     </row>
     <row r="36" spans="2:6" ht="30" customHeight="1">
       <c r="B36" s="51" t="s">
-        <v>300</v>
+        <v>331</v>
       </c>
       <c r="C36" s="51"/>
       <c r="D36" s="54">
@@ -13166,7 +13589,7 @@
     <row r="2" spans="1:9" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>301</v>
+        <v>332</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -13215,7 +13638,7 @@
     </row>
     <row r="7" spans="1:9" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>302</v>
+        <v>333</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -13223,7 +13646,7 @@
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="8" t="s">
-        <v>303</v>
+        <v>334</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="36" customHeight="1">
@@ -13231,30 +13654,30 @@
         <v>25</v>
       </c>
       <c r="C8" s="32" t="s">
-        <v>304</v>
+        <v>335</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>142</v>
+        <v>179</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>305</v>
+        <v>336</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>294</v>
+        <v>325</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>293</v>
+        <v>324</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>295</v>
+        <v>326</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="21" customHeight="1">
       <c r="B9" s="21" t="s">
-        <v>147</v>
+        <v>183</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>306</v>
+        <v>337</v>
       </c>
       <c r="D9" s="45">
         <v>527</v>
@@ -13274,10 +13697,10 @@
     </row>
     <row r="10" spans="1:9" ht="21" customHeight="1">
       <c r="B10" s="24" t="s">
-        <v>150</v>
+        <v>186</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>226</v>
+        <v>260</v>
       </c>
       <c r="D10" s="47">
         <v>141</v>
@@ -13297,10 +13720,10 @@
     </row>
     <row r="11" spans="1:9" ht="21" customHeight="1">
       <c r="B11" s="21" t="s">
-        <v>146</v>
+        <v>182</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>307</v>
+        <v>338</v>
       </c>
       <c r="D11" s="45">
         <v>780</v>
@@ -13320,10 +13743,10 @@
     </row>
     <row r="12" spans="1:9" ht="21" customHeight="1">
       <c r="B12" s="24" t="s">
-        <v>159</v>
+        <v>193</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>204</v>
+        <v>238</v>
       </c>
       <c r="D12" s="47">
         <v>7</v>
@@ -13343,10 +13766,10 @@
     </row>
     <row r="13" spans="1:9" ht="21" customHeight="1">
       <c r="B13" s="21" t="s">
-        <v>149</v>
+        <v>185</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>172</v>
+        <v>206</v>
       </c>
       <c r="D13" s="45">
         <v>250</v>
@@ -13369,7 +13792,7 @@
         <v>26</v>
       </c>
       <c r="C14" s="34" t="s">
-        <v>308</v>
+        <v>339</v>
       </c>
       <c r="D14" s="47">
         <v>66</v>
@@ -13387,12 +13810,12 @@
         <v>55022.19</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="21" customHeight="1">
+    <row r="15" spans="1:9" ht="35" customHeight="1">
       <c r="B15" s="21" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>309</v>
+        <v>340</v>
       </c>
       <c r="D15" s="45">
         <v>3820</v>
@@ -13415,7 +13838,7 @@
         <v>27</v>
       </c>
       <c r="C16" s="34" t="s">
-        <v>310</v>
+        <v>341</v>
       </c>
       <c r="D16" s="47">
         <v>6850</v>
@@ -13435,10 +13858,10 @@
     </row>
     <row r="17" spans="2:8" ht="21" customHeight="1">
       <c r="B17" s="21" t="s">
-        <v>148</v>
+        <v>184</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>217</v>
+        <v>251</v>
       </c>
       <c r="D17" s="45">
         <v>498</v>
@@ -13458,10 +13881,10 @@
     </row>
     <row r="18" spans="2:8" ht="21" customHeight="1">
       <c r="B18" s="24" t="s">
-        <v>151</v>
+        <v>187</v>
       </c>
       <c r="C18" s="34" t="s">
-        <v>311</v>
+        <v>342</v>
       </c>
       <c r="D18" s="47">
         <v>79</v>
@@ -13481,10 +13904,10 @@
     </row>
     <row r="19" spans="2:8" ht="21" customHeight="1">
       <c r="B19" s="21" t="s">
-        <v>153</v>
+        <v>102</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>240</v>
+        <v>103</v>
       </c>
       <c r="D19" s="45">
         <v>64</v>
@@ -13502,12 +13925,12 @@
         <v>33033.06</v>
       </c>
     </row>
-    <row r="20" spans="2:8" ht="21" customHeight="1">
+    <row r="20" spans="2:8" ht="35" customHeight="1">
       <c r="B20" s="24" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="C20" s="34" t="s">
-        <v>312</v>
+        <v>343</v>
       </c>
       <c r="D20" s="47">
         <v>75</v>
@@ -13527,10 +13950,10 @@
     </row>
     <row r="21" spans="2:8" ht="21" customHeight="1">
       <c r="B21" s="21" t="s">
-        <v>154</v>
+        <v>189</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>313</v>
+        <v>344</v>
       </c>
       <c r="D21" s="45">
         <v>60</v>
@@ -13550,10 +13973,10 @@
     </row>
     <row r="22" spans="2:8" ht="21" customHeight="1">
       <c r="B22" s="24" t="s">
-        <v>160</v>
+        <v>194</v>
       </c>
       <c r="C22" s="34" t="s">
-        <v>314</v>
+        <v>345</v>
       </c>
       <c r="D22" s="47">
         <v>7</v>
@@ -13573,10 +13996,10 @@
     </row>
     <row r="23" spans="2:8" ht="35" customHeight="1">
       <c r="B23" s="21" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>315</v>
+        <v>346</v>
       </c>
       <c r="D23" s="45">
         <v>64</v>
@@ -13599,7 +14022,7 @@
         <v>28</v>
       </c>
       <c r="C24" s="34" t="s">
-        <v>316</v>
+        <v>347</v>
       </c>
       <c r="D24" s="47">
         <v>13</v>
@@ -13619,10 +14042,10 @@
     </row>
     <row r="25" spans="2:8" ht="21" customHeight="1">
       <c r="B25" s="21" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>263</v>
+        <v>155</v>
       </c>
       <c r="D25" s="45">
         <v>17</v>
@@ -13642,10 +14065,10 @@
     </row>
     <row r="26" spans="2:8" ht="21" customHeight="1">
       <c r="B26" s="24" t="s">
-        <v>155</v>
+        <v>190</v>
       </c>
       <c r="C26" s="34" t="s">
-        <v>249</v>
+        <v>282</v>
       </c>
       <c r="D26" s="47">
         <v>44</v>
@@ -13665,10 +14088,10 @@
     </row>
     <row r="27" spans="2:8" ht="21" customHeight="1">
       <c r="B27" s="21" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="D27" s="45">
         <v>17</v>
@@ -13688,10 +14111,10 @@
     </row>
     <row r="28" spans="2:8" ht="21" customHeight="1">
       <c r="B28" s="24" t="s">
-        <v>158</v>
+        <v>192</v>
       </c>
       <c r="C28" s="34" t="s">
-        <v>317</v>
+        <v>348</v>
       </c>
       <c r="D28" s="47">
         <v>11</v>
@@ -13772,7 +14195,7 @@
     <row r="2" spans="1:4" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>318</v>
+        <v>349</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -13801,7 +14224,7 @@
     </row>
     <row r="6" spans="1:4" ht="32" customHeight="1">
       <c r="B6" s="55" t="s">
-        <v>319</v>
+        <v>350</v>
       </c>
       <c r="C6" s="56" t="s">
         <v>4</v>
@@ -13809,31 +14232,31 @@
     </row>
     <row r="7" spans="1:4" ht="32" customHeight="1">
       <c r="B7" s="55" t="s">
-        <v>320</v>
+        <v>351</v>
       </c>
       <c r="C7" s="56" t="s">
-        <v>321</v>
+        <v>352</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="32" customHeight="1">
       <c r="B8" s="55" t="s">
-        <v>322</v>
+        <v>353</v>
       </c>
       <c r="C8" s="56" t="s">
-        <v>323</v>
+        <v>354</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="42" customHeight="1">
       <c r="B9" s="55" t="s">
-        <v>324</v>
+        <v>355</v>
       </c>
       <c r="C9" s="56" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="42" customHeight="1">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="32" customHeight="1">
       <c r="B10" s="55" t="s">
-        <v>326</v>
+        <v>357</v>
       </c>
       <c r="C10" s="56" t="s">
         <v>33</v>
@@ -13841,50 +14264,50 @@
     </row>
     <row r="11" spans="1:4" ht="32" customHeight="1">
       <c r="B11" s="55" t="s">
-        <v>327</v>
+        <v>358</v>
       </c>
       <c r="C11" s="57" t="s">
-        <v>328</v>
+        <v>359</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="42" customHeight="1">
       <c r="B12" s="55" t="s">
-        <v>329</v>
+        <v>360</v>
       </c>
       <c r="C12" s="56" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="87" customHeight="1">
+    <row r="13" spans="1:4" ht="102" customHeight="1">
       <c r="B13" s="55" t="s">
-        <v>330</v>
+        <v>361</v>
       </c>
       <c r="C13" s="56" t="s">
-        <v>331</v>
+        <v>362</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="72" customHeight="1">
       <c r="B14" s="55" t="s">
-        <v>142</v>
+        <v>179</v>
       </c>
       <c r="C14" s="56" t="s">
-        <v>164</v>
+        <v>198</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="72" customHeight="1">
       <c r="B15" s="55" t="s">
-        <v>289</v>
+        <v>320</v>
       </c>
       <c r="C15" s="56" t="s">
-        <v>332</v>
+        <v>363</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="57" customHeight="1">
       <c r="B16" s="55" t="s">
-        <v>333</v>
+        <v>364</v>
       </c>
       <c r="C16" s="56" t="s">
-        <v>334</v>
+        <v>365</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajustar el resumen de Riesgos a la estructura aprobada del Plan ENOS
- Página 2 como en el PDF aprobado: nota, las 21 alertas, alertas por provincia y por servicio
  y evolución de las alertas; la tabla toma el mayor tamaño de letra que deja espacio al resto.
- Página 3 solo con la respuesta por provincia, cifras alineadas como en la tabla aprobada.
- Página 1: servicios con sus nombres del boletín aprobado, provincia en negrita en el detalle
  y barras con su separación original.
- Los 6 reportes gerontológicos con fecha de reporte 26/10/2026: la evolución suma las 21 alertas
  (se conserva la redacción de la fuente para trazabilidad).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUCWMWZ6GMzdHUXxvK5iGa
</commit_message>
<xml_diff>
--- a/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
+++ b/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
@@ -31,9 +31,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1466" uniqueCount="506">
-  <si>
-    <t>Riesgos</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="505">
+  <si>
+    <t>Riesgos · Respuesta del Ministerio</t>
   </si>
   <si>
     <t>Del 14/09/2026 al 27/10/2026 · Nacional · Todos los servicios</t>
@@ -639,24 +639,90 @@
     <t>Prioridad</t>
   </si>
   <si>
+    <t>GER-2026-006</t>
+  </si>
+  <si>
+    <t>Santo Domingo de los Tsáchilas</t>
+  </si>
+  <si>
+    <t>Santo Domingo</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Centros gerontológicos</t>
+  </si>
+  <si>
+    <t>Filtraciones y humedad; mitigación inmediata. Servicio operativo.</t>
+  </si>
+  <si>
+    <t>En seguimiento</t>
+  </si>
+  <si>
+    <t>No reportada</t>
+  </si>
+  <si>
+    <t>GER-2026-005</t>
+  </si>
+  <si>
+    <t>Manabí</t>
+  </si>
+  <si>
+    <t>Pedernales</t>
+  </si>
+  <si>
+    <t>Filtraciones y humedad; medidas de contingencia. Servicio operativo.</t>
+  </si>
+  <si>
+    <t>GER-2026-004</t>
+  </si>
+  <si>
+    <t>Portoviejo</t>
+  </si>
+  <si>
+    <t>Filtraciones y humedad; adecuaciones provisionales. Servicio operativo.</t>
+  </si>
+  <si>
+    <t>GER-2026-003</t>
+  </si>
+  <si>
+    <t>Milagro</t>
+  </si>
+  <si>
+    <t>Filtraciones y humedad; medidas preventivas y correctivas. Servicio operativo.</t>
+  </si>
+  <si>
+    <t>GER-2026-002</t>
+  </si>
+  <si>
+    <t>Esmeraldas</t>
+  </si>
+  <si>
+    <t>San Lorenzo</t>
+  </si>
+  <si>
+    <t>Filtraciones y humedad; intervención emergente. Servicio operativo.</t>
+  </si>
+  <si>
+    <t>GER-2026-001</t>
+  </si>
+  <si>
+    <t>Huaquillas</t>
+  </si>
+  <si>
+    <t>Filtraciones en techo y daños en patio; mitigación temporal. Servicio operativo.</t>
+  </si>
+  <si>
     <t>DIS-2026-003</t>
   </si>
   <si>
-    <t>—</t>
-  </si>
-  <si>
     <t>Discapacidades · AHC</t>
   </si>
   <si>
     <t>Inundaciones en viviendas de usuarios; acompañamiento y monitoreo. Servicio operativo.</t>
   </si>
   <si>
-    <t>En seguimiento</t>
-  </si>
-  <si>
-    <t>No reportada</t>
-  </si>
-  <si>
     <t>DIS-2026-002</t>
   </si>
   <si>
@@ -696,9 +762,6 @@
     <t>ALT-2026-000325</t>
   </si>
   <si>
-    <t>Milagro</t>
-  </si>
-  <si>
     <t>62210</t>
   </si>
   <si>
@@ -789,9 +852,6 @@
     <t>ALT-2026-000310</t>
   </si>
   <si>
-    <t>Manabí</t>
-  </si>
-  <si>
     <t>Flavio Alfaro</t>
   </si>
   <si>
@@ -816,69 +876,6 @@
     <t>Correo Infantil</t>
   </si>
   <si>
-    <t>GER-2026-006</t>
-  </si>
-  <si>
-    <t>Agosto 2026 (sin día)</t>
-  </si>
-  <si>
-    <t>Santo Domingo de los Tsáchilas</t>
-  </si>
-  <si>
-    <t>Santo Domingo</t>
-  </si>
-  <si>
-    <t>Centros gerontológicos</t>
-  </si>
-  <si>
-    <t>Filtraciones y humedad; mitigación inmediata. Servicio operativo.</t>
-  </si>
-  <si>
-    <t>GER-2026-005</t>
-  </si>
-  <si>
-    <t>Pedernales</t>
-  </si>
-  <si>
-    <t>Filtraciones y humedad; medidas de contingencia. Servicio operativo.</t>
-  </si>
-  <si>
-    <t>GER-2026-004</t>
-  </si>
-  <si>
-    <t>Portoviejo</t>
-  </si>
-  <si>
-    <t>Filtraciones y humedad; adecuaciones provisionales. Servicio operativo.</t>
-  </si>
-  <si>
-    <t>GER-2026-003</t>
-  </si>
-  <si>
-    <t>Filtraciones y humedad; medidas preventivas y correctivas. Servicio operativo.</t>
-  </si>
-  <si>
-    <t>GER-2026-002</t>
-  </si>
-  <si>
-    <t>Esmeraldas</t>
-  </si>
-  <si>
-    <t>San Lorenzo</t>
-  </si>
-  <si>
-    <t>Filtraciones y humedad; intervención emergente. Servicio operativo.</t>
-  </si>
-  <si>
-    <t>GER-2026-001</t>
-  </si>
-  <si>
-    <t>Huaquillas</t>
-  </si>
-  <si>
-    <t>Filtraciones en techo y daños en patio; mitigación temporal. Servicio operativo.</t>
-  </si>
-  <si>
     <t>Desde el 14/09/2026</t>
   </si>
   <si>
@@ -1539,7 +1536,7 @@
     <t>Alertas</t>
   </si>
   <si>
-    <t>Seguimiento desde el 14/09/2026, complementado con reportes sectoriales de octubre: 10 alertas con código UA y 11 reportes sectoriales. Los 6 reportes gerontológicos describen sucesos de agosto sin día exacto; no se asignan a la evolución diaria. Los identificadores DIS/GER permiten localizar las filas incorporadas, no son códigos oficiales ni códigos UA. Las fuentes sectoriales indican que la prestación del servicio se mantiene. Alertas, unidades y personas son medidas distintas.</t>
+    <t>Seguimiento desde el 14/09/2026, complementado con reportes sectoriales de octubre: 10 alertas con código UA y 11 reportes sectoriales. Los 6 reportes gerontológicos se incorporan con fecha de reporte 26/10/2026. Los identificadores DIS/GER permiten localizar las filas incorporadas, no son códigos oficiales ni códigos UA. Las fuentes sectoriales indican que la prestación del servicio se mantiene. Alertas, unidades y personas son medidas distintas.</t>
   </si>
   <si>
     <t>La ayuda memoria no identifica pagos exclusivamente atribuibles a ENOS ni fechas individuales para recortar desde el 14/09. Se muestran únicamente las filas de inundación como referencia: pagos gestionados desde el 29/08 y casos en articulación al 23/10. Articulación no equivale a pago. Las proyecciones corresponden a planificación nacional 2026–2027.</t>
@@ -2790,7 +2787,7 @@
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>3</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="43">
                   <c:v>0</c:v>
@@ -3095,10 +3092,10 @@
                   <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>15</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>15</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3581,7 +3578,7 @@
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>3</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="43">
                   <c:v>0</c:v>
@@ -3886,10 +3883,10 @@
                   <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>15</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>15</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10973,7 +10970,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="35" customHeight="1">
+    <row r="9" spans="1:12" ht="49" customHeight="1">
       <c r="B9" s="21" t="s">
         <v>202</v>
       </c>
@@ -10981,646 +10978,646 @@
         <v>46321</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>30</v>
+        <v>203</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>47</v>
+        <v>204</v>
       </c>
       <c r="F9" s="38"/>
       <c r="G9" s="33" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="H9" s="33" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I9" s="33" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="J9" s="33" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="K9" s="33" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="35" customHeight="1">
       <c r="B10" s="24" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C10" s="39">
         <v>46321</v>
       </c>
       <c r="D10" s="34" t="s">
-        <v>30</v>
+        <v>211</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="F10" s="40"/>
       <c r="G10" s="34" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="H10" s="34" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I10" s="34" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="J10" s="34" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="K10" s="34" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="35" customHeight="1">
       <c r="B11" s="21" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C11" s="37">
         <v>46321</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>30</v>
+        <v>211</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>51</v>
+        <v>215</v>
       </c>
       <c r="F11" s="38"/>
       <c r="G11" s="33" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="H11" s="33" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I11" s="33" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="J11" s="33" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="K11" s="33" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="35" customHeight="1">
       <c r="B12" s="24" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="C12" s="39">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="D12" s="34" t="s">
-        <v>213</v>
+        <v>31</v>
       </c>
       <c r="E12" s="34" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="F12" s="40"/>
       <c r="G12" s="34" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="H12" s="34" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I12" s="34" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="J12" s="34" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="K12" s="34" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="35" customHeight="1">
       <c r="B13" s="21" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="C13" s="37">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="F13" s="38"/>
       <c r="G13" s="33" t="s">
-        <v>218</v>
+        <v>205</v>
       </c>
       <c r="H13" s="33" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I13" s="33" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J13" s="33" t="s">
+        <v>208</v>
+      </c>
+      <c r="K13" s="33" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="35" customHeight="1">
+      <c r="B14" s="24" t="s">
+        <v>224</v>
+      </c>
+      <c r="C14" s="39">
+        <v>46321</v>
+      </c>
+      <c r="D14" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" s="34" t="s">
+        <v>225</v>
+      </c>
+      <c r="F14" s="40"/>
+      <c r="G14" s="34" t="s">
+        <v>205</v>
+      </c>
+      <c r="H14" s="34" t="s">
         <v>206</v>
       </c>
-      <c r="K13" s="33" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="21" customHeight="1">
-      <c r="B14" s="24" t="s">
-        <v>220</v>
-      </c>
-      <c r="C14" s="39">
-        <v>46315</v>
-      </c>
-      <c r="D14" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="E14" s="34" t="s">
-        <v>221</v>
-      </c>
-      <c r="F14" s="40" t="s">
-        <v>222</v>
-      </c>
-      <c r="G14" s="34" t="s">
-        <v>223</v>
-      </c>
-      <c r="H14" s="34" t="s">
-        <v>224</v>
-      </c>
       <c r="I14" s="34" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J14" s="34" t="s">
-        <v>226</v>
+        <v>208</v>
       </c>
       <c r="K14" s="34" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="35" customHeight="1">
+      <c r="B15" s="21" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" ht="21" customHeight="1">
-      <c r="B15" s="21" t="s">
+      <c r="C15" s="37">
+        <v>46321</v>
+      </c>
+      <c r="D15" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="F15" s="38"/>
+      <c r="G15" s="33" t="s">
+        <v>205</v>
+      </c>
+      <c r="H15" s="33" t="s">
         <v>228</v>
       </c>
-      <c r="C15" s="37">
-        <v>46315</v>
-      </c>
-      <c r="D15" s="33" t="s">
-        <v>31</v>
-      </c>
-      <c r="E15" s="33" t="s">
-        <v>221</v>
-      </c>
-      <c r="F15" s="38" t="s">
+      <c r="I15" s="33" t="s">
         <v>229</v>
       </c>
-      <c r="G15" s="33" t="s">
-        <v>191</v>
-      </c>
-      <c r="H15" s="33" t="s">
-        <v>224</v>
-      </c>
-      <c r="I15" s="33" t="s">
+      <c r="J15" s="33" t="s">
+        <v>208</v>
+      </c>
+      <c r="K15" s="33" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="35" customHeight="1">
+      <c r="B16" s="24" t="s">
         <v>230</v>
       </c>
-      <c r="J15" s="33" t="s">
-        <v>226</v>
-      </c>
-      <c r="K15" s="33" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="21" customHeight="1">
-      <c r="B16" s="24" t="s">
+      <c r="C16" s="39">
+        <v>46321</v>
+      </c>
+      <c r="D16" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" s="34" t="s">
         <v>231</v>
       </c>
-      <c r="C16" s="39">
-        <v>46315</v>
-      </c>
-      <c r="D16" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="E16" s="34" t="s">
-        <v>221</v>
-      </c>
-      <c r="F16" s="40" t="s">
+      <c r="F16" s="40"/>
+      <c r="G16" s="34" t="s">
+        <v>205</v>
+      </c>
+      <c r="H16" s="34" t="s">
+        <v>228</v>
+      </c>
+      <c r="I16" s="34" t="s">
         <v>232</v>
       </c>
-      <c r="G16" s="34" t="s">
+      <c r="J16" s="34" t="s">
+        <v>208</v>
+      </c>
+      <c r="K16" s="34" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" ht="35" customHeight="1">
+      <c r="B17" s="21" t="s">
         <v>233</v>
       </c>
-      <c r="H16" s="34" t="s">
-        <v>224</v>
-      </c>
-      <c r="I16" s="34" t="s">
-        <v>234</v>
-      </c>
-      <c r="J16" s="34" t="s">
-        <v>226</v>
-      </c>
-      <c r="K16" s="34" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="17" spans="2:11" ht="21" customHeight="1">
-      <c r="B17" s="21" t="s">
-        <v>235</v>
-      </c>
       <c r="C17" s="37">
-        <v>46315</v>
+        <v>46321</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>221</v>
-      </c>
-      <c r="F17" s="38" t="s">
-        <v>236</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="F17" s="38"/>
       <c r="G17" s="33" t="s">
-        <v>237</v>
+        <v>205</v>
       </c>
       <c r="H17" s="33" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="I17" s="33" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="J17" s="33" t="s">
-        <v>226</v>
+        <v>208</v>
       </c>
       <c r="K17" s="33" t="s">
-        <v>227</v>
+        <v>209</v>
       </c>
     </row>
     <row r="18" spans="2:11" ht="35" customHeight="1">
       <c r="B18" s="24" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="C18" s="39">
-        <v>46315</v>
+        <v>46320</v>
       </c>
       <c r="D18" s="34" t="s">
-        <v>30</v>
+        <v>235</v>
       </c>
       <c r="E18" s="34" t="s">
-        <v>47</v>
-      </c>
-      <c r="F18" s="40" t="s">
-        <v>240</v>
-      </c>
+        <v>236</v>
+      </c>
+      <c r="F18" s="40"/>
       <c r="G18" s="34" t="s">
-        <v>48</v>
+        <v>237</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="I18" s="34" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="J18" s="34" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="K18" s="34" t="s">
-        <v>227</v>
+        <v>209</v>
       </c>
     </row>
     <row r="19" spans="2:11" ht="35" customHeight="1">
       <c r="B19" s="21" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C19" s="37">
-        <v>46315</v>
+        <v>46320</v>
       </c>
       <c r="D19" s="33" t="s">
-        <v>30</v>
+        <v>235</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>47</v>
-      </c>
-      <c r="F19" s="38" t="s">
-        <v>243</v>
-      </c>
+        <v>236</v>
+      </c>
+      <c r="F19" s="38"/>
       <c r="G19" s="33" t="s">
-        <v>50</v>
+        <v>240</v>
       </c>
       <c r="H19" s="33" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="I19" s="33" t="s">
         <v>241</v>
       </c>
       <c r="J19" s="33" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="K19" s="33" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="20" spans="2:11" ht="35" customHeight="1">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" ht="21" customHeight="1">
       <c r="B20" s="24" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C20" s="39">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="D20" s="34" t="s">
         <v>31</v>
       </c>
       <c r="E20" s="34" t="s">
-        <v>169</v>
+        <v>218</v>
       </c>
       <c r="F20" s="40" t="s">
+        <v>243</v>
+      </c>
+      <c r="G20" s="34" t="s">
+        <v>244</v>
+      </c>
+      <c r="H20" s="34" t="s">
         <v>245</v>
       </c>
-      <c r="G20" s="34" t="s">
+      <c r="I20" s="34" t="s">
         <v>246</v>
       </c>
-      <c r="H20" s="34" t="s">
-        <v>224</v>
-      </c>
-      <c r="I20" s="34" t="s">
+      <c r="J20" s="34" t="s">
         <v>247</v>
       </c>
-      <c r="J20" s="34" t="s">
-        <v>226</v>
-      </c>
       <c r="K20" s="34" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="21" spans="2:11" ht="35" customHeight="1">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" ht="21" customHeight="1">
       <c r="B21" s="21" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C21" s="37">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="D21" s="33" t="s">
         <v>31</v>
       </c>
       <c r="E21" s="33" t="s">
-        <v>169</v>
+        <v>218</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G21" s="33" t="s">
-        <v>250</v>
+        <v>191</v>
       </c>
       <c r="H21" s="33" t="s">
-        <v>224</v>
+        <v>245</v>
       </c>
       <c r="I21" s="33" t="s">
+        <v>251</v>
+      </c>
+      <c r="J21" s="33" t="s">
         <v>247</v>
       </c>
-      <c r="J21" s="33" t="s">
-        <v>226</v>
-      </c>
       <c r="K21" s="33" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="22" spans="2:11" ht="35" customHeight="1">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" ht="21" customHeight="1">
       <c r="B22" s="24" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C22" s="39">
-        <v>46311</v>
+        <v>46315</v>
       </c>
       <c r="D22" s="34" t="s">
-        <v>252</v>
+        <v>31</v>
       </c>
       <c r="E22" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="F22" s="40" t="s">
         <v>253</v>
       </c>
-      <c r="F22" s="40" t="s">
+      <c r="G22" s="34" t="s">
         <v>254</v>
       </c>
-      <c r="G22" s="34" t="s">
+      <c r="H22" s="34" t="s">
+        <v>245</v>
+      </c>
+      <c r="I22" s="34" t="s">
         <v>255</v>
       </c>
-      <c r="H22" s="34" t="s">
+      <c r="J22" s="34" t="s">
+        <v>247</v>
+      </c>
+      <c r="K22" s="34" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" ht="21" customHeight="1">
+      <c r="B23" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="I22" s="34" t="s">
+      <c r="C23" s="37">
+        <v>46315</v>
+      </c>
+      <c r="D23" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="E23" s="33" t="s">
+        <v>218</v>
+      </c>
+      <c r="F23" s="38" t="s">
         <v>257</v>
       </c>
-      <c r="J22" s="34" t="s">
-        <v>226</v>
-      </c>
-      <c r="K22" s="34" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="23" spans="2:11" ht="35" customHeight="1">
-      <c r="B23" s="21" t="s">
+      <c r="G23" s="33" t="s">
         <v>258</v>
       </c>
-      <c r="C23" s="37">
-        <v>46311</v>
-      </c>
-      <c r="D23" s="33" t="s">
-        <v>252</v>
-      </c>
-      <c r="E23" s="33" t="s">
-        <v>253</v>
-      </c>
-      <c r="F23" s="38" t="s">
+      <c r="H23" s="33" t="s">
+        <v>245</v>
+      </c>
+      <c r="I23" s="33" t="s">
         <v>259</v>
       </c>
-      <c r="G23" s="33" t="s">
+      <c r="J23" s="33" t="s">
+        <v>247</v>
+      </c>
+      <c r="K23" s="33" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" ht="35" customHeight="1">
+      <c r="B24" s="24" t="s">
         <v>260</v>
       </c>
-      <c r="H23" s="33" t="s">
-        <v>256</v>
-      </c>
-      <c r="I23" s="33" t="s">
-        <v>257</v>
-      </c>
-      <c r="J23" s="33" t="s">
-        <v>226</v>
-      </c>
-      <c r="K23" s="33" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="24" spans="2:11" ht="49" customHeight="1">
-      <c r="B24" s="24" t="s">
+      <c r="C24" s="39">
+        <v>46315</v>
+      </c>
+      <c r="D24" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="E24" s="34" t="s">
+        <v>47</v>
+      </c>
+      <c r="F24" s="40" t="s">
         <v>261</v>
       </c>
-      <c r="C24" s="39" t="s">
+      <c r="G24" s="34" t="s">
+        <v>48</v>
+      </c>
+      <c r="H24" s="34" t="s">
+        <v>245</v>
+      </c>
+      <c r="I24" s="34" t="s">
         <v>262</v>
       </c>
-      <c r="D24" s="34" t="s">
-        <v>263</v>
-      </c>
-      <c r="E24" s="34" t="s">
-        <v>264</v>
-      </c>
-      <c r="F24" s="40"/>
-      <c r="G24" s="34" t="s">
-        <v>203</v>
-      </c>
-      <c r="H24" s="34" t="s">
-        <v>265</v>
-      </c>
-      <c r="I24" s="34" t="s">
-        <v>266</v>
-      </c>
       <c r="J24" s="34" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="K24" s="34" t="s">
-        <v>207</v>
+        <v>248</v>
       </c>
     </row>
     <row r="25" spans="2:11" ht="35" customHeight="1">
       <c r="B25" s="21" t="s">
-        <v>267</v>
-      </c>
-      <c r="C25" s="37" t="s">
+        <v>263</v>
+      </c>
+      <c r="C25" s="37">
+        <v>46315</v>
+      </c>
+      <c r="D25" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="E25" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="F25" s="38" t="s">
+        <v>264</v>
+      </c>
+      <c r="G25" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="H25" s="33" t="s">
+        <v>245</v>
+      </c>
+      <c r="I25" s="33" t="s">
         <v>262</v>
       </c>
-      <c r="D25" s="33" t="s">
-        <v>252</v>
-      </c>
-      <c r="E25" s="33" t="s">
-        <v>268</v>
-      </c>
-      <c r="F25" s="38"/>
-      <c r="G25" s="33" t="s">
-        <v>203</v>
-      </c>
-      <c r="H25" s="33" t="s">
-        <v>265</v>
-      </c>
-      <c r="I25" s="33" t="s">
-        <v>269</v>
-      </c>
       <c r="J25" s="33" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="K25" s="33" t="s">
-        <v>207</v>
+        <v>248</v>
       </c>
     </row>
     <row r="26" spans="2:11" ht="35" customHeight="1">
       <c r="B26" s="24" t="s">
-        <v>270</v>
-      </c>
-      <c r="C26" s="39" t="s">
-        <v>262</v>
+        <v>265</v>
+      </c>
+      <c r="C26" s="39">
+        <v>46314</v>
       </c>
       <c r="D26" s="34" t="s">
-        <v>252</v>
+        <v>31</v>
       </c>
       <c r="E26" s="34" t="s">
-        <v>271</v>
-      </c>
-      <c r="F26" s="40"/>
+        <v>169</v>
+      </c>
+      <c r="F26" s="40" t="s">
+        <v>266</v>
+      </c>
       <c r="G26" s="34" t="s">
-        <v>203</v>
+        <v>267</v>
       </c>
       <c r="H26" s="34" t="s">
-        <v>265</v>
+        <v>245</v>
       </c>
       <c r="I26" s="34" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="J26" s="34" t="s">
-        <v>206</v>
+        <v>247</v>
       </c>
       <c r="K26" s="34" t="s">
-        <v>207</v>
+        <v>248</v>
       </c>
     </row>
     <row r="27" spans="2:11" ht="35" customHeight="1">
       <c r="B27" s="21" t="s">
-        <v>273</v>
-      </c>
-      <c r="C27" s="37" t="s">
-        <v>262</v>
+        <v>269</v>
+      </c>
+      <c r="C27" s="37">
+        <v>46314</v>
       </c>
       <c r="D27" s="33" t="s">
         <v>31</v>
       </c>
       <c r="E27" s="33" t="s">
-        <v>221</v>
-      </c>
-      <c r="F27" s="38"/>
+        <v>169</v>
+      </c>
+      <c r="F27" s="38" t="s">
+        <v>270</v>
+      </c>
       <c r="G27" s="33" t="s">
-        <v>203</v>
+        <v>271</v>
       </c>
       <c r="H27" s="33" t="s">
-        <v>265</v>
+        <v>245</v>
       </c>
       <c r="I27" s="33" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="J27" s="33" t="s">
-        <v>206</v>
+        <v>247</v>
       </c>
       <c r="K27" s="33" t="s">
-        <v>207</v>
+        <v>248</v>
       </c>
     </row>
     <row r="28" spans="2:11" ht="35" customHeight="1">
       <c r="B28" s="24" t="s">
+        <v>272</v>
+      </c>
+      <c r="C28" s="39">
+        <v>46311</v>
+      </c>
+      <c r="D28" s="34" t="s">
+        <v>211</v>
+      </c>
+      <c r="E28" s="34" t="s">
+        <v>273</v>
+      </c>
+      <c r="F28" s="40" t="s">
+        <v>274</v>
+      </c>
+      <c r="G28" s="34" t="s">
         <v>275</v>
       </c>
-      <c r="C28" s="39" t="s">
-        <v>262</v>
-      </c>
-      <c r="D28" s="34" t="s">
+      <c r="H28" s="34" t="s">
         <v>276</v>
       </c>
-      <c r="E28" s="34" t="s">
+      <c r="I28" s="34" t="s">
         <v>277</v>
       </c>
-      <c r="F28" s="40"/>
-      <c r="G28" s="34" t="s">
-        <v>203</v>
-      </c>
-      <c r="H28" s="34" t="s">
-        <v>265</v>
-      </c>
-      <c r="I28" s="34" t="s">
-        <v>278</v>
-      </c>
       <c r="J28" s="34" t="s">
-        <v>206</v>
+        <v>247</v>
       </c>
       <c r="K28" s="34" t="s">
-        <v>207</v>
+        <v>248</v>
       </c>
     </row>
     <row r="29" spans="2:11" ht="35" customHeight="1">
       <c r="B29" s="21" t="s">
+        <v>278</v>
+      </c>
+      <c r="C29" s="37">
+        <v>46311</v>
+      </c>
+      <c r="D29" s="33" t="s">
+        <v>211</v>
+      </c>
+      <c r="E29" s="33" t="s">
+        <v>273</v>
+      </c>
+      <c r="F29" s="38" t="s">
         <v>279</v>
       </c>
-      <c r="C29" s="37" t="s">
-        <v>262</v>
-      </c>
-      <c r="D29" s="33" t="s">
-        <v>30</v>
-      </c>
-      <c r="E29" s="33" t="s">
+      <c r="G29" s="33" t="s">
         <v>280</v>
       </c>
-      <c r="F29" s="38"/>
-      <c r="G29" s="33" t="s">
-        <v>203</v>
-      </c>
       <c r="H29" s="33" t="s">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="I29" s="33" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="J29" s="33" t="s">
-        <v>206</v>
+        <v>247</v>
       </c>
       <c r="K29" s="33" t="s">
-        <v>207</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -11747,20 +11744,20 @@
     </row>
     <row r="7" spans="1:15" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
     </row>
     <row r="8" spans="1:15" ht="36" customHeight="1">
       <c r="B8" s="19" t="s">
+        <v>282</v>
+      </c>
+      <c r="C8" s="20" t="s">
         <v>283</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="D8" s="20" t="s">
         <v>284</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="19" customHeight="1">
@@ -12230,10 +12227,10 @@
         <v>46321</v>
       </c>
       <c r="C51" s="22">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D51" s="22">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="52" spans="2:4" ht="19" customHeight="1">
@@ -12244,7 +12241,7 @@
         <v>0</v>
       </c>
       <c r="D52" s="25">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="53" spans="2:4" ht="22" customHeight="1">
@@ -12253,7 +12250,7 @@
       </c>
       <c r="C53" s="28">
         <f>SUM(C9:C52)</f>
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D53" s="35"/>
     </row>
@@ -12310,7 +12307,7 @@
     <row r="2" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -12389,7 +12386,7 @@
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="F7" s="8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.25">
@@ -12397,16 +12394,16 @@
         <v>29</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D8" s="20" t="s">
         <v>20</v>
       </c>
       <c r="E8" s="20" t="s">
+        <v>288</v>
+      </c>
+      <c r="F8" s="20" t="s">
         <v>289</v>
-      </c>
-      <c r="F8" s="20" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
@@ -12428,7 +12425,7 @@
     </row>
     <row r="10" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="24" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="C10" s="25">
         <v>3820</v>
@@ -12445,7 +12442,7 @@
     </row>
     <row r="11" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="21" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C11" s="22">
         <v>780</v>
@@ -12462,7 +12459,7 @@
     </row>
     <row r="12" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="24" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C12" s="25">
         <v>757</v>
@@ -12479,7 +12476,7 @@
     </row>
     <row r="13" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="21" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C13" s="22">
         <v>498</v>
@@ -12496,7 +12493,7 @@
     </row>
     <row r="14" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C14" s="25">
         <v>250</v>
@@ -12513,7 +12510,7 @@
     </row>
     <row r="15" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="21" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C15" s="22">
         <v>205</v>
@@ -12530,7 +12527,7 @@
     </row>
     <row r="16" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="24" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C16" s="25">
         <v>180</v>
@@ -12547,7 +12544,7 @@
     </row>
     <row r="17" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="21" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C17" s="22">
         <v>141</v>
@@ -12564,7 +12561,7 @@
     </row>
     <row r="18" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="24" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="C18" s="25">
         <v>110</v>
@@ -12581,7 +12578,7 @@
     </row>
     <row r="19" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="21" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C19" s="22">
         <v>79</v>
@@ -12615,7 +12612,7 @@
     </row>
     <row r="21" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="21" t="s">
-        <v>213</v>
+        <v>235</v>
       </c>
       <c r="C21" s="22">
         <v>64</v>
@@ -12632,7 +12629,7 @@
     </row>
     <row r="22" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="24" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C22" s="25">
         <v>64</v>
@@ -12649,7 +12646,7 @@
     </row>
     <row r="23" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="21" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C23" s="22">
         <v>44</v>
@@ -12666,7 +12663,7 @@
     </row>
     <row r="24" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="24" t="s">
-        <v>263</v>
+        <v>203</v>
       </c>
       <c r="C24" s="25">
         <v>17</v>
@@ -12683,7 +12680,7 @@
     </row>
     <row r="25" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="21" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C25" s="22">
         <v>17</v>
@@ -12717,7 +12714,7 @@
     </row>
     <row r="27" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="21" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C27" s="22">
         <v>11</v>
@@ -12734,7 +12731,7 @@
     </row>
     <row r="28" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="24" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C28" s="25">
         <v>7</v>
@@ -12751,7 +12748,7 @@
     </row>
     <row r="29" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="21" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C29" s="22">
         <v>7</v>
@@ -12768,7 +12765,7 @@
     </row>
     <row r="30" spans="2:6" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="24" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C30" s="25">
         <v>1</v>
@@ -12805,7 +12802,7 @@
     </row>
     <row r="33" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="43" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C33" s="43"/>
       <c r="D33" s="43"/>
@@ -12896,7 +12893,7 @@
     <row r="2" spans="1:9" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -12945,7 +12942,7 @@
     </row>
     <row r="7" spans="1:9" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -12953,12 +12950,12 @@
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="46" customHeight="1">
       <c r="B8" s="44" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C8" s="44"/>
       <c r="D8" s="44"/>
@@ -12970,7 +12967,7 @@
     <row r="9" spans="1:9" ht="8" customHeight="1"/>
     <row r="10" spans="1:9" ht="36" customHeight="1">
       <c r="B10" s="19" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C10" s="32" t="s">
         <v>29</v>
@@ -12979,16 +12976,16 @@
         <v>43</v>
       </c>
       <c r="E10" s="20" t="s">
+        <v>287</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="G10" s="20" t="s">
         <v>288</v>
       </c>
-      <c r="F10" s="20" t="s">
+      <c r="H10" s="36" t="s">
         <v>310</v>
-      </c>
-      <c r="G10" s="20" t="s">
-        <v>289</v>
-      </c>
-      <c r="H10" s="36" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="19" customHeight="1">
@@ -12996,10 +12993,10 @@
         <v>46265</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E11" s="22">
         <v>399</v>
@@ -13011,7 +13008,7 @@
         <v>399</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="19" customHeight="1">
@@ -13019,10 +13016,10 @@
         <v>46265</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D12" s="34" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E12" s="25">
         <v>3</v>
@@ -13034,7 +13031,7 @@
         <v>3</v>
       </c>
       <c r="H12" s="40" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="19" customHeight="1">
@@ -13042,10 +13039,10 @@
         <v>46265</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E13" s="22">
         <v>1</v>
@@ -13057,7 +13054,7 @@
         <v>1</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="19" customHeight="1">
@@ -13065,10 +13062,10 @@
         <v>46268</v>
       </c>
       <c r="C14" s="34" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D14" s="34" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E14" s="25">
         <v>250</v>
@@ -13080,7 +13077,7 @@
         <v>249</v>
       </c>
       <c r="H14" s="40" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="19" customHeight="1">
@@ -13088,10 +13085,10 @@
         <v>46268</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E15" s="22">
         <v>10</v>
@@ -13103,7 +13100,7 @@
         <v>1</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="19" customHeight="1">
@@ -13111,10 +13108,10 @@
         <v>46268</v>
       </c>
       <c r="C16" s="34" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D16" s="34" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E16" s="25">
         <v>10</v>
@@ -13126,7 +13123,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="40" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="19" customHeight="1">
@@ -13134,10 +13131,10 @@
         <v>46269</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E17" s="22">
         <v>7</v>
@@ -13149,7 +13146,7 @@
         <v>1</v>
       </c>
       <c r="H17" s="38" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="19" customHeight="1">
@@ -13157,10 +13154,10 @@
         <v>46272</v>
       </c>
       <c r="C18" s="34" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D18" s="34" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E18" s="25">
         <v>8</v>
@@ -13172,7 +13169,7 @@
         <v>2</v>
       </c>
       <c r="H18" s="40" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="19" customHeight="1">
@@ -13180,10 +13177,10 @@
         <v>46273</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D19" s="33" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E19" s="22">
         <v>25</v>
@@ -13195,7 +13192,7 @@
         <v>20</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="19" customHeight="1">
@@ -13203,10 +13200,10 @@
         <v>46274</v>
       </c>
       <c r="C20" s="34" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D20" s="34" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E20" s="25">
         <v>20</v>
@@ -13218,7 +13215,7 @@
         <v>3</v>
       </c>
       <c r="H20" s="40" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="19" customHeight="1">
@@ -13226,10 +13223,10 @@
         <v>46274</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D21" s="33" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E21" s="22">
         <v>8</v>
@@ -13241,7 +13238,7 @@
         <v>2</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="19" customHeight="1">
@@ -13249,10 +13246,10 @@
         <v>46274</v>
       </c>
       <c r="C22" s="34" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D22" s="34" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E22" s="25">
         <v>4</v>
@@ -13264,7 +13261,7 @@
         <v>1</v>
       </c>
       <c r="H22" s="40" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="19" customHeight="1">
@@ -13272,10 +13269,10 @@
         <v>46274</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D23" s="33" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E23" s="22">
         <v>2</v>
@@ -13287,7 +13284,7 @@
         <v>1</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="19" customHeight="1">
@@ -13295,10 +13292,10 @@
         <v>46274</v>
       </c>
       <c r="C24" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D24" s="34" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E24" s="25">
         <v>1</v>
@@ -13310,7 +13307,7 @@
         <v>1</v>
       </c>
       <c r="H24" s="40" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="25" spans="2:8" ht="19" customHeight="1">
@@ -13318,10 +13315,10 @@
         <v>46274</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D25" s="33" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E25" s="22">
         <v>1</v>
@@ -13333,7 +13330,7 @@
         <v>1</v>
       </c>
       <c r="H25" s="38" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="19" customHeight="1">
@@ -13341,10 +13338,10 @@
         <v>46275</v>
       </c>
       <c r="C26" s="34" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D26" s="34" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E26" s="25">
         <v>4</v>
@@ -13356,7 +13353,7 @@
         <v>1</v>
       </c>
       <c r="H26" s="40" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="27" spans="2:8" ht="19" customHeight="1">
@@ -13379,7 +13376,7 @@
         <v>1</v>
       </c>
       <c r="H27" s="38" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="28" spans="2:8" ht="19" customHeight="1">
@@ -13402,7 +13399,7 @@
         <v>2</v>
       </c>
       <c r="H28" s="40" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="29" spans="2:8" ht="19" customHeight="1">
@@ -13410,10 +13407,10 @@
         <v>46275</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D29" s="33" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E29" s="22">
         <v>1</v>
@@ -13425,7 +13422,7 @@
         <v>1</v>
       </c>
       <c r="H29" s="38" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="30" spans="2:8" ht="19" customHeight="1">
@@ -13433,10 +13430,10 @@
         <v>46275</v>
       </c>
       <c r="C30" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D30" s="34" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E30" s="25">
         <v>1</v>
@@ -13448,7 +13445,7 @@
         <v>1</v>
       </c>
       <c r="H30" s="40" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="31" spans="2:8" ht="19" customHeight="1">
@@ -13456,10 +13453,10 @@
         <v>46280</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D31" s="33" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E31" s="22">
         <v>1</v>
@@ -13471,7 +13468,7 @@
         <v>1</v>
       </c>
       <c r="H31" s="38" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="32" spans="2:8" ht="19" customHeight="1">
@@ -13479,10 +13476,10 @@
         <v>46282</v>
       </c>
       <c r="C32" s="34" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D32" s="34" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E32" s="25">
         <v>10</v>
@@ -13494,7 +13491,7 @@
         <v>5</v>
       </c>
       <c r="H32" s="40" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="33" spans="2:8" ht="19" customHeight="1">
@@ -13502,10 +13499,10 @@
         <v>46283</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D33" s="33" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E33" s="22">
         <v>66</v>
@@ -13517,7 +13514,7 @@
         <v>66</v>
       </c>
       <c r="H33" s="38" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="34" spans="2:8" ht="19" customHeight="1">
@@ -13525,10 +13522,10 @@
         <v>46283</v>
       </c>
       <c r="C34" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D34" s="34" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E34" s="25">
         <v>1</v>
@@ -13540,7 +13537,7 @@
         <v>1</v>
       </c>
       <c r="H34" s="40" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="35" spans="2:8" ht="19" customHeight="1">
@@ -13548,10 +13545,10 @@
         <v>46285</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D35" s="33" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E35" s="22">
         <v>10</v>
@@ -13563,7 +13560,7 @@
         <v>10</v>
       </c>
       <c r="H35" s="38" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="36" spans="2:8" ht="19" customHeight="1">
@@ -13571,10 +13568,10 @@
         <v>46287</v>
       </c>
       <c r="C36" s="34" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D36" s="34" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E36" s="25">
         <v>12</v>
@@ -13586,7 +13583,7 @@
         <v>3</v>
       </c>
       <c r="H36" s="40" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="37" spans="2:8" ht="19" customHeight="1">
@@ -13597,7 +13594,7 @@
         <v>31</v>
       </c>
       <c r="D37" s="33" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E37" s="22">
         <v>1500</v>
@@ -13609,7 +13606,7 @@
         <v>1500</v>
       </c>
       <c r="H37" s="38" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="38" spans="2:8" ht="19" customHeight="1">
@@ -13617,10 +13614,10 @@
         <v>46289</v>
       </c>
       <c r="C38" s="34" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D38" s="34" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E38" s="25">
         <v>182</v>
@@ -13632,7 +13629,7 @@
         <v>182</v>
       </c>
       <c r="H38" s="40" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="39" spans="2:8" ht="19" customHeight="1">
@@ -13640,10 +13637,10 @@
         <v>46289</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D39" s="33" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E39" s="22">
         <v>130</v>
@@ -13655,7 +13652,7 @@
         <v>65</v>
       </c>
       <c r="H39" s="38" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="40" spans="2:8" ht="19" customHeight="1">
@@ -13666,7 +13663,7 @@
         <v>31</v>
       </c>
       <c r="D40" s="34" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E40" s="25">
         <v>700</v>
@@ -13678,7 +13675,7 @@
         <v>700</v>
       </c>
       <c r="H40" s="40" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="41" spans="2:8" ht="19" customHeight="1">
@@ -13686,10 +13683,10 @@
         <v>46290</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D41" s="33" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E41" s="22">
         <v>4</v>
@@ -13701,7 +13698,7 @@
         <v>1</v>
       </c>
       <c r="H41" s="38" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="42" spans="2:8" ht="19" customHeight="1">
@@ -13712,7 +13709,7 @@
         <v>31</v>
       </c>
       <c r="D42" s="34" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E42" s="25">
         <v>400</v>
@@ -13724,7 +13721,7 @@
         <v>400</v>
       </c>
       <c r="H42" s="40" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="43" spans="2:8" ht="19" customHeight="1">
@@ -13732,10 +13729,10 @@
         <v>46293</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D43" s="33" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E43" s="22">
         <v>140</v>
@@ -13747,7 +13744,7 @@
         <v>140</v>
       </c>
       <c r="H43" s="38" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="44" spans="2:8" ht="19" customHeight="1">
@@ -13758,7 +13755,7 @@
         <v>31</v>
       </c>
       <c r="D44" s="34" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E44" s="25">
         <v>300</v>
@@ -13770,7 +13767,7 @@
         <v>300</v>
       </c>
       <c r="H44" s="40" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="45" spans="2:8" ht="19" customHeight="1">
@@ -13778,10 +13775,10 @@
         <v>46294</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D45" s="33" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E45" s="22">
         <v>60</v>
@@ -13793,7 +13790,7 @@
         <v>23</v>
       </c>
       <c r="H45" s="38" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="46" spans="2:8" ht="19" customHeight="1">
@@ -13801,10 +13798,10 @@
         <v>46294</v>
       </c>
       <c r="C46" s="34" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D46" s="34" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E46" s="25">
         <v>7</v>
@@ -13816,7 +13813,7 @@
         <v>1</v>
       </c>
       <c r="H46" s="40" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="47" spans="2:8" ht="19" customHeight="1">
@@ -13824,10 +13821,10 @@
         <v>46295</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="D47" s="33" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E47" s="22">
         <v>10</v>
@@ -13839,7 +13836,7 @@
         <v>3</v>
       </c>
       <c r="H47" s="38" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="48" spans="2:8" ht="19" customHeight="1">
@@ -13847,10 +13844,10 @@
         <v>46296</v>
       </c>
       <c r="C48" s="34" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D48" s="34" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E48" s="25">
         <v>540</v>
@@ -13862,7 +13859,7 @@
         <v>270</v>
       </c>
       <c r="H48" s="40" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="49" spans="2:8" ht="19" customHeight="1">
@@ -13870,10 +13867,10 @@
         <v>46296</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D49" s="33" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E49" s="22">
         <v>120</v>
@@ -13885,7 +13882,7 @@
         <v>120</v>
       </c>
       <c r="H49" s="38" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="50" spans="2:8" ht="19" customHeight="1">
@@ -13893,10 +13890,10 @@
         <v>46296</v>
       </c>
       <c r="C50" s="34" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D50" s="34" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E50" s="25">
         <v>80</v>
@@ -13908,7 +13905,7 @@
         <v>80</v>
       </c>
       <c r="H50" s="40" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="51" spans="2:8" ht="19" customHeight="1">
@@ -13916,10 +13913,10 @@
         <v>46296</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D51" s="33" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E51" s="22">
         <v>5</v>
@@ -13931,7 +13928,7 @@
         <v>5</v>
       </c>
       <c r="H51" s="38" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="52" spans="2:8" ht="19" customHeight="1">
@@ -13939,10 +13936,10 @@
         <v>46296</v>
       </c>
       <c r="C52" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D52" s="34" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E52" s="25">
         <v>1</v>
@@ -13954,7 +13951,7 @@
         <v>1</v>
       </c>
       <c r="H52" s="40" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="53" spans="2:8" ht="19" customHeight="1">
@@ -13962,10 +13959,10 @@
         <v>46296</v>
       </c>
       <c r="C53" s="33" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D53" s="33" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E53" s="22">
         <v>1</v>
@@ -13977,7 +13974,7 @@
         <v>1</v>
       </c>
       <c r="H53" s="38" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="54" spans="2:8" ht="19" customHeight="1">
@@ -13985,10 +13982,10 @@
         <v>46297</v>
       </c>
       <c r="C54" s="34" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D54" s="34" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E54" s="25">
         <v>87</v>
@@ -14000,7 +13997,7 @@
         <v>87</v>
       </c>
       <c r="H54" s="40" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="55" spans="2:8" ht="19" customHeight="1">
@@ -14008,10 +14005,10 @@
         <v>46297</v>
       </c>
       <c r="C55" s="33" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D55" s="33" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E55" s="22">
         <v>85</v>
@@ -14023,7 +14020,7 @@
         <v>85</v>
       </c>
       <c r="H55" s="38" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="56" spans="2:8" ht="19" customHeight="1">
@@ -14031,10 +14028,10 @@
         <v>46297</v>
       </c>
       <c r="C56" s="34" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D56" s="34" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E56" s="25">
         <v>85</v>
@@ -14046,7 +14043,7 @@
         <v>85</v>
       </c>
       <c r="H56" s="40" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="57" spans="2:8" ht="19" customHeight="1">
@@ -14054,10 +14051,10 @@
         <v>46298</v>
       </c>
       <c r="C57" s="33" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D57" s="33" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E57" s="22">
         <v>772</v>
@@ -14069,7 +14066,7 @@
         <v>772</v>
       </c>
       <c r="H57" s="38" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="58" spans="2:8" ht="19" customHeight="1">
@@ -14077,10 +14074,10 @@
         <v>46298</v>
       </c>
       <c r="C58" s="34" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D58" s="34" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E58" s="25">
         <v>18</v>
@@ -14092,7 +14089,7 @@
         <v>18</v>
       </c>
       <c r="H58" s="40" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="59" spans="2:8" ht="19" customHeight="1">
@@ -14100,10 +14097,10 @@
         <v>46299</v>
       </c>
       <c r="C59" s="33" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D59" s="33" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E59" s="22">
         <v>30</v>
@@ -14115,7 +14112,7 @@
         <v>30</v>
       </c>
       <c r="H59" s="38" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="60" spans="2:8" ht="19" customHeight="1">
@@ -14138,7 +14135,7 @@
         <v>1500</v>
       </c>
       <c r="H60" s="40" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="61" spans="2:8" ht="19" customHeight="1">
@@ -14146,10 +14143,10 @@
         <v>46300</v>
       </c>
       <c r="C61" s="33" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="D61" s="33" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E61" s="22">
         <v>10</v>
@@ -14161,7 +14158,7 @@
         <v>10</v>
       </c>
       <c r="H61" s="38" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="62" spans="2:8" ht="19" customHeight="1">
@@ -14169,10 +14166,10 @@
         <v>46301</v>
       </c>
       <c r="C62" s="34" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D62" s="34" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="E62" s="25">
         <v>1270</v>
@@ -14184,7 +14181,7 @@
         <v>1270</v>
       </c>
       <c r="H62" s="40" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="63" spans="2:8" ht="19" customHeight="1">
@@ -14192,10 +14189,10 @@
         <v>46301</v>
       </c>
       <c r="C63" s="33" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D63" s="33" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E63" s="22">
         <v>50</v>
@@ -14207,7 +14204,7 @@
         <v>50</v>
       </c>
       <c r="H63" s="38" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="64" spans="2:8" ht="19" customHeight="1">
@@ -14215,10 +14212,10 @@
         <v>46301</v>
       </c>
       <c r="C64" s="34" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D64" s="34" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E64" s="25">
         <v>10</v>
@@ -14230,7 +14227,7 @@
         <v>5</v>
       </c>
       <c r="H64" s="40" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="65" spans="2:8" ht="19" customHeight="1">
@@ -14238,10 +14235,10 @@
         <v>46302</v>
       </c>
       <c r="C65" s="33" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D65" s="33" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E65" s="22">
         <v>10</v>
@@ -14253,7 +14250,7 @@
         <v>10</v>
       </c>
       <c r="H65" s="38" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="66" spans="2:8" ht="19" customHeight="1">
@@ -14261,10 +14258,10 @@
         <v>46303</v>
       </c>
       <c r="C66" s="34" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D66" s="34" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E66" s="25">
         <v>141</v>
@@ -14276,7 +14273,7 @@
         <v>141</v>
       </c>
       <c r="H66" s="40" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="67" spans="2:8" ht="19" customHeight="1">
@@ -14284,10 +14281,10 @@
         <v>46303</v>
       </c>
       <c r="C67" s="33" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D67" s="33" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E67" s="22">
         <v>125</v>
@@ -14299,7 +14296,7 @@
         <v>125</v>
       </c>
       <c r="H67" s="38" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="68" spans="2:8" ht="19" customHeight="1">
@@ -14307,10 +14304,10 @@
         <v>46303</v>
       </c>
       <c r="C68" s="34" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D68" s="34" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E68" s="25">
         <v>75</v>
@@ -14322,7 +14319,7 @@
         <v>75</v>
       </c>
       <c r="H68" s="40" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="69" spans="2:8" ht="19" customHeight="1">
@@ -14330,10 +14327,10 @@
         <v>46303</v>
       </c>
       <c r="C69" s="33" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D69" s="33" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E69" s="22">
         <v>40</v>
@@ -14345,7 +14342,7 @@
         <v>40</v>
       </c>
       <c r="H69" s="38" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="70" spans="2:8" ht="19" customHeight="1">
@@ -14353,10 +14350,10 @@
         <v>46303</v>
       </c>
       <c r="C70" s="34" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D70" s="34" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E70" s="25">
         <v>40</v>
@@ -14368,7 +14365,7 @@
         <v>40</v>
       </c>
       <c r="H70" s="40" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="71" spans="2:8" ht="19" customHeight="1">
@@ -14376,10 +14373,10 @@
         <v>46304</v>
       </c>
       <c r="C71" s="33" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D71" s="33" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E71" s="22">
         <v>11</v>
@@ -14391,7 +14388,7 @@
         <v>11</v>
       </c>
       <c r="H71" s="38" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="72" spans="2:8" ht="19" customHeight="1">
@@ -14399,10 +14396,10 @@
         <v>46305</v>
       </c>
       <c r="C72" s="34" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D72" s="34" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E72" s="25">
         <v>70</v>
@@ -14414,7 +14411,7 @@
         <v>30</v>
       </c>
       <c r="H72" s="40" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="73" spans="2:8" ht="19" customHeight="1">
@@ -14422,10 +14419,10 @@
         <v>46305</v>
       </c>
       <c r="C73" s="33" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D73" s="33" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="E73" s="22">
         <v>29</v>
@@ -14437,7 +14434,7 @@
         <v>30</v>
       </c>
       <c r="H73" s="38" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="74" spans="2:8" ht="19" customHeight="1">
@@ -14445,10 +14442,10 @@
         <v>46307</v>
       </c>
       <c r="C74" s="34" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D74" s="34" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E74" s="25">
         <v>22</v>
@@ -14460,7 +14457,7 @@
         <v>22</v>
       </c>
       <c r="H74" s="40" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="75" spans="2:8" ht="19" customHeight="1">
@@ -14468,10 +14465,10 @@
         <v>46307</v>
       </c>
       <c r="C75" s="33" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D75" s="33" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="E75" s="22">
         <v>6</v>
@@ -14483,7 +14480,7 @@
         <v>1</v>
       </c>
       <c r="H75" s="38" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="76" spans="2:8" ht="19" customHeight="1">
@@ -14491,10 +14488,10 @@
         <v>46308</v>
       </c>
       <c r="C76" s="34" t="s">
-        <v>213</v>
+        <v>235</v>
       </c>
       <c r="D76" s="34" t="s">
-        <v>214</v>
+        <v>236</v>
       </c>
       <c r="E76" s="25">
         <v>64</v>
@@ -14506,7 +14503,7 @@
         <v>32</v>
       </c>
       <c r="H76" s="40" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="77" spans="2:8" ht="19" customHeight="1">
@@ -14514,10 +14511,10 @@
         <v>46308</v>
       </c>
       <c r="C77" s="33" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D77" s="33" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E77" s="22">
         <v>24</v>
@@ -14529,7 +14526,7 @@
         <v>6</v>
       </c>
       <c r="H77" s="38" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="78" spans="2:8" ht="19" customHeight="1">
@@ -14537,10 +14534,10 @@
         <v>46308</v>
       </c>
       <c r="C78" s="34" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D78" s="34" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E78" s="25">
         <v>24</v>
@@ -14552,7 +14549,7 @@
         <v>6</v>
       </c>
       <c r="H78" s="40" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="79" spans="2:8" ht="19" customHeight="1">
@@ -14560,10 +14557,10 @@
         <v>46308</v>
       </c>
       <c r="C79" s="33" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D79" s="33" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E79" s="22">
         <v>24</v>
@@ -14575,7 +14572,7 @@
         <v>6</v>
       </c>
       <c r="H79" s="38" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="80" spans="2:8" ht="19" customHeight="1">
@@ -14583,10 +14580,10 @@
         <v>46309</v>
       </c>
       <c r="C80" s="34" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D80" s="34" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E80" s="25">
         <v>135</v>
@@ -14598,7 +14595,7 @@
         <v>135</v>
       </c>
       <c r="H80" s="40" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="81" spans="2:8" ht="19" customHeight="1">
@@ -14609,7 +14606,7 @@
         <v>32</v>
       </c>
       <c r="D81" s="33" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E81" s="22">
         <v>7</v>
@@ -14621,7 +14618,7 @@
         <v>7</v>
       </c>
       <c r="H81" s="38" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="82" spans="2:8" ht="19" customHeight="1">
@@ -14629,10 +14626,10 @@
         <v>46311</v>
       </c>
       <c r="C82" s="34" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D82" s="34" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E82" s="25">
         <v>200</v>
@@ -14644,7 +14641,7 @@
         <v>200</v>
       </c>
       <c r="H82" s="40" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="83" spans="2:8" ht="19" customHeight="1">
@@ -14652,10 +14649,10 @@
         <v>46311</v>
       </c>
       <c r="C83" s="33" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D83" s="33" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E83" s="22">
         <v>44</v>
@@ -14667,7 +14664,7 @@
         <v>44</v>
       </c>
       <c r="H83" s="38" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="84" spans="2:8" ht="19" customHeight="1">
@@ -14675,10 +14672,10 @@
         <v>46311</v>
       </c>
       <c r="C84" s="34" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D84" s="34" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E84" s="25">
         <v>30</v>
@@ -14690,7 +14687,7 @@
         <v>30</v>
       </c>
       <c r="H84" s="40" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="85" spans="2:8" ht="19" customHeight="1">
@@ -14698,10 +14695,10 @@
         <v>46311</v>
       </c>
       <c r="C85" s="33" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D85" s="33" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E85" s="22">
         <v>4</v>
@@ -14713,7 +14710,7 @@
         <v>4</v>
       </c>
       <c r="H85" s="38" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="86" spans="2:8" ht="19" customHeight="1">
@@ -14721,10 +14718,10 @@
         <v>46311</v>
       </c>
       <c r="C86" s="34" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D86" s="34" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E86" s="25">
         <v>3</v>
@@ -14736,7 +14733,7 @@
         <v>3</v>
       </c>
       <c r="H86" s="40" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="87" spans="2:8" ht="19" customHeight="1">
@@ -14744,10 +14741,10 @@
         <v>46312</v>
       </c>
       <c r="C87" s="33" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D87" s="33" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E87" s="22">
         <v>20</v>
@@ -14759,7 +14756,7 @@
         <v>20</v>
       </c>
       <c r="H87" s="38" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="88" spans="2:8" ht="19" customHeight="1">
@@ -14767,10 +14764,10 @@
         <v>46314</v>
       </c>
       <c r="C88" s="34" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D88" s="34" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E88" s="25">
         <v>36</v>
@@ -14782,7 +14779,7 @@
         <v>9</v>
       </c>
       <c r="H88" s="40" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="89" spans="2:8" ht="19" customHeight="1">
@@ -14790,10 +14787,10 @@
         <v>46314</v>
       </c>
       <c r="C89" s="33" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D89" s="33" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E89" s="22">
         <v>36</v>
@@ -14805,7 +14802,7 @@
         <v>9</v>
       </c>
       <c r="H89" s="38" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="90" spans="2:8" ht="19" customHeight="1">
@@ -14828,7 +14825,7 @@
         <v>1000</v>
       </c>
       <c r="H90" s="40" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="91" spans="2:8" ht="19" customHeight="1">
@@ -14839,7 +14836,7 @@
         <v>31</v>
       </c>
       <c r="D91" s="33" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E91" s="22">
         <v>800</v>
@@ -14851,7 +14848,7 @@
         <v>800</v>
       </c>
       <c r="H91" s="38" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="92" spans="2:8" ht="19" customHeight="1">
@@ -14862,7 +14859,7 @@
         <v>31</v>
       </c>
       <c r="D92" s="34" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E92" s="25">
         <v>300</v>
@@ -14874,7 +14871,7 @@
         <v>300</v>
       </c>
       <c r="H92" s="40" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="93" spans="2:8" ht="19" customHeight="1">
@@ -14882,10 +14879,10 @@
         <v>46315</v>
       </c>
       <c r="C93" s="33" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D93" s="33" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E93" s="22">
         <v>216</v>
@@ -14897,7 +14894,7 @@
         <v>216</v>
       </c>
       <c r="H93" s="38" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="94" spans="2:8" ht="19" customHeight="1">
@@ -14905,10 +14902,10 @@
         <v>46316</v>
       </c>
       <c r="C94" s="34" t="s">
-        <v>263</v>
+        <v>203</v>
       </c>
       <c r="D94" s="34" t="s">
-        <v>264</v>
+        <v>204</v>
       </c>
       <c r="E94" s="25">
         <v>17</v>
@@ -14920,7 +14917,7 @@
         <v>17</v>
       </c>
       <c r="H94" s="40" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="95" spans="2:8" ht="19" customHeight="1">
@@ -14928,10 +14925,10 @@
         <v>46316</v>
       </c>
       <c r="C95" s="33" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D95" s="33" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E95" s="22">
         <v>5</v>
@@ -14943,7 +14940,7 @@
         <v>1</v>
       </c>
       <c r="H95" s="38" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="96" spans="2:8" ht="19" customHeight="1">
@@ -14951,10 +14948,10 @@
         <v>46316</v>
       </c>
       <c r="C96" s="34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D96" s="34" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E96" s="25">
         <v>3</v>
@@ -14966,7 +14963,7 @@
         <v>5</v>
       </c>
       <c r="H96" s="40" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="97" spans="2:8" ht="19" customHeight="1">
@@ -14974,10 +14971,10 @@
         <v>46317</v>
       </c>
       <c r="C97" s="33" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D97" s="33" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E97" s="22">
         <v>100</v>
@@ -14989,7 +14986,7 @@
         <v>98</v>
       </c>
       <c r="H97" s="38" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="98" spans="2:8" ht="19" customHeight="1">
@@ -14997,10 +14994,10 @@
         <v>46317</v>
       </c>
       <c r="C98" s="34" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D98" s="34" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E98" s="25">
         <v>11</v>
@@ -15012,7 +15009,7 @@
         <v>1</v>
       </c>
       <c r="H98" s="40" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="99" spans="2:8" ht="19" customHeight="1">
@@ -15035,7 +15032,7 @@
         <v>3</v>
       </c>
       <c r="H99" s="38" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="100" spans="2:8" ht="19" customHeight="1">
@@ -15046,7 +15043,7 @@
         <v>31</v>
       </c>
       <c r="D100" s="34" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E100" s="25">
         <v>250</v>
@@ -15058,7 +15055,7 @@
         <v>250</v>
       </c>
       <c r="H100" s="40" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="101" spans="2:8" ht="19" customHeight="1">
@@ -15066,10 +15063,10 @@
         <v>46319</v>
       </c>
       <c r="C101" s="33" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D101" s="33" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="E101" s="22">
         <v>150</v>
@@ -15081,7 +15078,7 @@
         <v>150</v>
       </c>
       <c r="H101" s="38" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="102" spans="2:8" ht="19" customHeight="1">
@@ -15089,10 +15086,10 @@
         <v>46319</v>
       </c>
       <c r="C102" s="34" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D102" s="34" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E102" s="25">
         <v>100</v>
@@ -15104,7 +15101,7 @@
         <v>35</v>
       </c>
       <c r="H102" s="40" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="103" spans="2:8" ht="19" customHeight="1">
@@ -15115,7 +15112,7 @@
         <v>31</v>
       </c>
       <c r="D103" s="33" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="E103" s="22">
         <v>100</v>
@@ -15127,7 +15124,7 @@
         <v>100</v>
       </c>
       <c r="H103" s="38" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="104" spans="2:8" ht="19" customHeight="1">
@@ -15135,10 +15132,10 @@
         <v>46319</v>
       </c>
       <c r="C104" s="34" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D104" s="34" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E104" s="25">
         <v>97</v>
@@ -15150,7 +15147,7 @@
         <v>30</v>
       </c>
       <c r="H104" s="40" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="105" spans="2:8" ht="19" customHeight="1">
@@ -15161,7 +15158,7 @@
         <v>30</v>
       </c>
       <c r="D105" s="33" t="s">
-        <v>209</v>
+        <v>231</v>
       </c>
       <c r="E105" s="22">
         <v>66</v>
@@ -15173,7 +15170,7 @@
         <v>66</v>
       </c>
       <c r="H105" s="38" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="106" spans="2:8" ht="19" customHeight="1">
@@ -15181,10 +15178,10 @@
         <v>46319</v>
       </c>
       <c r="C106" s="34" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="D106" s="34" t="s">
-        <v>271</v>
+        <v>215</v>
       </c>
       <c r="E106" s="25">
         <v>30</v>
@@ -15196,7 +15193,7 @@
         <v>20</v>
       </c>
       <c r="H106" s="40" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="107" spans="2:8" ht="19" customHeight="1">
@@ -15204,10 +15201,10 @@
         <v>46319</v>
       </c>
       <c r="C107" s="33" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="D107" s="33" t="s">
-        <v>271</v>
+        <v>215</v>
       </c>
       <c r="E107" s="22">
         <v>25</v>
@@ -15219,7 +15216,7 @@
         <v>20</v>
       </c>
       <c r="H107" s="38" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="108" spans="2:8" ht="19" customHeight="1">
@@ -15227,10 +15224,10 @@
         <v>46319</v>
       </c>
       <c r="C108" s="34" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D108" s="34" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="E108" s="25">
         <v>15</v>
@@ -15242,7 +15239,7 @@
         <v>15</v>
       </c>
       <c r="H108" s="40" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="109" spans="2:8" ht="19" customHeight="1">
@@ -15250,10 +15247,10 @@
         <v>46320</v>
       </c>
       <c r="C109" s="33" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D109" s="33" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E109" s="22">
         <v>15</v>
@@ -15265,7 +15262,7 @@
         <v>15</v>
       </c>
       <c r="H109" s="38" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="110" spans="2:8" ht="19" customHeight="1">
@@ -15273,10 +15270,10 @@
         <v>46320</v>
       </c>
       <c r="C110" s="34" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D110" s="34" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E110" s="25">
         <v>2</v>
@@ -15288,7 +15285,7 @@
         <v>1</v>
       </c>
       <c r="H110" s="40" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="111" spans="2:8" ht="19" customHeight="1">
@@ -15296,10 +15293,10 @@
         <v>46320</v>
       </c>
       <c r="C111" s="33" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D111" s="33" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E111" s="22">
         <v>1</v>
@@ -15311,7 +15308,7 @@
         <v>1</v>
       </c>
       <c r="H111" s="38" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="112" spans="2:8" ht="19" customHeight="1">
@@ -15319,10 +15316,10 @@
         <v>46320</v>
       </c>
       <c r="C112" s="34" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D112" s="34" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E112" s="25">
         <v>1</v>
@@ -15334,7 +15331,7 @@
         <v>1</v>
       </c>
       <c r="H112" s="40" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="113" spans="2:8" ht="19" customHeight="1">
@@ -15342,10 +15339,10 @@
         <v>46320</v>
       </c>
       <c r="C113" s="33" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D113" s="33" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E113" s="22">
         <v>1</v>
@@ -15357,7 +15354,7 @@
         <v>1</v>
       </c>
       <c r="H113" s="38" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="114" spans="2:8" ht="19" customHeight="1">
@@ -15365,10 +15362,10 @@
         <v>46320</v>
       </c>
       <c r="C114" s="34" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D114" s="34" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E114" s="25">
         <v>1</v>
@@ -15380,7 +15377,7 @@
         <v>1</v>
       </c>
       <c r="H114" s="40" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="115" spans="2:8" ht="19" customHeight="1">
@@ -15388,10 +15385,10 @@
         <v>46321</v>
       </c>
       <c r="C115" s="33" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D115" s="33" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E115" s="22">
         <v>225</v>
@@ -15403,7 +15400,7 @@
         <v>225</v>
       </c>
       <c r="H115" s="38" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="116" spans="2:8" ht="19" customHeight="1">
@@ -15411,10 +15408,10 @@
         <v>46321</v>
       </c>
       <c r="C116" s="34" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D116" s="34" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E116" s="25">
         <v>36</v>
@@ -15426,7 +15423,7 @@
         <v>9</v>
       </c>
       <c r="H116" s="40" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="117" spans="2:8" ht="19" customHeight="1">
@@ -15434,10 +15431,10 @@
         <v>46321</v>
       </c>
       <c r="C117" s="33" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="D117" s="33" t="s">
-        <v>271</v>
+        <v>215</v>
       </c>
       <c r="E117" s="22">
         <v>25</v>
@@ -15449,7 +15446,7 @@
         <v>13</v>
       </c>
       <c r="H117" s="38" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="118" spans="2:8" ht="19" customHeight="1">
@@ -15457,10 +15454,10 @@
         <v>46321</v>
       </c>
       <c r="C118" s="34" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="D118" s="34" t="s">
-        <v>271</v>
+        <v>215</v>
       </c>
       <c r="E118" s="25">
         <v>5</v>
@@ -15472,7 +15469,7 @@
         <v>2</v>
       </c>
       <c r="H118" s="40" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="119" spans="2:8" ht="19" customHeight="1">
@@ -15480,10 +15477,10 @@
         <v>46321</v>
       </c>
       <c r="C119" s="33" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="D119" s="33" t="s">
-        <v>271</v>
+        <v>215</v>
       </c>
       <c r="E119" s="22">
         <v>5</v>
@@ -15495,7 +15492,7 @@
         <v>2</v>
       </c>
       <c r="H119" s="38" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="120" spans="2:8" ht="19" customHeight="1">
@@ -15503,10 +15500,10 @@
         <v>46321</v>
       </c>
       <c r="C120" s="34" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D120" s="34" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="E120" s="25">
         <v>1</v>
@@ -15518,7 +15515,7 @@
         <v>1</v>
       </c>
       <c r="H120" s="40" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="121" spans="2:8" ht="19" customHeight="1">
@@ -15526,10 +15523,10 @@
         <v>46322</v>
       </c>
       <c r="C121" s="33" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D121" s="33" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E121" s="22">
         <v>200</v>
@@ -15541,7 +15538,7 @@
         <v>70</v>
       </c>
       <c r="H121" s="38" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="122" spans="2:8" ht="22" customHeight="1">
@@ -15605,7 +15602,7 @@
     <row r="2" spans="1:7" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -15646,13 +15643,13 @@
     </row>
     <row r="7" spans="1:7" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="F7" s="8" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="36" customHeight="1">
@@ -15660,21 +15657,21 @@
         <v>29</v>
       </c>
       <c r="C8" s="20" t="s">
+        <v>461</v>
+      </c>
+      <c r="D8" s="20" t="s">
         <v>462</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="E8" s="20" t="s">
         <v>463</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="F8" s="20" t="s">
         <v>464</v>
-      </c>
-      <c r="F8" s="20" t="s">
-        <v>465</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="19" customHeight="1">
       <c r="B9" s="21" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="C9" s="45">
         <v>0</v>
@@ -15725,7 +15722,7 @@
     </row>
     <row r="12" spans="1:7" ht="19" customHeight="1">
       <c r="B12" s="24" t="s">
-        <v>213</v>
+        <v>235</v>
       </c>
       <c r="C12" s="47">
         <v>0</v>
@@ -15742,7 +15739,7 @@
     </row>
     <row r="13" spans="1:7" ht="19" customHeight="1">
       <c r="B13" s="21" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="C13" s="45">
         <v>45</v>
@@ -15759,7 +15756,7 @@
     </row>
     <row r="14" spans="1:7" ht="19" customHeight="1">
       <c r="B14" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C14" s="47">
         <v>0</v>
@@ -15776,7 +15773,7 @@
     </row>
     <row r="15" spans="1:7" ht="19" customHeight="1">
       <c r="B15" s="21" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C15" s="45">
         <v>1</v>
@@ -15814,18 +15811,18 @@
     </row>
     <row r="33" spans="2:6" ht="27" customHeight="1">
       <c r="B33" s="6" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
       <c r="E33" s="7"/>
       <c r="F33" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="34" spans="2:6" ht="30" customHeight="1">
       <c r="B34" s="51" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C34" s="51"/>
       <c r="D34" s="52">
@@ -15836,7 +15833,7 @@
     </row>
     <row r="35" spans="2:6" ht="30" customHeight="1">
       <c r="B35" s="51" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C35" s="51"/>
       <c r="D35" s="52">
@@ -15847,7 +15844,7 @@
     </row>
     <row r="36" spans="2:6" ht="30" customHeight="1">
       <c r="B36" s="51" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C36" s="51"/>
       <c r="D36" s="54">
@@ -15908,7 +15905,7 @@
     <row r="2" spans="1:9" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -15957,7 +15954,7 @@
     </row>
     <row r="7" spans="1:9" ht="27" customHeight="1">
       <c r="B7" s="6" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -15965,7 +15962,7 @@
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="8" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="36" customHeight="1">
@@ -15973,30 +15970,30 @@
         <v>29</v>
       </c>
       <c r="C8" s="32" t="s">
+        <v>473</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>287</v>
+      </c>
+      <c r="E8" s="20" t="s">
         <v>474</v>
       </c>
-      <c r="D8" s="20" t="s">
-        <v>288</v>
-      </c>
-      <c r="E8" s="20" t="s">
-        <v>475</v>
-      </c>
       <c r="F8" s="20" t="s">
+        <v>463</v>
+      </c>
+      <c r="G8" s="20" t="s">
+        <v>462</v>
+      </c>
+      <c r="H8" s="20" t="s">
         <v>464</v>
-      </c>
-      <c r="G8" s="20" t="s">
-        <v>463</v>
-      </c>
-      <c r="H8" s="20" t="s">
-        <v>465</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="21" customHeight="1">
       <c r="B9" s="21" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D9" s="45">
         <v>757</v>
@@ -16016,10 +16013,10 @@
     </row>
     <row r="10" spans="1:9" ht="21" customHeight="1">
       <c r="B10" s="24" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D10" s="47">
         <v>141</v>
@@ -16039,10 +16036,10 @@
     </row>
     <row r="11" spans="1:9" ht="21" customHeight="1">
       <c r="B11" s="21" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="D11" s="45">
         <v>780</v>
@@ -16062,10 +16059,10 @@
     </row>
     <row r="12" spans="1:9" ht="21" customHeight="1">
       <c r="B12" s="24" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="D12" s="47">
         <v>1</v>
@@ -16085,10 +16082,10 @@
     </row>
     <row r="13" spans="1:9" ht="21" customHeight="1">
       <c r="B13" s="21" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D13" s="45">
         <v>7</v>
@@ -16108,10 +16105,10 @@
     </row>
     <row r="14" spans="1:9" ht="21" customHeight="1">
       <c r="B14" s="24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C14" s="34" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D14" s="47">
         <v>250</v>
@@ -16134,7 +16131,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="D15" s="45">
         <v>66</v>
@@ -16154,10 +16151,10 @@
     </row>
     <row r="16" spans="1:9" ht="35" customHeight="1">
       <c r="B16" s="24" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="C16" s="34" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="D16" s="47">
         <v>3820</v>
@@ -16180,7 +16177,7 @@
         <v>31</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="D17" s="45">
         <v>6850</v>
@@ -16200,10 +16197,10 @@
     </row>
     <row r="18" spans="2:8" ht="21" customHeight="1">
       <c r="B18" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C18" s="34" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D18" s="47">
         <v>498</v>
@@ -16223,10 +16220,10 @@
     </row>
     <row r="19" spans="2:8" ht="21" customHeight="1">
       <c r="B19" s="21" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="D19" s="45">
         <v>79</v>
@@ -16246,10 +16243,10 @@
     </row>
     <row r="20" spans="2:8" ht="21" customHeight="1">
       <c r="B20" s="24" t="s">
-        <v>213</v>
+        <v>235</v>
       </c>
       <c r="C20" s="34" t="s">
-        <v>214</v>
+        <v>236</v>
       </c>
       <c r="D20" s="47">
         <v>64</v>
@@ -16269,10 +16266,10 @@
     </row>
     <row r="21" spans="2:8" ht="35" customHeight="1">
       <c r="B21" s="21" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="D21" s="45">
         <v>110</v>
@@ -16292,10 +16289,10 @@
     </row>
     <row r="22" spans="2:8" ht="21" customHeight="1">
       <c r="B22" s="24" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C22" s="34" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="D22" s="47">
         <v>205</v>
@@ -16315,10 +16312,10 @@
     </row>
     <row r="23" spans="2:8" ht="21" customHeight="1">
       <c r="B23" s="21" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="D23" s="45">
         <v>180</v>
@@ -16338,10 +16335,10 @@
     </row>
     <row r="24" spans="2:8" ht="21" customHeight="1">
       <c r="B24" s="24" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C24" s="34" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="D24" s="47">
         <v>7</v>
@@ -16361,10 +16358,10 @@
     </row>
     <row r="25" spans="2:8" ht="35" customHeight="1">
       <c r="B25" s="21" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="D25" s="45">
         <v>64</v>
@@ -16387,7 +16384,7 @@
         <v>32</v>
       </c>
       <c r="C26" s="34" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="D26" s="47">
         <v>13</v>
@@ -16407,10 +16404,10 @@
     </row>
     <row r="27" spans="2:8" ht="21" customHeight="1">
       <c r="B27" s="21" t="s">
-        <v>263</v>
+        <v>203</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>264</v>
+        <v>204</v>
       </c>
       <c r="D27" s="45">
         <v>17</v>
@@ -16430,10 +16427,10 @@
     </row>
     <row r="28" spans="2:8" ht="21" customHeight="1">
       <c r="B28" s="24" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C28" s="34" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D28" s="47">
         <v>44</v>
@@ -16453,10 +16450,10 @@
     </row>
     <row r="29" spans="2:8" ht="21" customHeight="1">
       <c r="B29" s="21" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D29" s="45">
         <v>17</v>
@@ -16476,10 +16473,10 @@
     </row>
     <row r="30" spans="2:8" ht="21" customHeight="1">
       <c r="B30" s="24" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C30" s="34" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D30" s="47">
         <v>11</v>
@@ -16560,7 +16557,7 @@
     <row r="2" spans="1:4" ht="40" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -16589,7 +16586,7 @@
     </row>
     <row r="6" spans="1:4" ht="32" customHeight="1">
       <c r="B6" s="55" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C6" s="56" t="s">
         <v>4</v>
@@ -16597,31 +16594,31 @@
     </row>
     <row r="7" spans="1:4" ht="32" customHeight="1">
       <c r="B7" s="55" t="s">
+        <v>490</v>
+      </c>
+      <c r="C7" s="56" t="s">
         <v>491</v>
-      </c>
-      <c r="C7" s="56" t="s">
-        <v>492</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="32" customHeight="1">
       <c r="B8" s="55" t="s">
+        <v>492</v>
+      </c>
+      <c r="C8" s="56" t="s">
         <v>493</v>
-      </c>
-      <c r="C8" s="56" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="42" customHeight="1">
       <c r="B9" s="55" t="s">
+        <v>494</v>
+      </c>
+      <c r="C9" s="56" t="s">
         <v>495</v>
-      </c>
-      <c r="C9" s="56" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="32" customHeight="1">
       <c r="B10" s="55" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="C10" s="56" t="s">
         <v>37</v>
@@ -16629,50 +16626,50 @@
     </row>
     <row r="11" spans="1:4" ht="32" customHeight="1">
       <c r="B11" s="55" t="s">
+        <v>497</v>
+      </c>
+      <c r="C11" s="57" t="s">
         <v>498</v>
-      </c>
-      <c r="C11" s="57" t="s">
-        <v>499</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="42" customHeight="1">
       <c r="B12" s="55" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="C12" s="56" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="102" customHeight="1">
+    <row r="13" spans="1:4" ht="87" customHeight="1">
       <c r="B13" s="55" t="s">
+        <v>500</v>
+      </c>
+      <c r="C13" s="56" t="s">
         <v>501</v>
-      </c>
-      <c r="C13" s="56" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="72" customHeight="1">
       <c r="B14" s="55" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C14" s="56" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="72" customHeight="1">
       <c r="B15" s="55" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C15" s="56" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="57" customHeight="1">
       <c r="B16" s="55" t="s">
+        <v>503</v>
+      </c>
+      <c r="C16" s="56" t="s">
         <v>504</v>
-      </c>
-      <c r="C16" s="56" t="s">
-        <v>505</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Nombrar los servicios de continuidad sin siglas en Riesgos
- PAM, PCD, PE y AF se leen como Personas Adultas Mayores, Personas con Discapacidad, Protección
  Especial y Acompañamiento Familiar en el resumen, el tablero, la presentación y el libro; CNH y CDI
  conservan la forma del boletín aprobado.
- Resumen: leyenda de la banda en dos líneas y columna Servicio del detalle con espacio para el nombre.
- Tablero: la cifra de unidades suspendidas resume «67 CNH · 37 CDI · 39 en otros servicios» y el
  mosaico parte los nombres largos para conservar sus etiquetas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AUCWMWZ6GMzdHUXxvK5iGa
</commit_message>
<xml_diff>
--- a/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
+++ b/docs/reportes/Seguimiento_ENOS_2026-10-26.xlsx
@@ -75,7 +75,7 @@
     <t>Unidades cerradas / suspendidas</t>
   </si>
   <si>
-    <t>67 CNH · 37 CDI · 18 PAM · 12 PCD · 7 PE · 2 AF · corte El Oro 27/10; otros 26/10</t>
+    <t>67 CNH · 37 CDI · 39 en otros servicios · corte El Oro 27/10; otros 26/10</t>
   </si>
   <si>
     <t>Continuidad de los servicios</t>
@@ -102,16 +102,16 @@
     <t>CDI</t>
   </si>
   <si>
-    <t>PAM</t>
-  </si>
-  <si>
-    <t>PCD</t>
-  </si>
-  <si>
-    <t>PE</t>
-  </si>
-  <si>
-    <t>AF</t>
+    <t>Personas Adultas Mayores</t>
+  </si>
+  <si>
+    <t>Personas con Discapacidad</t>
+  </si>
+  <si>
+    <t>Protección Especial</t>
+  </si>
+  <si>
+    <t>Acompañamiento Familiar</t>
   </si>
   <si>
     <t>Total de la selección</t>
@@ -141,7 +141,7 @@
     <t>Aspectos destacados</t>
   </si>
   <si>
-    <t>143 unidades de atención con atención suspendida (67 CNH · 37 CDI · 18 PAM · 12 PCD · 7 PE · 2 AF); El Oro concentra 119 (83,2 %).</t>
+    <t>143 unidades de atención con atención suspendida (67 CNH · 37 CDI · 18 Personas Adultas Mayores · 12 Personas con Discapacidad · 7 Protección Especial · 2 Acompañamiento Familiar); El Oro concentra 119 (83,2 %).</t>
   </si>
   <si>
     <t>21 alertas reportadas: 10 con código UA y 11 reportes sectoriales.</t>
@@ -156,7 +156,7 @@
     <t>Unidades de atención suspendidas</t>
   </si>
   <si>
-    <t>143 unidades suspendidas · 67 CNH · 37 CDI · 18 PAM · 12 PCD · 7 PE · 2 AF</t>
+    <t>143 unidades suspendidas</t>
   </si>
   <si>
     <t>Fuente: unidades no operativas de El Oro al 27/10/2026; último reporte disponible de Guayas y Santa Elena al 26/10/2026.</t>
@@ -2352,16 +2352,16 @@
                   <c:v>CDI</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>PAM</c:v>
+                  <c:v>Personas Adultas Mayores</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>PCD</c:v>
+                  <c:v>Personas con Discapacidad</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>PE</c:v>
+                  <c:v>Protección Especial</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>AF</c:v>
+                  <c:v>Acompañamiento Familiar</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>

</xml_diff>